<commit_message>
Market data 14-Sep-2026 09:00 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X981"/>
+  <dimension ref="A1:X985"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -78422,6 +78422,326 @@
       <c r="W981" s="6" t="inlineStr"/>
       <c r="X981" s="6" t="inlineStr"/>
     </row>
+    <row r="982">
+      <c r="A982" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B982" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C982" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D982" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E982" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F982" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="G982" s="2" t="n">
+        <v>412.6</v>
+      </c>
+      <c r="H982" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="I982" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="J982" s="2" t="n">
+        <v>414.04</v>
+      </c>
+      <c r="K982" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="L982" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="M982" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="N982" s="4" t="n">
+        <v>420.05</v>
+      </c>
+      <c r="O982" s="5" t="n">
+        <v>414.57</v>
+      </c>
+      <c r="P982" s="3" t="n">
+        <v>425.43</v>
+      </c>
+      <c r="Q982" s="3" t="n">
+        <v>430.8</v>
+      </c>
+      <c r="R982" s="2" t="n">
+        <v>546</v>
+      </c>
+      <c r="S982" s="2" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T982" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U982" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V982" s="2" t="inlineStr"/>
+      <c r="W982" s="2" t="inlineStr"/>
+      <c r="X982" s="2" t="inlineStr"/>
+    </row>
+    <row r="983">
+      <c r="A983" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B983" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C983" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D983" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E983" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F983" s="2" t="n">
+        <v>1679.8</v>
+      </c>
+      <c r="G983" s="2" t="n">
+        <v>1666.7</v>
+      </c>
+      <c r="H983" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="I983" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="J983" s="2" t="n">
+        <v>1651.35</v>
+      </c>
+      <c r="K983" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="L983" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="M983" s="2" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N983" s="4" t="n">
+        <v>1681.45</v>
+      </c>
+      <c r="O983" s="5" t="n">
+        <v>1668.4</v>
+      </c>
+      <c r="P983" s="3" t="n">
+        <v>1694.4</v>
+      </c>
+      <c r="Q983" s="3" t="n">
+        <v>1707.35</v>
+      </c>
+      <c r="R983" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S983" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T983" s="2" t="n">
+        <v>2953</v>
+      </c>
+      <c r="U983" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V983" s="2" t="inlineStr"/>
+      <c r="W983" s="2" t="inlineStr"/>
+      <c r="X983" s="2" t="inlineStr"/>
+    </row>
+    <row r="984">
+      <c r="A984" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B984" s="6" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="C984" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D984" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E984" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F984" s="6" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="G984" s="6" t="n">
+        <v>990</v>
+      </c>
+      <c r="H984" s="6" t="n">
+        <v>992.8</v>
+      </c>
+      <c r="I984" s="6" t="n">
+        <v>973.1</v>
+      </c>
+      <c r="J984" s="6" t="n">
+        <v>1025.56</v>
+      </c>
+      <c r="K984" s="6" t="n">
+        <v>992.8</v>
+      </c>
+      <c r="L984" s="6" t="n">
+        <v>973.1</v>
+      </c>
+      <c r="M984" s="6" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="N984" s="8" t="n">
+        <v>973.05</v>
+      </c>
+      <c r="O984" s="7" t="n">
+        <v>983</v>
+      </c>
+      <c r="P984" s="9" t="n">
+        <v>963.2</v>
+      </c>
+      <c r="Q984" s="9" t="n">
+        <v>953.35</v>
+      </c>
+      <c r="R984" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="S984" s="6" t="n">
+        <v>2985</v>
+      </c>
+      <c r="T984" s="6" t="n">
+        <v>2955</v>
+      </c>
+      <c r="U984" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V984" s="6" t="inlineStr"/>
+      <c r="W984" s="6" t="inlineStr"/>
+      <c r="X984" s="6" t="inlineStr"/>
+    </row>
+    <row r="985">
+      <c r="A985" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B985" s="6" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+      <c r="C985" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D985" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E985" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F985" s="6" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="G985" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="H985" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="I985" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="J985" s="6" t="n">
+        <v>85.19</v>
+      </c>
+      <c r="K985" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="L985" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="M985" s="6" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="N985" s="8" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="O985" s="7" t="n">
+        <v>83.06999999999999</v>
+      </c>
+      <c r="P985" s="9" t="n">
+        <v>81.43000000000001</v>
+      </c>
+      <c r="Q985" s="9" t="n">
+        <v>80.66</v>
+      </c>
+      <c r="R985" s="6" t="n">
+        <v>3447</v>
+      </c>
+      <c r="S985" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T985" s="6" t="n">
+        <v>2654</v>
+      </c>
+      <c r="U985" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V985" s="6" t="inlineStr"/>
+      <c r="W985" s="6" t="inlineStr"/>
+      <c r="X985" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 14-Sep-2026 09:11 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X985"/>
+  <dimension ref="A1:X989"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -78742,6 +78742,326 @@
       <c r="W985" s="6" t="inlineStr"/>
       <c r="X985" s="6" t="inlineStr"/>
     </row>
+    <row r="986">
+      <c r="A986" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B986" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C986" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D986" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E986" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F986" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="G986" s="2" t="n">
+        <v>412.6</v>
+      </c>
+      <c r="H986" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="I986" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="J986" s="2" t="n">
+        <v>414.04</v>
+      </c>
+      <c r="K986" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="L986" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="M986" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="N986" s="4" t="n">
+        <v>420.05</v>
+      </c>
+      <c r="O986" s="5" t="n">
+        <v>414.57</v>
+      </c>
+      <c r="P986" s="3" t="n">
+        <v>425.43</v>
+      </c>
+      <c r="Q986" s="3" t="n">
+        <v>430.8</v>
+      </c>
+      <c r="R986" s="2" t="n">
+        <v>546</v>
+      </c>
+      <c r="S986" s="2" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T986" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U986" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V986" s="2" t="inlineStr"/>
+      <c r="W986" s="2" t="inlineStr"/>
+      <c r="X986" s="2" t="inlineStr"/>
+    </row>
+    <row r="987">
+      <c r="A987" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B987" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C987" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D987" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E987" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F987" s="2" t="n">
+        <v>1679.8</v>
+      </c>
+      <c r="G987" s="2" t="n">
+        <v>1666.7</v>
+      </c>
+      <c r="H987" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="I987" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="J987" s="2" t="n">
+        <v>1651.35</v>
+      </c>
+      <c r="K987" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="L987" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="M987" s="2" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N987" s="4" t="n">
+        <v>1681.45</v>
+      </c>
+      <c r="O987" s="5" t="n">
+        <v>1668.4</v>
+      </c>
+      <c r="P987" s="3" t="n">
+        <v>1694.4</v>
+      </c>
+      <c r="Q987" s="3" t="n">
+        <v>1707.35</v>
+      </c>
+      <c r="R987" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S987" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T987" s="2" t="n">
+        <v>2953</v>
+      </c>
+      <c r="U987" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V987" s="2" t="inlineStr"/>
+      <c r="W987" s="2" t="inlineStr"/>
+      <c r="X987" s="2" t="inlineStr"/>
+    </row>
+    <row r="988">
+      <c r="A988" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B988" s="6" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C988" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D988" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E988" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F988" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="G988" s="6" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="H988" s="6" t="n">
+        <v>243.16</v>
+      </c>
+      <c r="I988" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="J988" s="6" t="n">
+        <v>236.25</v>
+      </c>
+      <c r="K988" s="6" t="n">
+        <v>243.16</v>
+      </c>
+      <c r="L988" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="M988" s="6" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="N988" s="8" t="n">
+        <v>232.45</v>
+      </c>
+      <c r="O988" s="7" t="n">
+        <v>237.88</v>
+      </c>
+      <c r="P988" s="9" t="n">
+        <v>227.12</v>
+      </c>
+      <c r="Q988" s="9" t="n">
+        <v>221.79</v>
+      </c>
+      <c r="R988" s="6" t="n">
+        <v>552</v>
+      </c>
+      <c r="S988" s="6" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T988" s="6" t="n">
+        <v>2942</v>
+      </c>
+      <c r="U988" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V988" s="6" t="inlineStr"/>
+      <c r="W988" s="6" t="inlineStr"/>
+      <c r="X988" s="6" t="inlineStr"/>
+    </row>
+    <row r="989">
+      <c r="A989" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B989" s="6" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="C989" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D989" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E989" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F989" s="6" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="G989" s="6" t="n">
+        <v>990</v>
+      </c>
+      <c r="H989" s="6" t="n">
+        <v>992.8</v>
+      </c>
+      <c r="I989" s="6" t="n">
+        <v>973.1</v>
+      </c>
+      <c r="J989" s="6" t="n">
+        <v>1025.56</v>
+      </c>
+      <c r="K989" s="6" t="n">
+        <v>992.8</v>
+      </c>
+      <c r="L989" s="6" t="n">
+        <v>973.1</v>
+      </c>
+      <c r="M989" s="6" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="N989" s="8" t="n">
+        <v>973.05</v>
+      </c>
+      <c r="O989" s="7" t="n">
+        <v>983</v>
+      </c>
+      <c r="P989" s="9" t="n">
+        <v>963.2</v>
+      </c>
+      <c r="Q989" s="9" t="n">
+        <v>953.35</v>
+      </c>
+      <c r="R989" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="S989" s="6" t="n">
+        <v>2985</v>
+      </c>
+      <c r="T989" s="6" t="n">
+        <v>2955</v>
+      </c>
+      <c r="U989" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V989" s="6" t="inlineStr"/>
+      <c r="W989" s="6" t="inlineStr"/>
+      <c r="X989" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 14-Sep-2026 09:44 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X989"/>
+  <dimension ref="A1:X993"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -79062,6 +79062,326 @@
       <c r="W989" s="6" t="inlineStr"/>
       <c r="X989" s="6" t="inlineStr"/>
     </row>
+    <row r="990">
+      <c r="A990" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B990" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C990" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D990" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E990" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F990" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="G990" s="2" t="n">
+        <v>412.6</v>
+      </c>
+      <c r="H990" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="I990" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="J990" s="2" t="n">
+        <v>414.04</v>
+      </c>
+      <c r="K990" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="L990" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="M990" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="N990" s="4" t="n">
+        <v>420.05</v>
+      </c>
+      <c r="O990" s="5" t="n">
+        <v>414.57</v>
+      </c>
+      <c r="P990" s="3" t="n">
+        <v>425.43</v>
+      </c>
+      <c r="Q990" s="3" t="n">
+        <v>430.8</v>
+      </c>
+      <c r="R990" s="2" t="n">
+        <v>546</v>
+      </c>
+      <c r="S990" s="2" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T990" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U990" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V990" s="2" t="inlineStr"/>
+      <c r="W990" s="2" t="inlineStr"/>
+      <c r="X990" s="2" t="inlineStr"/>
+    </row>
+    <row r="991">
+      <c r="A991" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B991" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C991" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D991" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E991" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F991" s="2" t="n">
+        <v>1679.8</v>
+      </c>
+      <c r="G991" s="2" t="n">
+        <v>1666.7</v>
+      </c>
+      <c r="H991" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="I991" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="J991" s="2" t="n">
+        <v>1651.35</v>
+      </c>
+      <c r="K991" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="L991" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="M991" s="2" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N991" s="4" t="n">
+        <v>1681.45</v>
+      </c>
+      <c r="O991" s="5" t="n">
+        <v>1668.4</v>
+      </c>
+      <c r="P991" s="3" t="n">
+        <v>1694.4</v>
+      </c>
+      <c r="Q991" s="3" t="n">
+        <v>1707.35</v>
+      </c>
+      <c r="R991" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S991" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T991" s="2" t="n">
+        <v>2953</v>
+      </c>
+      <c r="U991" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V991" s="2" t="inlineStr"/>
+      <c r="W991" s="2" t="inlineStr"/>
+      <c r="X991" s="2" t="inlineStr"/>
+    </row>
+    <row r="992">
+      <c r="A992" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B992" s="6" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C992" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D992" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E992" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F992" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="G992" s="6" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="H992" s="6" t="n">
+        <v>243.16</v>
+      </c>
+      <c r="I992" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="J992" s="6" t="n">
+        <v>236.25</v>
+      </c>
+      <c r="K992" s="6" t="n">
+        <v>243.16</v>
+      </c>
+      <c r="L992" s="6" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="M992" s="6" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="N992" s="8" t="n">
+        <v>232.45</v>
+      </c>
+      <c r="O992" s="7" t="n">
+        <v>237.88</v>
+      </c>
+      <c r="P992" s="9" t="n">
+        <v>227.12</v>
+      </c>
+      <c r="Q992" s="9" t="n">
+        <v>221.79</v>
+      </c>
+      <c r="R992" s="6" t="n">
+        <v>552</v>
+      </c>
+      <c r="S992" s="6" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T992" s="6" t="n">
+        <v>2942</v>
+      </c>
+      <c r="U992" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V992" s="6" t="inlineStr"/>
+      <c r="W992" s="6" t="inlineStr"/>
+      <c r="X992" s="6" t="inlineStr"/>
+    </row>
+    <row r="993">
+      <c r="A993" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B993" s="6" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+      <c r="C993" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D993" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E993" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F993" s="6" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="G993" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="H993" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="I993" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="J993" s="6" t="n">
+        <v>85.19</v>
+      </c>
+      <c r="K993" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="L993" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="M993" s="6" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="N993" s="8" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="O993" s="7" t="n">
+        <v>83.06999999999999</v>
+      </c>
+      <c r="P993" s="9" t="n">
+        <v>81.43000000000001</v>
+      </c>
+      <c r="Q993" s="9" t="n">
+        <v>80.66</v>
+      </c>
+      <c r="R993" s="6" t="n">
+        <v>3447</v>
+      </c>
+      <c r="S993" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T993" s="6" t="n">
+        <v>2654</v>
+      </c>
+      <c r="U993" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V993" s="6" t="inlineStr"/>
+      <c r="W993" s="6" t="inlineStr"/>
+      <c r="X993" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 14-Sep-2026 09:52 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X993"/>
+  <dimension ref="A1:X997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -79382,6 +79382,326 @@
       <c r="W993" s="6" t="inlineStr"/>
       <c r="X993" s="6" t="inlineStr"/>
     </row>
+    <row r="994">
+      <c r="A994" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B994" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C994" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D994" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E994" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F994" s="2" t="n">
+        <v>419</v>
+      </c>
+      <c r="G994" s="2" t="n">
+        <v>412.6</v>
+      </c>
+      <c r="H994" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="I994" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="J994" s="2" t="n">
+        <v>414.04</v>
+      </c>
+      <c r="K994" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="L994" s="2" t="n">
+        <v>409.25</v>
+      </c>
+      <c r="M994" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="N994" s="4" t="n">
+        <v>420.05</v>
+      </c>
+      <c r="O994" s="5" t="n">
+        <v>414.57</v>
+      </c>
+      <c r="P994" s="3" t="n">
+        <v>425.43</v>
+      </c>
+      <c r="Q994" s="3" t="n">
+        <v>430.8</v>
+      </c>
+      <c r="R994" s="2" t="n">
+        <v>546</v>
+      </c>
+      <c r="S994" s="2" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T994" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U994" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V994" s="2" t="inlineStr"/>
+      <c r="W994" s="2" t="inlineStr"/>
+      <c r="X994" s="2" t="inlineStr"/>
+    </row>
+    <row r="995">
+      <c r="A995" s="2" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B995" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C995" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D995" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E995" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F995" s="2" t="n">
+        <v>1679.8</v>
+      </c>
+      <c r="G995" s="2" t="n">
+        <v>1666.7</v>
+      </c>
+      <c r="H995" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="I995" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="J995" s="2" t="n">
+        <v>1651.35</v>
+      </c>
+      <c r="K995" s="2" t="n">
+        <v>1681.4</v>
+      </c>
+      <c r="L995" s="2" t="n">
+        <v>1655.5</v>
+      </c>
+      <c r="M995" s="2" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="N995" s="4" t="n">
+        <v>1681.45</v>
+      </c>
+      <c r="O995" s="5" t="n">
+        <v>1668.4</v>
+      </c>
+      <c r="P995" s="3" t="n">
+        <v>1694.4</v>
+      </c>
+      <c r="Q995" s="3" t="n">
+        <v>1707.35</v>
+      </c>
+      <c r="R995" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S995" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T995" s="2" t="n">
+        <v>2953</v>
+      </c>
+      <c r="U995" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V995" s="2" t="inlineStr"/>
+      <c r="W995" s="2" t="inlineStr"/>
+      <c r="X995" s="2" t="inlineStr"/>
+    </row>
+    <row r="996">
+      <c r="A996" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B996" s="6" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+      <c r="C996" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D996" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E996" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F996" s="6" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="G996" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="H996" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="I996" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="J996" s="6" t="n">
+        <v>85.19</v>
+      </c>
+      <c r="K996" s="6" t="n">
+        <v>83.79000000000001</v>
+      </c>
+      <c r="L996" s="6" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="M996" s="6" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="N996" s="8" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="O996" s="7" t="n">
+        <v>83.06999999999999</v>
+      </c>
+      <c r="P996" s="9" t="n">
+        <v>81.43000000000001</v>
+      </c>
+      <c r="Q996" s="9" t="n">
+        <v>80.66</v>
+      </c>
+      <c r="R996" s="6" t="n">
+        <v>3447</v>
+      </c>
+      <c r="S996" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T996" s="6" t="n">
+        <v>2654</v>
+      </c>
+      <c r="U996" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V996" s="6" t="inlineStr"/>
+      <c r="W996" s="6" t="inlineStr"/>
+      <c r="X996" s="6" t="inlineStr"/>
+    </row>
+    <row r="997">
+      <c r="A997" s="6" t="inlineStr">
+        <is>
+          <t>14-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B997" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C997" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D997" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E997" s="6" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F997" s="6" t="n">
+        <v>1034.5</v>
+      </c>
+      <c r="G997" s="6" t="n">
+        <v>1031</v>
+      </c>
+      <c r="H997" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="I997" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="J997" s="6" t="n">
+        <v>1065.72</v>
+      </c>
+      <c r="K997" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="L997" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="M997" s="6" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="N997" s="8" t="n">
+        <v>1015.05</v>
+      </c>
+      <c r="O997" s="7" t="n">
+        <v>1025.1</v>
+      </c>
+      <c r="P997" s="9" t="n">
+        <v>1005.1</v>
+      </c>
+      <c r="Q997" s="9" t="n">
+        <v>995.15</v>
+      </c>
+      <c r="R997" s="6" t="n">
+        <v>297</v>
+      </c>
+      <c r="S997" s="6" t="n">
+        <v>2985</v>
+      </c>
+      <c r="T997" s="6" t="n">
+        <v>2955</v>
+      </c>
+      <c r="U997" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V997" s="6" t="inlineStr"/>
+      <c r="W997" s="6" t="inlineStr"/>
+      <c r="X997" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 15-Sep-2026 08:45 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X997"/>
+  <dimension ref="A1:X1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -79702,6 +79702,326 @@
       <c r="W997" s="6" t="inlineStr"/>
       <c r="X997" s="6" t="inlineStr"/>
     </row>
+    <row r="998">
+      <c r="A998" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B998" s="2" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C998" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D998" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E998" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F998" s="2" t="n">
+        <v>170.01</v>
+      </c>
+      <c r="G998" s="2" t="n">
+        <v>172.2</v>
+      </c>
+      <c r="H998" s="2" t="n">
+        <v>173.35</v>
+      </c>
+      <c r="I998" s="2" t="n">
+        <v>169.9</v>
+      </c>
+      <c r="J998" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K998" s="2" t="n">
+        <v>173.35</v>
+      </c>
+      <c r="L998" s="2" t="n">
+        <v>169.9</v>
+      </c>
+      <c r="M998" s="2" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="N998" s="4" t="n">
+        <v>173.4</v>
+      </c>
+      <c r="O998" s="5" t="n">
+        <v>171.57</v>
+      </c>
+      <c r="P998" s="3" t="n">
+        <v>175.12</v>
+      </c>
+      <c r="Q998" s="3" t="n">
+        <v>176.85</v>
+      </c>
+      <c r="R998" s="2" t="n">
+        <v>1638</v>
+      </c>
+      <c r="S998" s="2" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T998" s="2" t="n">
+        <v>2817</v>
+      </c>
+      <c r="U998" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V998" s="2" t="inlineStr"/>
+      <c r="W998" s="2" t="inlineStr"/>
+      <c r="X998" s="2" t="inlineStr"/>
+    </row>
+    <row r="999">
+      <c r="A999" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B999" s="2" t="inlineStr">
+        <is>
+          <t>COFORGE</t>
+        </is>
+      </c>
+      <c r="C999" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D999" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E999" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F999" s="2" t="n">
+        <v>1778.3</v>
+      </c>
+      <c r="G999" s="2" t="n">
+        <v>1887.3</v>
+      </c>
+      <c r="H999" s="2" t="n">
+        <v>1893.6</v>
+      </c>
+      <c r="I999" s="2" t="n">
+        <v>1775.4</v>
+      </c>
+      <c r="J999" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K999" s="2" t="n">
+        <v>1893.6</v>
+      </c>
+      <c r="L999" s="2" t="n">
+        <v>1775.4</v>
+      </c>
+      <c r="M999" s="2" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="N999" s="4" t="n">
+        <v>1893.65</v>
+      </c>
+      <c r="O999" s="5" t="n">
+        <v>1834.45</v>
+      </c>
+      <c r="P999" s="3" t="n">
+        <v>1952.75</v>
+      </c>
+      <c r="Q999" s="3" t="n">
+        <v>2011.85</v>
+      </c>
+      <c r="R999" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="S999" s="2" t="n">
+        <v>2842</v>
+      </c>
+      <c r="T999" s="2" t="n">
+        <v>2837</v>
+      </c>
+      <c r="U999" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V999" s="2" t="inlineStr"/>
+      <c r="W999" s="2" t="inlineStr"/>
+      <c r="X999" s="2" t="inlineStr"/>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1000" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1000" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1000" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1000" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1000" s="6" t="n">
+        <v>1010.1</v>
+      </c>
+      <c r="G1000" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="H1000" s="6" t="n">
+        <v>1038.6</v>
+      </c>
+      <c r="I1000" s="6" t="n">
+        <v>1008.4</v>
+      </c>
+      <c r="J1000" s="6" t="n">
+        <v>1063.43</v>
+      </c>
+      <c r="K1000" s="6" t="n">
+        <v>1038.6</v>
+      </c>
+      <c r="L1000" s="6" t="n">
+        <v>1008.4</v>
+      </c>
+      <c r="M1000" s="6" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="N1000" s="8" t="n">
+        <v>1008.35</v>
+      </c>
+      <c r="O1000" s="7" t="n">
+        <v>1023.55</v>
+      </c>
+      <c r="P1000" s="9" t="n">
+        <v>993.25</v>
+      </c>
+      <c r="Q1000" s="9" t="n">
+        <v>978.15</v>
+      </c>
+      <c r="R1000" s="6" t="n">
+        <v>195</v>
+      </c>
+      <c r="S1000" s="6" t="n">
+        <v>2964</v>
+      </c>
+      <c r="T1000" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="U1000" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1000" s="6" t="inlineStr"/>
+      <c r="W1000" s="6" t="inlineStr"/>
+      <c r="X1000" s="6" t="inlineStr"/>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1001" s="6" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1001" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1001" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1001" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1001" s="6" t="n">
+        <v>523.6</v>
+      </c>
+      <c r="G1001" s="6" t="n">
+        <v>530</v>
+      </c>
+      <c r="H1001" s="6" t="n">
+        <v>530.65</v>
+      </c>
+      <c r="I1001" s="6" t="n">
+        <v>520.65</v>
+      </c>
+      <c r="J1001" s="6" t="n">
+        <v>536.88</v>
+      </c>
+      <c r="K1001" s="6" t="n">
+        <v>530.65</v>
+      </c>
+      <c r="L1001" s="6" t="n">
+        <v>520.65</v>
+      </c>
+      <c r="M1001" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N1001" s="8" t="n">
+        <v>520.6</v>
+      </c>
+      <c r="O1001" s="7" t="n">
+        <v>525.7</v>
+      </c>
+      <c r="P1001" s="9" t="n">
+        <v>515.6</v>
+      </c>
+      <c r="Q1001" s="9" t="n">
+        <v>510.6</v>
+      </c>
+      <c r="R1001" s="6" t="n">
+        <v>588</v>
+      </c>
+      <c r="S1001" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1001" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1001" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1001" s="6" t="inlineStr"/>
+      <c r="W1001" s="6" t="inlineStr"/>
+      <c r="X1001" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 15-Sep-2026 08:53 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1001"/>
+  <dimension ref="A1:X1005"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80022,6 +80022,326 @@
       <c r="W1001" s="6" t="inlineStr"/>
       <c r="X1001" s="6" t="inlineStr"/>
     </row>
+    <row r="1002">
+      <c r="A1002" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1002" s="2" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1002" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1002" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1002" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1002" s="2" t="n">
+        <v>1074.9</v>
+      </c>
+      <c r="G1002" s="2" t="n">
+        <v>1085</v>
+      </c>
+      <c r="H1002" s="2" t="n">
+        <v>1097.7</v>
+      </c>
+      <c r="I1002" s="2" t="n">
+        <v>1071.7</v>
+      </c>
+      <c r="J1002" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1002" s="2" t="n">
+        <v>1097.7</v>
+      </c>
+      <c r="L1002" s="2" t="n">
+        <v>1071.7</v>
+      </c>
+      <c r="M1002" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="N1002" s="4" t="n">
+        <v>1097.75</v>
+      </c>
+      <c r="O1002" s="5" t="n">
+        <v>1084.65</v>
+      </c>
+      <c r="P1002" s="3" t="n">
+        <v>1110.75</v>
+      </c>
+      <c r="Q1002" s="3" t="n">
+        <v>1123.75</v>
+      </c>
+      <c r="R1002" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S1002" s="2" t="n">
+        <v>2987</v>
+      </c>
+      <c r="T1002" s="2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="U1002" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1002" s="2" t="inlineStr"/>
+      <c r="W1002" s="2" t="inlineStr"/>
+      <c r="X1002" s="2" t="inlineStr"/>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1003" s="2" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="C1003" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1003" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1003" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1003" s="2" t="n">
+        <v>11764</v>
+      </c>
+      <c r="G1003" s="2" t="n">
+        <v>11910</v>
+      </c>
+      <c r="H1003" s="2" t="n">
+        <v>12099</v>
+      </c>
+      <c r="I1003" s="2" t="n">
+        <v>11716</v>
+      </c>
+      <c r="J1003" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1003" s="2" t="n">
+        <v>12099</v>
+      </c>
+      <c r="L1003" s="2" t="n">
+        <v>11716</v>
+      </c>
+      <c r="M1003" s="2" t="n">
+        <v>383</v>
+      </c>
+      <c r="N1003" s="4" t="n">
+        <v>12099.05</v>
+      </c>
+      <c r="O1003" s="5" t="n">
+        <v>11907.45</v>
+      </c>
+      <c r="P1003" s="3" t="n">
+        <v>12290.55</v>
+      </c>
+      <c r="Q1003" s="3" t="n">
+        <v>12482.05</v>
+      </c>
+      <c r="R1003" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="S1003" s="2" t="n">
+        <v>2874</v>
+      </c>
+      <c r="T1003" s="2" t="n">
+        <v>2872</v>
+      </c>
+      <c r="U1003" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1003" s="2" t="inlineStr"/>
+      <c r="W1003" s="2" t="inlineStr"/>
+      <c r="X1003" s="2" t="inlineStr"/>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1004" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1004" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1004" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1004" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1004" s="6" t="n">
+        <v>1864.7</v>
+      </c>
+      <c r="G1004" s="6" t="n">
+        <v>1921.4</v>
+      </c>
+      <c r="H1004" s="6" t="n">
+        <v>1930.6</v>
+      </c>
+      <c r="I1004" s="6" t="n">
+        <v>1863.8</v>
+      </c>
+      <c r="J1004" s="6" t="n">
+        <v>1978.22</v>
+      </c>
+      <c r="K1004" s="6" t="n">
+        <v>1930.6</v>
+      </c>
+      <c r="L1004" s="6" t="n">
+        <v>1863.8</v>
+      </c>
+      <c r="M1004" s="6" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="N1004" s="8" t="n">
+        <v>1863.75</v>
+      </c>
+      <c r="O1004" s="7" t="n">
+        <v>1897.25</v>
+      </c>
+      <c r="P1004" s="9" t="n">
+        <v>1830.35</v>
+      </c>
+      <c r="Q1004" s="9" t="n">
+        <v>1796.95</v>
+      </c>
+      <c r="R1004" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="S1004" s="6" t="n">
+        <v>2914</v>
+      </c>
+      <c r="T1004" s="6" t="n">
+        <v>2906</v>
+      </c>
+      <c r="U1004" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1004" s="6" t="inlineStr"/>
+      <c r="W1004" s="6" t="inlineStr"/>
+      <c r="X1004" s="6" t="inlineStr"/>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1005" s="6" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1005" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1005" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1005" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1005" s="6" t="n">
+        <v>1658.8</v>
+      </c>
+      <c r="G1005" s="6" t="n">
+        <v>1672.1</v>
+      </c>
+      <c r="H1005" s="6" t="n">
+        <v>1683.1</v>
+      </c>
+      <c r="I1005" s="6" t="n">
+        <v>1656.7</v>
+      </c>
+      <c r="J1005" s="6" t="n">
+        <v>1745.87</v>
+      </c>
+      <c r="K1005" s="6" t="n">
+        <v>1683.1</v>
+      </c>
+      <c r="L1005" s="6" t="n">
+        <v>1656.7</v>
+      </c>
+      <c r="M1005" s="6" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="N1005" s="8" t="n">
+        <v>1656.65</v>
+      </c>
+      <c r="O1005" s="7" t="n">
+        <v>1669.95</v>
+      </c>
+      <c r="P1005" s="9" t="n">
+        <v>1643.45</v>
+      </c>
+      <c r="Q1005" s="9" t="n">
+        <v>1630.25</v>
+      </c>
+      <c r="R1005" s="6" t="n">
+        <v>225</v>
+      </c>
+      <c r="S1005" s="6" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T1005" s="6" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1005" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1005" s="6" t="inlineStr"/>
+      <c r="W1005" s="6" t="inlineStr"/>
+      <c r="X1005" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 15-Sep-2026 09:21 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1005"/>
+  <dimension ref="A1:X1009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80342,6 +80342,326 @@
       <c r="W1005" s="6" t="inlineStr"/>
       <c r="X1005" s="6" t="inlineStr"/>
     </row>
+    <row r="1006">
+      <c r="A1006" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1006" s="2" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1006" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1006" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1006" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1006" s="2" t="n">
+        <v>1075.9</v>
+      </c>
+      <c r="G1006" s="2" t="n">
+        <v>1085</v>
+      </c>
+      <c r="H1006" s="2" t="n">
+        <v>1097.7</v>
+      </c>
+      <c r="I1006" s="2" t="n">
+        <v>1071.7</v>
+      </c>
+      <c r="J1006" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1006" s="2" t="n">
+        <v>1097.7</v>
+      </c>
+      <c r="L1006" s="2" t="n">
+        <v>1071.7</v>
+      </c>
+      <c r="M1006" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="N1006" s="4" t="n">
+        <v>1097.75</v>
+      </c>
+      <c r="O1006" s="5" t="n">
+        <v>1084.65</v>
+      </c>
+      <c r="P1006" s="3" t="n">
+        <v>1110.75</v>
+      </c>
+      <c r="Q1006" s="3" t="n">
+        <v>1123.75</v>
+      </c>
+      <c r="R1006" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S1006" s="2" t="n">
+        <v>2987</v>
+      </c>
+      <c r="T1006" s="2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="U1006" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1006" s="2" t="inlineStr"/>
+      <c r="W1006" s="2" t="inlineStr"/>
+      <c r="X1006" s="2" t="inlineStr"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1007" s="2" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="C1007" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1007" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1007" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1007" s="2" t="n">
+        <v>11753</v>
+      </c>
+      <c r="G1007" s="2" t="n">
+        <v>11910</v>
+      </c>
+      <c r="H1007" s="2" t="n">
+        <v>12099</v>
+      </c>
+      <c r="I1007" s="2" t="n">
+        <v>11716</v>
+      </c>
+      <c r="J1007" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1007" s="2" t="n">
+        <v>12099</v>
+      </c>
+      <c r="L1007" s="2" t="n">
+        <v>11716</v>
+      </c>
+      <c r="M1007" s="2" t="n">
+        <v>383</v>
+      </c>
+      <c r="N1007" s="4" t="n">
+        <v>12099.05</v>
+      </c>
+      <c r="O1007" s="5" t="n">
+        <v>11907.45</v>
+      </c>
+      <c r="P1007" s="3" t="n">
+        <v>12290.55</v>
+      </c>
+      <c r="Q1007" s="3" t="n">
+        <v>12482.05</v>
+      </c>
+      <c r="R1007" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="S1007" s="2" t="n">
+        <v>2874</v>
+      </c>
+      <c r="T1007" s="2" t="n">
+        <v>2872</v>
+      </c>
+      <c r="U1007" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1007" s="2" t="inlineStr"/>
+      <c r="W1007" s="2" t="inlineStr"/>
+      <c r="X1007" s="2" t="inlineStr"/>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1008" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1008" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1008" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1008" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1008" s="6" t="n">
+        <v>1007.5</v>
+      </c>
+      <c r="G1008" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="H1008" s="6" t="n">
+        <v>1038.6</v>
+      </c>
+      <c r="I1008" s="6" t="n">
+        <v>1007.3</v>
+      </c>
+      <c r="J1008" s="6" t="n">
+        <v>1062.92</v>
+      </c>
+      <c r="K1008" s="6" t="n">
+        <v>1038.6</v>
+      </c>
+      <c r="L1008" s="6" t="n">
+        <v>1007.3</v>
+      </c>
+      <c r="M1008" s="6" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="N1008" s="8" t="n">
+        <v>1007.25</v>
+      </c>
+      <c r="O1008" s="7" t="n">
+        <v>1023</v>
+      </c>
+      <c r="P1008" s="9" t="n">
+        <v>991.6</v>
+      </c>
+      <c r="Q1008" s="9" t="n">
+        <v>975.95</v>
+      </c>
+      <c r="R1008" s="6" t="n">
+        <v>189</v>
+      </c>
+      <c r="S1008" s="6" t="n">
+        <v>2977</v>
+      </c>
+      <c r="T1008" s="6" t="n">
+        <v>2958</v>
+      </c>
+      <c r="U1008" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1008" s="6" t="inlineStr"/>
+      <c r="W1008" s="6" t="inlineStr"/>
+      <c r="X1008" s="6" t="inlineStr"/>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="6" t="inlineStr">
+        <is>
+          <t>15-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1009" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1009" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1009" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1009" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1009" s="6" t="n">
+        <v>1861.7</v>
+      </c>
+      <c r="G1009" s="6" t="n">
+        <v>1921.4</v>
+      </c>
+      <c r="H1009" s="6" t="n">
+        <v>1930.6</v>
+      </c>
+      <c r="I1009" s="6" t="n">
+        <v>1861.1</v>
+      </c>
+      <c r="J1009" s="6" t="n">
+        <v>1977.96</v>
+      </c>
+      <c r="K1009" s="6" t="n">
+        <v>1930.6</v>
+      </c>
+      <c r="L1009" s="6" t="n">
+        <v>1861.1</v>
+      </c>
+      <c r="M1009" s="6" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="N1009" s="8" t="n">
+        <v>1861.05</v>
+      </c>
+      <c r="O1009" s="7" t="n">
+        <v>1895.9</v>
+      </c>
+      <c r="P1009" s="9" t="n">
+        <v>1826.3</v>
+      </c>
+      <c r="Q1009" s="9" t="n">
+        <v>1791.55</v>
+      </c>
+      <c r="R1009" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="S1009" s="6" t="n">
+        <v>2927</v>
+      </c>
+      <c r="T1009" s="6" t="n">
+        <v>2919</v>
+      </c>
+      <c r="U1009" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1009" s="6" t="inlineStr"/>
+      <c r="W1009" s="6" t="inlineStr"/>
+      <c r="X1009" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 16-Sep-2026 08:39 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1009"/>
+  <dimension ref="A1:X1013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80662,6 +80662,326 @@
       <c r="W1009" s="6" t="inlineStr"/>
       <c r="X1009" s="6" t="inlineStr"/>
     </row>
+    <row r="1010">
+      <c r="A1010" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1010" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C1010" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1010" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1010" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1010" s="2" t="n">
+        <v>415.4</v>
+      </c>
+      <c r="G1010" s="2" t="n">
+        <v>413.6</v>
+      </c>
+      <c r="H1010" s="2" t="n">
+        <v>416.7</v>
+      </c>
+      <c r="I1010" s="2" t="n">
+        <v>409.35</v>
+      </c>
+      <c r="J1010" s="2" t="n">
+        <v>414.97</v>
+      </c>
+      <c r="K1010" s="2" t="n">
+        <v>416.7</v>
+      </c>
+      <c r="L1010" s="2" t="n">
+        <v>409.35</v>
+      </c>
+      <c r="M1010" s="2" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="N1010" s="4" t="n">
+        <v>416.75</v>
+      </c>
+      <c r="O1010" s="5" t="n">
+        <v>412.97</v>
+      </c>
+      <c r="P1010" s="3" t="n">
+        <v>420.43</v>
+      </c>
+      <c r="Q1010" s="3" t="n">
+        <v>424.1</v>
+      </c>
+      <c r="R1010" s="2" t="n">
+        <v>792</v>
+      </c>
+      <c r="S1010" s="2" t="n">
+        <v>2994</v>
+      </c>
+      <c r="T1010" s="2" t="n">
+        <v>2915</v>
+      </c>
+      <c r="U1010" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1010" s="2" t="inlineStr"/>
+      <c r="W1010" s="2" t="inlineStr"/>
+      <c r="X1010" s="2" t="inlineStr"/>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1011" s="2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C1011" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1011" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1011" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1011" s="2" t="n">
+        <v>718.3</v>
+      </c>
+      <c r="G1011" s="2" t="n">
+        <v>714.9</v>
+      </c>
+      <c r="H1011" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="I1011" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="J1011" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1011" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="L1011" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="M1011" s="2" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="N1011" s="4" t="n">
+        <v>720.35</v>
+      </c>
+      <c r="O1011" s="5" t="n">
+        <v>715.53</v>
+      </c>
+      <c r="P1011" s="3" t="n">
+        <v>725.08</v>
+      </c>
+      <c r="Q1011" s="3" t="n">
+        <v>729.8</v>
+      </c>
+      <c r="R1011" s="2" t="n">
+        <v>621</v>
+      </c>
+      <c r="S1011" s="2" t="n">
+        <v>2993</v>
+      </c>
+      <c r="T1011" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U1011" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1011" s="2" t="inlineStr"/>
+      <c r="W1011" s="2" t="inlineStr"/>
+      <c r="X1011" s="2" t="inlineStr"/>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1012" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1012" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1012" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1012" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1012" s="6" t="n">
+        <v>1010.7</v>
+      </c>
+      <c r="G1012" s="6" t="n">
+        <v>1010.5</v>
+      </c>
+      <c r="H1012" s="6" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="I1012" s="6" t="n">
+        <v>1007.4</v>
+      </c>
+      <c r="J1012" s="6" t="n">
+        <v>1059.81</v>
+      </c>
+      <c r="K1012" s="6" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="L1012" s="6" t="n">
+        <v>1007.4</v>
+      </c>
+      <c r="M1012" s="6" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="N1012" s="8" t="n">
+        <v>1007.35</v>
+      </c>
+      <c r="O1012" s="7" t="n">
+        <v>1013.4</v>
+      </c>
+      <c r="P1012" s="9" t="n">
+        <v>1001.4</v>
+      </c>
+      <c r="Q1012" s="9" t="n">
+        <v>995.45</v>
+      </c>
+      <c r="R1012" s="6" t="n">
+        <v>495</v>
+      </c>
+      <c r="S1012" s="6" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1012" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="U1012" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1012" s="6" t="inlineStr"/>
+      <c r="W1012" s="6" t="inlineStr"/>
+      <c r="X1012" s="6" t="inlineStr"/>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1013" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1013" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1013" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1013" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1013" s="6" t="n">
+        <v>1842.2</v>
+      </c>
+      <c r="G1013" s="6" t="n">
+        <v>1864</v>
+      </c>
+      <c r="H1013" s="6" t="n">
+        <v>1874.8</v>
+      </c>
+      <c r="I1013" s="6" t="n">
+        <v>1836.5</v>
+      </c>
+      <c r="J1013" s="6" t="n">
+        <v>1971.37</v>
+      </c>
+      <c r="K1013" s="6" t="n">
+        <v>1874.8</v>
+      </c>
+      <c r="L1013" s="6" t="n">
+        <v>1836.5</v>
+      </c>
+      <c r="M1013" s="6" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="N1013" s="8" t="n">
+        <v>1836.45</v>
+      </c>
+      <c r="O1013" s="7" t="n">
+        <v>1855.7</v>
+      </c>
+      <c r="P1013" s="9" t="n">
+        <v>1817.3</v>
+      </c>
+      <c r="Q1013" s="9" t="n">
+        <v>1798.15</v>
+      </c>
+      <c r="R1013" s="6" t="n">
+        <v>153</v>
+      </c>
+      <c r="S1013" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="T1013" s="6" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1013" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1013" s="6" t="inlineStr"/>
+      <c r="W1013" s="6" t="inlineStr"/>
+      <c r="X1013" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 16-Sep-2026 08:47 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1013"/>
+  <dimension ref="A1:X1017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80982,6 +80982,326 @@
       <c r="W1013" s="6" t="inlineStr"/>
       <c r="X1013" s="6" t="inlineStr"/>
     </row>
+    <row r="1014">
+      <c r="A1014" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1014" s="2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C1014" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1014" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1014" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1014" s="2" t="n">
+        <v>718.25</v>
+      </c>
+      <c r="G1014" s="2" t="n">
+        <v>714.9</v>
+      </c>
+      <c r="H1014" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="I1014" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="J1014" s="2" t="n">
+        <v>712.5700000000001</v>
+      </c>
+      <c r="K1014" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="L1014" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="M1014" s="2" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="N1014" s="4" t="n">
+        <v>720.35</v>
+      </c>
+      <c r="O1014" s="5" t="n">
+        <v>715.53</v>
+      </c>
+      <c r="P1014" s="3" t="n">
+        <v>725.08</v>
+      </c>
+      <c r="Q1014" s="3" t="n">
+        <v>729.8</v>
+      </c>
+      <c r="R1014" s="2" t="n">
+        <v>621</v>
+      </c>
+      <c r="S1014" s="2" t="n">
+        <v>2993</v>
+      </c>
+      <c r="T1014" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U1014" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1014" s="2" t="inlineStr"/>
+      <c r="W1014" s="2" t="inlineStr"/>
+      <c r="X1014" s="2" t="inlineStr"/>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1015" s="2" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C1015" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1015" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1015" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1015" s="2" t="n">
+        <v>988.5</v>
+      </c>
+      <c r="G1015" s="2" t="n">
+        <v>976</v>
+      </c>
+      <c r="H1015" s="2" t="n">
+        <v>989.2</v>
+      </c>
+      <c r="I1015" s="2" t="n">
+        <v>973.2</v>
+      </c>
+      <c r="J1015" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1015" s="2" t="n">
+        <v>989.2</v>
+      </c>
+      <c r="L1015" s="2" t="n">
+        <v>973.2</v>
+      </c>
+      <c r="M1015" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="N1015" s="4" t="n">
+        <v>989.25</v>
+      </c>
+      <c r="O1015" s="5" t="n">
+        <v>981.15</v>
+      </c>
+      <c r="P1015" s="3" t="n">
+        <v>997.25</v>
+      </c>
+      <c r="Q1015" s="3" t="n">
+        <v>1005.25</v>
+      </c>
+      <c r="R1015" s="2" t="n">
+        <v>369</v>
+      </c>
+      <c r="S1015" s="2" t="n">
+        <v>2989</v>
+      </c>
+      <c r="T1015" s="2" t="n">
+        <v>2952</v>
+      </c>
+      <c r="U1015" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1015" s="2" t="inlineStr"/>
+      <c r="W1015" s="2" t="inlineStr"/>
+      <c r="X1015" s="2" t="inlineStr"/>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1016" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1016" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1016" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1016" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1016" s="6" t="n">
+        <v>1012.1</v>
+      </c>
+      <c r="G1016" s="6" t="n">
+        <v>1010.5</v>
+      </c>
+      <c r="H1016" s="6" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="I1016" s="6" t="n">
+        <v>1007.4</v>
+      </c>
+      <c r="J1016" s="6" t="n">
+        <v>1059.78</v>
+      </c>
+      <c r="K1016" s="6" t="n">
+        <v>1019.3</v>
+      </c>
+      <c r="L1016" s="6" t="n">
+        <v>1007.4</v>
+      </c>
+      <c r="M1016" s="6" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="N1016" s="8" t="n">
+        <v>1007.35</v>
+      </c>
+      <c r="O1016" s="7" t="n">
+        <v>1013.4</v>
+      </c>
+      <c r="P1016" s="9" t="n">
+        <v>1001.4</v>
+      </c>
+      <c r="Q1016" s="9" t="n">
+        <v>995.45</v>
+      </c>
+      <c r="R1016" s="6" t="n">
+        <v>495</v>
+      </c>
+      <c r="S1016" s="6" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1016" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="U1016" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1016" s="6" t="inlineStr"/>
+      <c r="W1016" s="6" t="inlineStr"/>
+      <c r="X1016" s="6" t="inlineStr"/>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1017" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1017" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1017" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1017" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1017" s="6" t="n">
+        <v>1768.5</v>
+      </c>
+      <c r="G1017" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="H1017" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="I1017" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="J1017" s="6" t="n">
+        <v>1839.21</v>
+      </c>
+      <c r="K1017" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="L1017" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="M1017" s="6" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="N1017" s="8" t="n">
+        <v>1756.25</v>
+      </c>
+      <c r="O1017" s="7" t="n">
+        <v>1778.55</v>
+      </c>
+      <c r="P1017" s="9" t="n">
+        <v>1734.05</v>
+      </c>
+      <c r="Q1017" s="9" t="n">
+        <v>1711.85</v>
+      </c>
+      <c r="R1017" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1017" s="6" t="n">
+        <v>2944</v>
+      </c>
+      <c r="T1017" s="6" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1017" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1017" s="6" t="inlineStr"/>
+      <c r="W1017" s="6" t="inlineStr"/>
+      <c r="X1017" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 16-Sep-2026 09:12 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1017"/>
+  <dimension ref="A1:X1021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81302,6 +81302,326 @@
       <c r="W1017" s="6" t="inlineStr"/>
       <c r="X1017" s="6" t="inlineStr"/>
     </row>
+    <row r="1018">
+      <c r="A1018" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1018" s="2" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="C1018" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1018" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1018" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1018" s="2" t="n">
+        <v>1774.2</v>
+      </c>
+      <c r="G1018" s="2" t="n">
+        <v>1754.9</v>
+      </c>
+      <c r="H1018" s="2" t="n">
+        <v>1781.3</v>
+      </c>
+      <c r="I1018" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="J1018" s="2" t="n">
+        <v>1714.1</v>
+      </c>
+      <c r="K1018" s="2" t="n">
+        <v>1781.3</v>
+      </c>
+      <c r="L1018" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="M1018" s="2" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N1018" s="4" t="n">
+        <v>1781.35</v>
+      </c>
+      <c r="O1018" s="5" t="n">
+        <v>1760.6</v>
+      </c>
+      <c r="P1018" s="3" t="n">
+        <v>1802</v>
+      </c>
+      <c r="Q1018" s="3" t="n">
+        <v>1822.65</v>
+      </c>
+      <c r="R1018" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="S1018" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1018" s="2" t="n">
+        <v>2974</v>
+      </c>
+      <c r="U1018" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1018" s="2" t="inlineStr"/>
+      <c r="W1018" s="2" t="inlineStr"/>
+      <c r="X1018" s="2" t="inlineStr"/>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1019" s="2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C1019" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1019" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1019" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1019" s="2" t="n">
+        <v>720.05</v>
+      </c>
+      <c r="G1019" s="2" t="n">
+        <v>714.9</v>
+      </c>
+      <c r="H1019" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="I1019" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="J1019" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1019" s="2" t="n">
+        <v>720.3</v>
+      </c>
+      <c r="L1019" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="M1019" s="2" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="N1019" s="4" t="n">
+        <v>720.35</v>
+      </c>
+      <c r="O1019" s="5" t="n">
+        <v>715.53</v>
+      </c>
+      <c r="P1019" s="3" t="n">
+        <v>725.08</v>
+      </c>
+      <c r="Q1019" s="3" t="n">
+        <v>729.8</v>
+      </c>
+      <c r="R1019" s="2" t="n">
+        <v>621</v>
+      </c>
+      <c r="S1019" s="2" t="n">
+        <v>2993</v>
+      </c>
+      <c r="T1019" s="2" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U1019" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1019" s="2" t="inlineStr"/>
+      <c r="W1019" s="2" t="inlineStr"/>
+      <c r="X1019" s="2" t="inlineStr"/>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1020" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1020" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1020" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1020" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1020" s="6" t="n">
+        <v>1838.6</v>
+      </c>
+      <c r="G1020" s="6" t="n">
+        <v>1864</v>
+      </c>
+      <c r="H1020" s="6" t="n">
+        <v>1874.8</v>
+      </c>
+      <c r="I1020" s="6" t="n">
+        <v>1836.5</v>
+      </c>
+      <c r="J1020" s="6" t="n">
+        <v>1971.02</v>
+      </c>
+      <c r="K1020" s="6" t="n">
+        <v>1874.8</v>
+      </c>
+      <c r="L1020" s="6" t="n">
+        <v>1836.5</v>
+      </c>
+      <c r="M1020" s="6" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="N1020" s="8" t="n">
+        <v>1836.45</v>
+      </c>
+      <c r="O1020" s="7" t="n">
+        <v>1855.7</v>
+      </c>
+      <c r="P1020" s="9" t="n">
+        <v>1817.3</v>
+      </c>
+      <c r="Q1020" s="9" t="n">
+        <v>1798.15</v>
+      </c>
+      <c r="R1020" s="6" t="n">
+        <v>153</v>
+      </c>
+      <c r="S1020" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="T1020" s="6" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1020" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1020" s="6" t="inlineStr"/>
+      <c r="W1020" s="6" t="inlineStr"/>
+      <c r="X1020" s="6" t="inlineStr"/>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1021" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1021" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1021" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1021" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1021" s="6" t="n">
+        <v>1767.3</v>
+      </c>
+      <c r="G1021" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="H1021" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="I1021" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="J1021" s="6" t="n">
+        <v>1838.97</v>
+      </c>
+      <c r="K1021" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="L1021" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="M1021" s="6" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="N1021" s="8" t="n">
+        <v>1756.25</v>
+      </c>
+      <c r="O1021" s="7" t="n">
+        <v>1778.55</v>
+      </c>
+      <c r="P1021" s="9" t="n">
+        <v>1734.05</v>
+      </c>
+      <c r="Q1021" s="9" t="n">
+        <v>1711.85</v>
+      </c>
+      <c r="R1021" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1021" s="6" t="n">
+        <v>2944</v>
+      </c>
+      <c r="T1021" s="6" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1021" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1021" s="6" t="inlineStr"/>
+      <c r="W1021" s="6" t="inlineStr"/>
+      <c r="X1021" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 16-Sep-2026 09:19 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1021"/>
+  <dimension ref="A1:X1025"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81622,6 +81622,326 @@
       <c r="W1021" s="6" t="inlineStr"/>
       <c r="X1021" s="6" t="inlineStr"/>
     </row>
+    <row r="1022">
+      <c r="A1022" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1022" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="C1022" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1022" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1022" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1022" s="2" t="n">
+        <v>416.65</v>
+      </c>
+      <c r="G1022" s="2" t="n">
+        <v>413.6</v>
+      </c>
+      <c r="H1022" s="2" t="n">
+        <v>417</v>
+      </c>
+      <c r="I1022" s="2" t="n">
+        <v>409.35</v>
+      </c>
+      <c r="J1022" s="2" t="n">
+        <v>414.98</v>
+      </c>
+      <c r="K1022" s="2" t="n">
+        <v>417</v>
+      </c>
+      <c r="L1022" s="2" t="n">
+        <v>409.35</v>
+      </c>
+      <c r="M1022" s="2" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="N1022" s="4" t="n">
+        <v>417.05</v>
+      </c>
+      <c r="O1022" s="5" t="n">
+        <v>413.13</v>
+      </c>
+      <c r="P1022" s="3" t="n">
+        <v>420.88</v>
+      </c>
+      <c r="Q1022" s="3" t="n">
+        <v>424.7</v>
+      </c>
+      <c r="R1022" s="2" t="n">
+        <v>765</v>
+      </c>
+      <c r="S1022" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1022" s="2" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1022" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1022" s="2" t="inlineStr"/>
+      <c r="W1022" s="2" t="inlineStr"/>
+      <c r="X1022" s="2" t="inlineStr"/>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="2" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1023" s="2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="C1023" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1023" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1023" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1023" s="2" t="n">
+        <v>720.5</v>
+      </c>
+      <c r="G1023" s="2" t="n">
+        <v>714.9</v>
+      </c>
+      <c r="H1023" s="2" t="n">
+        <v>720.9</v>
+      </c>
+      <c r="I1023" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="J1023" s="2" t="n">
+        <v>712.62</v>
+      </c>
+      <c r="K1023" s="2" t="n">
+        <v>720.9</v>
+      </c>
+      <c r="L1023" s="2" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="M1023" s="2" t="n">
+        <v>10.05</v>
+      </c>
+      <c r="N1023" s="4" t="n">
+        <v>720.95</v>
+      </c>
+      <c r="O1023" s="5" t="n">
+        <v>715.83</v>
+      </c>
+      <c r="P1023" s="3" t="n">
+        <v>725.98</v>
+      </c>
+      <c r="Q1023" s="3" t="n">
+        <v>731</v>
+      </c>
+      <c r="R1023" s="2" t="n">
+        <v>585</v>
+      </c>
+      <c r="S1023" s="2" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1023" s="2" t="n">
+        <v>2943</v>
+      </c>
+      <c r="U1023" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1023" s="2" t="inlineStr"/>
+      <c r="W1023" s="2" t="inlineStr"/>
+      <c r="X1023" s="2" t="inlineStr"/>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1024" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1024" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1024" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1024" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1024" s="6" t="n">
+        <v>1768</v>
+      </c>
+      <c r="G1024" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="H1024" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="I1024" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="J1024" s="6" t="n">
+        <v>1838.92</v>
+      </c>
+      <c r="K1024" s="6" t="n">
+        <v>1800.7</v>
+      </c>
+      <c r="L1024" s="6" t="n">
+        <v>1756.3</v>
+      </c>
+      <c r="M1024" s="6" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="N1024" s="8" t="n">
+        <v>1756.25</v>
+      </c>
+      <c r="O1024" s="7" t="n">
+        <v>1778.55</v>
+      </c>
+      <c r="P1024" s="9" t="n">
+        <v>1734.05</v>
+      </c>
+      <c r="Q1024" s="9" t="n">
+        <v>1711.85</v>
+      </c>
+      <c r="R1024" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1024" s="6" t="n">
+        <v>2944</v>
+      </c>
+      <c r="T1024" s="6" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1024" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1024" s="6" t="inlineStr"/>
+      <c r="W1024" s="6" t="inlineStr"/>
+      <c r="X1024" s="6" t="inlineStr"/>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="6" t="inlineStr">
+        <is>
+          <t>16-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1025" s="6" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="C1025" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1025" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1025" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1025" s="6" t="n">
+        <v>979</v>
+      </c>
+      <c r="G1025" s="6" t="n">
+        <v>979</v>
+      </c>
+      <c r="H1025" s="6" t="n">
+        <v>990.3</v>
+      </c>
+      <c r="I1025" s="6" t="n">
+        <v>972.6</v>
+      </c>
+      <c r="J1025" s="6" t="n">
+        <v>1061.06</v>
+      </c>
+      <c r="K1025" s="6" t="n">
+        <v>990.3</v>
+      </c>
+      <c r="L1025" s="6" t="n">
+        <v>972.6</v>
+      </c>
+      <c r="M1025" s="6" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="N1025" s="8" t="n">
+        <v>972.55</v>
+      </c>
+      <c r="O1025" s="7" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="P1025" s="9" t="n">
+        <v>963.7</v>
+      </c>
+      <c r="Q1025" s="9" t="n">
+        <v>954.85</v>
+      </c>
+      <c r="R1025" s="6" t="n">
+        <v>333</v>
+      </c>
+      <c r="S1025" s="6" t="n">
+        <v>2980</v>
+      </c>
+      <c r="T1025" s="6" t="n">
+        <v>2947</v>
+      </c>
+      <c r="U1025" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1025" s="6" t="inlineStr"/>
+      <c r="W1025" s="6" t="inlineStr"/>
+      <c r="X1025" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 17-Sep-2026 08:44 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1025"/>
+  <dimension ref="A1:X1029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81942,6 +81942,326 @@
       <c r="W1025" s="6" t="inlineStr"/>
       <c r="X1025" s="6" t="inlineStr"/>
     </row>
+    <row r="1026">
+      <c r="A1026" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1026" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C1026" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1026" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1026" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1026" s="2" t="n">
+        <v>1733.8</v>
+      </c>
+      <c r="G1026" s="2" t="n">
+        <v>1731</v>
+      </c>
+      <c r="H1026" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="I1026" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="J1026" s="2" t="n">
+        <v>1694.96</v>
+      </c>
+      <c r="K1026" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="L1026" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="M1026" s="2" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="N1026" s="4" t="n">
+        <v>1738.85</v>
+      </c>
+      <c r="O1026" s="5" t="n">
+        <v>1731.9</v>
+      </c>
+      <c r="P1026" s="3" t="n">
+        <v>1745.7</v>
+      </c>
+      <c r="Q1026" s="3" t="n">
+        <v>1752.55</v>
+      </c>
+      <c r="R1026" s="2" t="n">
+        <v>287</v>
+      </c>
+      <c r="S1026" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T1026" s="2" t="n">
+        <v>1966</v>
+      </c>
+      <c r="U1026" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1026" s="2" t="inlineStr"/>
+      <c r="W1026" s="2" t="inlineStr"/>
+      <c r="X1026" s="2" t="inlineStr"/>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1027" s="2" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="C1027" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1027" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1027" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1027" s="2" t="n">
+        <v>11466</v>
+      </c>
+      <c r="G1027" s="2" t="n">
+        <v>11568</v>
+      </c>
+      <c r="H1027" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="I1027" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="J1027" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1027" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="L1027" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="M1027" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="N1027" s="4" t="n">
+        <v>11576.05</v>
+      </c>
+      <c r="O1027" s="5" t="n">
+        <v>11505.45</v>
+      </c>
+      <c r="P1027" s="3" t="n">
+        <v>11646.55</v>
+      </c>
+      <c r="Q1027" s="3" t="n">
+        <v>11717.05</v>
+      </c>
+      <c r="R1027" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="S1027" s="2" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1027" s="2" t="n">
+        <v>2961</v>
+      </c>
+      <c r="U1027" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1027" s="2" t="inlineStr"/>
+      <c r="W1027" s="2" t="inlineStr"/>
+      <c r="X1027" s="2" t="inlineStr"/>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1028" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C1028" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1028" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1028" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1028" s="6" t="n">
+        <v>987.1</v>
+      </c>
+      <c r="G1028" s="6" t="n">
+        <v>991.2</v>
+      </c>
+      <c r="H1028" s="6" t="n">
+        <v>1000.9</v>
+      </c>
+      <c r="I1028" s="6" t="n">
+        <v>985.2</v>
+      </c>
+      <c r="J1028" s="6" t="n">
+        <v>1021.01</v>
+      </c>
+      <c r="K1028" s="6" t="n">
+        <v>1000.9</v>
+      </c>
+      <c r="L1028" s="6" t="n">
+        <v>985.2</v>
+      </c>
+      <c r="M1028" s="6" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="N1028" s="8" t="n">
+        <v>985.15</v>
+      </c>
+      <c r="O1028" s="7" t="n">
+        <v>993.1</v>
+      </c>
+      <c r="P1028" s="9" t="n">
+        <v>977.3</v>
+      </c>
+      <c r="Q1028" s="9" t="n">
+        <v>969.45</v>
+      </c>
+      <c r="R1028" s="6" t="n">
+        <v>375</v>
+      </c>
+      <c r="S1028" s="6" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1028" s="6" t="n">
+        <v>2944</v>
+      </c>
+      <c r="U1028" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1028" s="6" t="inlineStr"/>
+      <c r="W1028" s="6" t="inlineStr"/>
+      <c r="X1028" s="6" t="inlineStr"/>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1029" s="6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C1029" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1029" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1029" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1029" s="6" t="n">
+        <v>1241.4</v>
+      </c>
+      <c r="G1029" s="6" t="n">
+        <v>1238</v>
+      </c>
+      <c r="H1029" s="6" t="n">
+        <v>1257.6</v>
+      </c>
+      <c r="I1029" s="6" t="n">
+        <v>1233</v>
+      </c>
+      <c r="J1029" s="6" t="n">
+        <v>1252.19</v>
+      </c>
+      <c r="K1029" s="6" t="n">
+        <v>1257.6</v>
+      </c>
+      <c r="L1029" s="6" t="n">
+        <v>1233</v>
+      </c>
+      <c r="M1029" s="6" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="N1029" s="8" t="n">
+        <v>1232.95</v>
+      </c>
+      <c r="O1029" s="7" t="n">
+        <v>1245.35</v>
+      </c>
+      <c r="P1029" s="9" t="n">
+        <v>1220.65</v>
+      </c>
+      <c r="Q1029" s="9" t="n">
+        <v>1208.35</v>
+      </c>
+      <c r="R1029" s="6" t="n">
+        <v>240</v>
+      </c>
+      <c r="S1029" s="6" t="n">
+        <v>2976</v>
+      </c>
+      <c r="T1029" s="6" t="n">
+        <v>2952</v>
+      </c>
+      <c r="U1029" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1029" s="6" t="inlineStr"/>
+      <c r="W1029" s="6" t="inlineStr"/>
+      <c r="X1029" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 17-Sep-2026 08:51 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1029"/>
+  <dimension ref="A1:X1033"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -82262,6 +82262,326 @@
       <c r="W1029" s="6" t="inlineStr"/>
       <c r="X1029" s="6" t="inlineStr"/>
     </row>
+    <row r="1030">
+      <c r="A1030" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1030" s="2" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="C1030" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1030" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1030" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1030" s="2" t="n">
+        <v>11480</v>
+      </c>
+      <c r="G1030" s="2" t="n">
+        <v>11568</v>
+      </c>
+      <c r="H1030" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="I1030" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="J1030" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1030" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="L1030" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="M1030" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="N1030" s="4" t="n">
+        <v>11576.05</v>
+      </c>
+      <c r="O1030" s="5" t="n">
+        <v>11505.45</v>
+      </c>
+      <c r="P1030" s="3" t="n">
+        <v>11646.55</v>
+      </c>
+      <c r="Q1030" s="3" t="n">
+        <v>11717.05</v>
+      </c>
+      <c r="R1030" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="S1030" s="2" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1030" s="2" t="n">
+        <v>2961</v>
+      </c>
+      <c r="U1030" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1030" s="2" t="inlineStr"/>
+      <c r="W1030" s="2" t="inlineStr"/>
+      <c r="X1030" s="2" t="inlineStr"/>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1031" s="2" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="C1031" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1031" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1031" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1031" s="2" t="n">
+        <v>5311.5</v>
+      </c>
+      <c r="G1031" s="2" t="n">
+        <v>5253.5</v>
+      </c>
+      <c r="H1031" s="2" t="n">
+        <v>5341</v>
+      </c>
+      <c r="I1031" s="2" t="n">
+        <v>5243.5</v>
+      </c>
+      <c r="J1031" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1031" s="2" t="n">
+        <v>5341</v>
+      </c>
+      <c r="L1031" s="2" t="n">
+        <v>5243.5</v>
+      </c>
+      <c r="M1031" s="2" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="N1031" s="4" t="n">
+        <v>5341.05</v>
+      </c>
+      <c r="O1031" s="5" t="n">
+        <v>5292.2</v>
+      </c>
+      <c r="P1031" s="3" t="n">
+        <v>5389.8</v>
+      </c>
+      <c r="Q1031" s="3" t="n">
+        <v>5438.55</v>
+      </c>
+      <c r="R1031" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="S1031" s="2" t="n">
+        <v>2931</v>
+      </c>
+      <c r="T1031" s="2" t="n">
+        <v>2925</v>
+      </c>
+      <c r="U1031" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1031" s="2" t="inlineStr"/>
+      <c r="W1031" s="2" t="inlineStr"/>
+      <c r="X1031" s="2" t="inlineStr"/>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1032" s="6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C1032" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1032" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1032" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1032" s="6" t="n">
+        <v>1241.1</v>
+      </c>
+      <c r="G1032" s="6" t="n">
+        <v>1238</v>
+      </c>
+      <c r="H1032" s="6" t="n">
+        <v>1257.6</v>
+      </c>
+      <c r="I1032" s="6" t="n">
+        <v>1233</v>
+      </c>
+      <c r="J1032" s="6" t="n">
+        <v>1252.19</v>
+      </c>
+      <c r="K1032" s="6" t="n">
+        <v>1257.6</v>
+      </c>
+      <c r="L1032" s="6" t="n">
+        <v>1233</v>
+      </c>
+      <c r="M1032" s="6" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="N1032" s="8" t="n">
+        <v>1232.95</v>
+      </c>
+      <c r="O1032" s="7" t="n">
+        <v>1245.35</v>
+      </c>
+      <c r="P1032" s="9" t="n">
+        <v>1220.65</v>
+      </c>
+      <c r="Q1032" s="9" t="n">
+        <v>1208.35</v>
+      </c>
+      <c r="R1032" s="6" t="n">
+        <v>240</v>
+      </c>
+      <c r="S1032" s="6" t="n">
+        <v>2976</v>
+      </c>
+      <c r="T1032" s="6" t="n">
+        <v>2952</v>
+      </c>
+      <c r="U1032" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1032" s="6" t="inlineStr"/>
+      <c r="W1032" s="6" t="inlineStr"/>
+      <c r="X1032" s="6" t="inlineStr"/>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1033" s="6" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="C1033" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1033" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1033" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1033" s="6" t="n">
+        <v>232.39</v>
+      </c>
+      <c r="G1033" s="6" t="n">
+        <v>233.6</v>
+      </c>
+      <c r="H1033" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="I1033" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="J1033" s="6" t="n">
+        <v>239.13</v>
+      </c>
+      <c r="K1033" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="L1033" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="M1033" s="6" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="N1033" s="8" t="n">
+        <v>232.05</v>
+      </c>
+      <c r="O1033" s="7" t="n">
+        <v>234.33</v>
+      </c>
+      <c r="P1033" s="9" t="n">
+        <v>229.87</v>
+      </c>
+      <c r="Q1033" s="9" t="n">
+        <v>227.69</v>
+      </c>
+      <c r="R1033" s="6" t="n">
+        <v>1314</v>
+      </c>
+      <c r="S1033" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1033" s="6" t="n">
+        <v>2865</v>
+      </c>
+      <c r="U1033" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1033" s="6" t="inlineStr"/>
+      <c r="W1033" s="6" t="inlineStr"/>
+      <c r="X1033" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 17-Sep-2026 09:21 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1033"/>
+  <dimension ref="A1:X1037"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -82582,6 +82582,326 @@
       <c r="W1033" s="6" t="inlineStr"/>
       <c r="X1033" s="6" t="inlineStr"/>
     </row>
+    <row r="1034">
+      <c r="A1034" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1034" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C1034" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1034" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1034" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1034" s="2" t="n">
+        <v>1733.3</v>
+      </c>
+      <c r="G1034" s="2" t="n">
+        <v>1731</v>
+      </c>
+      <c r="H1034" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="I1034" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="J1034" s="2" t="n">
+        <v>1695</v>
+      </c>
+      <c r="K1034" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="L1034" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="M1034" s="2" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="N1034" s="4" t="n">
+        <v>1738.85</v>
+      </c>
+      <c r="O1034" s="5" t="n">
+        <v>1731.9</v>
+      </c>
+      <c r="P1034" s="3" t="n">
+        <v>1745.7</v>
+      </c>
+      <c r="Q1034" s="3" t="n">
+        <v>1752.55</v>
+      </c>
+      <c r="R1034" s="2" t="n">
+        <v>287</v>
+      </c>
+      <c r="S1034" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T1034" s="2" t="n">
+        <v>1966</v>
+      </c>
+      <c r="U1034" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1034" s="2" t="inlineStr"/>
+      <c r="W1034" s="2" t="inlineStr"/>
+      <c r="X1034" s="2" t="inlineStr"/>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1035" s="2" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="C1035" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1035" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1035" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1035" s="2" t="n">
+        <v>7527.5</v>
+      </c>
+      <c r="G1035" s="2" t="n">
+        <v>7495</v>
+      </c>
+      <c r="H1035" s="2" t="n">
+        <v>7550.5</v>
+      </c>
+      <c r="I1035" s="2" t="n">
+        <v>7489</v>
+      </c>
+      <c r="J1035" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1035" s="2" t="n">
+        <v>7550.5</v>
+      </c>
+      <c r="L1035" s="2" t="n">
+        <v>7489</v>
+      </c>
+      <c r="M1035" s="2" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="N1035" s="4" t="n">
+        <v>7550.55</v>
+      </c>
+      <c r="O1035" s="5" t="n">
+        <v>7519.7</v>
+      </c>
+      <c r="P1035" s="3" t="n">
+        <v>7581.3</v>
+      </c>
+      <c r="Q1035" s="3" t="n">
+        <v>7612.05</v>
+      </c>
+      <c r="R1035" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="S1035" s="2" t="n">
+        <v>2036</v>
+      </c>
+      <c r="T1035" s="2" t="n">
+        <v>2030</v>
+      </c>
+      <c r="U1035" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1035" s="2" t="inlineStr"/>
+      <c r="W1035" s="2" t="inlineStr"/>
+      <c r="X1035" s="2" t="inlineStr"/>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1036" s="6" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C1036" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1036" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1036" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1036" s="6" t="n">
+        <v>1350.9</v>
+      </c>
+      <c r="G1036" s="6" t="n">
+        <v>1352</v>
+      </c>
+      <c r="H1036" s="6" t="n">
+        <v>1363</v>
+      </c>
+      <c r="I1036" s="6" t="n">
+        <v>1349.1</v>
+      </c>
+      <c r="J1036" s="6" t="n">
+        <v>1410.63</v>
+      </c>
+      <c r="K1036" s="6" t="n">
+        <v>1363</v>
+      </c>
+      <c r="L1036" s="6" t="n">
+        <v>1349.1</v>
+      </c>
+      <c r="M1036" s="6" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="N1036" s="8" t="n">
+        <v>1349.05</v>
+      </c>
+      <c r="O1036" s="7" t="n">
+        <v>1356.1</v>
+      </c>
+      <c r="P1036" s="9" t="n">
+        <v>1342.1</v>
+      </c>
+      <c r="Q1036" s="9" t="n">
+        <v>1335.15</v>
+      </c>
+      <c r="R1036" s="6" t="n">
+        <v>370</v>
+      </c>
+      <c r="S1036" s="6" t="n">
+        <v>2608</v>
+      </c>
+      <c r="T1036" s="6" t="n">
+        <v>2572</v>
+      </c>
+      <c r="U1036" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1036" s="6" t="inlineStr"/>
+      <c r="W1036" s="6" t="inlineStr"/>
+      <c r="X1036" s="6" t="inlineStr"/>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1037" s="6" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="C1037" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1037" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1037" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1037" s="6" t="n">
+        <v>232.59</v>
+      </c>
+      <c r="G1037" s="6" t="n">
+        <v>233.6</v>
+      </c>
+      <c r="H1037" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="I1037" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="J1037" s="6" t="n">
+        <v>239.13</v>
+      </c>
+      <c r="K1037" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="L1037" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="M1037" s="6" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="N1037" s="8" t="n">
+        <v>232.05</v>
+      </c>
+      <c r="O1037" s="7" t="n">
+        <v>234.33</v>
+      </c>
+      <c r="P1037" s="9" t="n">
+        <v>229.87</v>
+      </c>
+      <c r="Q1037" s="9" t="n">
+        <v>227.69</v>
+      </c>
+      <c r="R1037" s="6" t="n">
+        <v>1314</v>
+      </c>
+      <c r="S1037" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1037" s="6" t="n">
+        <v>2865</v>
+      </c>
+      <c r="U1037" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1037" s="6" t="inlineStr"/>
+      <c r="W1037" s="6" t="inlineStr"/>
+      <c r="X1037" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 17-Sep-2026 09:28 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1037"/>
+  <dimension ref="A1:X1041"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -82902,6 +82902,326 @@
       <c r="W1037" s="6" t="inlineStr"/>
       <c r="X1037" s="6" t="inlineStr"/>
     </row>
+    <row r="1038">
+      <c r="A1038" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1038" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C1038" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1038" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1038" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1038" s="2" t="n">
+        <v>1731.4</v>
+      </c>
+      <c r="G1038" s="2" t="n">
+        <v>1731</v>
+      </c>
+      <c r="H1038" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="I1038" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="J1038" s="2" t="n">
+        <v>1695.02</v>
+      </c>
+      <c r="K1038" s="2" t="n">
+        <v>1738.8</v>
+      </c>
+      <c r="L1038" s="2" t="n">
+        <v>1725.1</v>
+      </c>
+      <c r="M1038" s="2" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="N1038" s="4" t="n">
+        <v>1738.85</v>
+      </c>
+      <c r="O1038" s="5" t="n">
+        <v>1731.9</v>
+      </c>
+      <c r="P1038" s="3" t="n">
+        <v>1745.7</v>
+      </c>
+      <c r="Q1038" s="3" t="n">
+        <v>1752.55</v>
+      </c>
+      <c r="R1038" s="2" t="n">
+        <v>287</v>
+      </c>
+      <c r="S1038" s="2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="T1038" s="2" t="n">
+        <v>1966</v>
+      </c>
+      <c r="U1038" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1038" s="2" t="inlineStr"/>
+      <c r="W1038" s="2" t="inlineStr"/>
+      <c r="X1038" s="2" t="inlineStr"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="2" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1039" s="2" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="C1039" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1039" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1039" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1039" s="2" t="n">
+        <v>11504</v>
+      </c>
+      <c r="G1039" s="2" t="n">
+        <v>11568</v>
+      </c>
+      <c r="H1039" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="I1039" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="J1039" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1039" s="2" t="n">
+        <v>11576</v>
+      </c>
+      <c r="L1039" s="2" t="n">
+        <v>11435</v>
+      </c>
+      <c r="M1039" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="N1039" s="4" t="n">
+        <v>11576.05</v>
+      </c>
+      <c r="O1039" s="5" t="n">
+        <v>11505.45</v>
+      </c>
+      <c r="P1039" s="3" t="n">
+        <v>11646.55</v>
+      </c>
+      <c r="Q1039" s="3" t="n">
+        <v>11717.05</v>
+      </c>
+      <c r="R1039" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="S1039" s="2" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1039" s="2" t="n">
+        <v>2961</v>
+      </c>
+      <c r="U1039" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1039" s="2" t="inlineStr"/>
+      <c r="W1039" s="2" t="inlineStr"/>
+      <c r="X1039" s="2" t="inlineStr"/>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1040" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="C1040" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1040" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1040" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1040" s="6" t="n">
+        <v>986.9</v>
+      </c>
+      <c r="G1040" s="6" t="n">
+        <v>991.2</v>
+      </c>
+      <c r="H1040" s="6" t="n">
+        <v>1000.9</v>
+      </c>
+      <c r="I1040" s="6" t="n">
+        <v>985.2</v>
+      </c>
+      <c r="J1040" s="6" t="n">
+        <v>1020.84</v>
+      </c>
+      <c r="K1040" s="6" t="n">
+        <v>1000.9</v>
+      </c>
+      <c r="L1040" s="6" t="n">
+        <v>985.2</v>
+      </c>
+      <c r="M1040" s="6" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="N1040" s="8" t="n">
+        <v>985.15</v>
+      </c>
+      <c r="O1040" s="7" t="n">
+        <v>993.1</v>
+      </c>
+      <c r="P1040" s="9" t="n">
+        <v>977.3</v>
+      </c>
+      <c r="Q1040" s="9" t="n">
+        <v>969.45</v>
+      </c>
+      <c r="R1040" s="6" t="n">
+        <v>375</v>
+      </c>
+      <c r="S1040" s="6" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1040" s="6" t="n">
+        <v>2944</v>
+      </c>
+      <c r="U1040" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1040" s="6" t="inlineStr"/>
+      <c r="W1040" s="6" t="inlineStr"/>
+      <c r="X1040" s="6" t="inlineStr"/>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="6" t="inlineStr">
+        <is>
+          <t>17-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1041" s="6" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="C1041" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1041" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1041" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1041" s="6" t="n">
+        <v>232.65</v>
+      </c>
+      <c r="G1041" s="6" t="n">
+        <v>233.6</v>
+      </c>
+      <c r="H1041" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="I1041" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="J1041" s="6" t="n">
+        <v>239.13</v>
+      </c>
+      <c r="K1041" s="6" t="n">
+        <v>236.46</v>
+      </c>
+      <c r="L1041" s="6" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="M1041" s="6" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="N1041" s="8" t="n">
+        <v>232.05</v>
+      </c>
+      <c r="O1041" s="7" t="n">
+        <v>234.33</v>
+      </c>
+      <c r="P1041" s="9" t="n">
+        <v>229.87</v>
+      </c>
+      <c r="Q1041" s="9" t="n">
+        <v>227.69</v>
+      </c>
+      <c r="R1041" s="6" t="n">
+        <v>1314</v>
+      </c>
+      <c r="S1041" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1041" s="6" t="n">
+        <v>2865</v>
+      </c>
+      <c r="U1041" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1041" s="6" t="inlineStr"/>
+      <c r="W1041" s="6" t="inlineStr"/>
+      <c r="X1041" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 18-Sep-2026 08:19 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1041"/>
+  <dimension ref="A1:X1045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -83222,6 +83222,326 @@
       <c r="W1041" s="6" t="inlineStr"/>
       <c r="X1041" s="6" t="inlineStr"/>
     </row>
+    <row r="1042">
+      <c r="A1042" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1042" s="2" t="inlineStr">
+        <is>
+          <t>BHEL</t>
+        </is>
+      </c>
+      <c r="C1042" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1042" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1042" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1042" s="2" t="n">
+        <v>431.4</v>
+      </c>
+      <c r="G1042" s="2" t="n">
+        <v>428.4</v>
+      </c>
+      <c r="H1042" s="2" t="n">
+        <v>435.5</v>
+      </c>
+      <c r="I1042" s="2" t="n">
+        <v>427.25</v>
+      </c>
+      <c r="J1042" s="2" t="n">
+        <v>425.78</v>
+      </c>
+      <c r="K1042" s="2" t="n">
+        <v>435.5</v>
+      </c>
+      <c r="L1042" s="2" t="n">
+        <v>427.25</v>
+      </c>
+      <c r="M1042" s="2" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="N1042" s="4" t="n">
+        <v>435.55</v>
+      </c>
+      <c r="O1042" s="5" t="n">
+        <v>431.33</v>
+      </c>
+      <c r="P1042" s="3" t="n">
+        <v>439.68</v>
+      </c>
+      <c r="Q1042" s="3" t="n">
+        <v>443.8</v>
+      </c>
+      <c r="R1042" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="S1042" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1042" s="2" t="n">
+        <v>2924</v>
+      </c>
+      <c r="U1042" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1042" s="2" t="inlineStr"/>
+      <c r="W1042" s="2" t="inlineStr"/>
+      <c r="X1042" s="2" t="inlineStr"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1043" s="2" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1043" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1043" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1043" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1043" s="2" t="n">
+        <v>559.65</v>
+      </c>
+      <c r="G1043" s="2" t="n">
+        <v>557.1</v>
+      </c>
+      <c r="H1043" s="2" t="n">
+        <v>564.95</v>
+      </c>
+      <c r="I1043" s="2" t="n">
+        <v>555.15</v>
+      </c>
+      <c r="J1043" s="2" t="n">
+        <v>538.17</v>
+      </c>
+      <c r="K1043" s="2" t="n">
+        <v>564.95</v>
+      </c>
+      <c r="L1043" s="2" t="n">
+        <v>555.15</v>
+      </c>
+      <c r="M1043" s="2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="N1043" s="4" t="n">
+        <v>565</v>
+      </c>
+      <c r="O1043" s="5" t="n">
+        <v>560</v>
+      </c>
+      <c r="P1043" s="3" t="n">
+        <v>569.9</v>
+      </c>
+      <c r="Q1043" s="3" t="n">
+        <v>574.8</v>
+      </c>
+      <c r="R1043" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="S1043" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1043" s="2" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1043" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1043" s="2" t="inlineStr"/>
+      <c r="W1043" s="2" t="inlineStr"/>
+      <c r="X1043" s="2" t="inlineStr"/>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1044" s="6" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C1044" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1044" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1044" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1044" s="6" t="n">
+        <v>2115.6</v>
+      </c>
+      <c r="G1044" s="6" t="n">
+        <v>2177.2</v>
+      </c>
+      <c r="H1044" s="6" t="n">
+        <v>2177.3</v>
+      </c>
+      <c r="I1044" s="6" t="n">
+        <v>2111</v>
+      </c>
+      <c r="J1044" s="6" t="n">
+        <v>2268.77</v>
+      </c>
+      <c r="K1044" s="6" t="n">
+        <v>2177.3</v>
+      </c>
+      <c r="L1044" s="6" t="n">
+        <v>2111</v>
+      </c>
+      <c r="M1044" s="6" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="N1044" s="8" t="n">
+        <v>2110.95</v>
+      </c>
+      <c r="O1044" s="7" t="n">
+        <v>2144.2</v>
+      </c>
+      <c r="P1044" s="9" t="n">
+        <v>2077.8</v>
+      </c>
+      <c r="Q1044" s="9" t="n">
+        <v>2044.65</v>
+      </c>
+      <c r="R1044" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="S1044" s="6" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T1044" s="6" t="n">
+        <v>2983</v>
+      </c>
+      <c r="U1044" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1044" s="6" t="inlineStr"/>
+      <c r="W1044" s="6" t="inlineStr"/>
+      <c r="X1044" s="6" t="inlineStr"/>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1045" s="6" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="C1045" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1045" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1045" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1045" s="6" t="n">
+        <v>1538.9</v>
+      </c>
+      <c r="G1045" s="6" t="n">
+        <v>1558.3</v>
+      </c>
+      <c r="H1045" s="6" t="n">
+        <v>1561.2</v>
+      </c>
+      <c r="I1045" s="6" t="n">
+        <v>1523.1</v>
+      </c>
+      <c r="J1045" s="6" t="n">
+        <v>1584.34</v>
+      </c>
+      <c r="K1045" s="6" t="n">
+        <v>1561.2</v>
+      </c>
+      <c r="L1045" s="6" t="n">
+        <v>1523.1</v>
+      </c>
+      <c r="M1045" s="6" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="N1045" s="8" t="n">
+        <v>1523.05</v>
+      </c>
+      <c r="O1045" s="7" t="n">
+        <v>1542.2</v>
+      </c>
+      <c r="P1045" s="9" t="n">
+        <v>1504</v>
+      </c>
+      <c r="Q1045" s="9" t="n">
+        <v>1484.95</v>
+      </c>
+      <c r="R1045" s="6" t="n">
+        <v>156</v>
+      </c>
+      <c r="S1045" s="6" t="n">
+        <v>2987</v>
+      </c>
+      <c r="T1045" s="6" t="n">
+        <v>2972</v>
+      </c>
+      <c r="U1045" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1045" s="6" t="inlineStr"/>
+      <c r="W1045" s="6" t="inlineStr"/>
+      <c r="X1045" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 18-Sep-2026 08:26 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1045"/>
+  <dimension ref="A1:X1049"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -83542,6 +83542,326 @@
       <c r="W1045" s="6" t="inlineStr"/>
       <c r="X1045" s="6" t="inlineStr"/>
     </row>
+    <row r="1046">
+      <c r="A1046" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1046" s="2" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1046" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1046" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1046" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1046" s="2" t="n">
+        <v>1762.7</v>
+      </c>
+      <c r="G1046" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="H1046" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="I1046" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="J1046" s="2" t="n">
+        <v>1736.84</v>
+      </c>
+      <c r="K1046" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="L1046" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="M1046" s="2" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="N1046" s="4" t="n">
+        <v>1770.05</v>
+      </c>
+      <c r="O1046" s="5" t="n">
+        <v>1760.6</v>
+      </c>
+      <c r="P1046" s="3" t="n">
+        <v>1779.4</v>
+      </c>
+      <c r="Q1046" s="3" t="n">
+        <v>1788.75</v>
+      </c>
+      <c r="R1046" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="S1046" s="2" t="n">
+        <v>2665</v>
+      </c>
+      <c r="T1046" s="2" t="n">
+        <v>2637</v>
+      </c>
+      <c r="U1046" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1046" s="2" t="inlineStr"/>
+      <c r="W1046" s="2" t="inlineStr"/>
+      <c r="X1046" s="2" t="inlineStr"/>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1047" s="2" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1047" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1047" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1047" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1047" s="2" t="n">
+        <v>559.5</v>
+      </c>
+      <c r="G1047" s="2" t="n">
+        <v>557.1</v>
+      </c>
+      <c r="H1047" s="2" t="n">
+        <v>564.95</v>
+      </c>
+      <c r="I1047" s="2" t="n">
+        <v>555.15</v>
+      </c>
+      <c r="J1047" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1047" s="2" t="n">
+        <v>564.95</v>
+      </c>
+      <c r="L1047" s="2" t="n">
+        <v>555.15</v>
+      </c>
+      <c r="M1047" s="2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="N1047" s="4" t="n">
+        <v>565</v>
+      </c>
+      <c r="O1047" s="5" t="n">
+        <v>560</v>
+      </c>
+      <c r="P1047" s="3" t="n">
+        <v>569.9</v>
+      </c>
+      <c r="Q1047" s="3" t="n">
+        <v>574.8</v>
+      </c>
+      <c r="R1047" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="S1047" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1047" s="2" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1047" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1047" s="2" t="inlineStr"/>
+      <c r="W1047" s="2" t="inlineStr"/>
+      <c r="X1047" s="2" t="inlineStr"/>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1048" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1048" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1048" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1048" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1048" s="6" t="n">
+        <v>1043.4</v>
+      </c>
+      <c r="G1048" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="H1048" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="I1048" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="J1048" s="6" t="n">
+        <v>1100.22</v>
+      </c>
+      <c r="K1048" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="L1048" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="M1048" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N1048" s="8" t="n">
+        <v>1039.25</v>
+      </c>
+      <c r="O1048" s="7" t="n">
+        <v>1050.65</v>
+      </c>
+      <c r="P1048" s="9" t="n">
+        <v>1027.95</v>
+      </c>
+      <c r="Q1048" s="9" t="n">
+        <v>1016.65</v>
+      </c>
+      <c r="R1048" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1048" s="6" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T1048" s="6" t="n">
+        <v>2949</v>
+      </c>
+      <c r="U1048" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1048" s="6" t="inlineStr"/>
+      <c r="W1048" s="6" t="inlineStr"/>
+      <c r="X1048" s="6" t="inlineStr"/>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1049" s="6" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C1049" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1049" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1049" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1049" s="6" t="n">
+        <v>2115.7</v>
+      </c>
+      <c r="G1049" s="6" t="n">
+        <v>2177.2</v>
+      </c>
+      <c r="H1049" s="6" t="n">
+        <v>2177.3</v>
+      </c>
+      <c r="I1049" s="6" t="n">
+        <v>2111</v>
+      </c>
+      <c r="J1049" s="6" t="n">
+        <v>2268.69</v>
+      </c>
+      <c r="K1049" s="6" t="n">
+        <v>2177.3</v>
+      </c>
+      <c r="L1049" s="6" t="n">
+        <v>2111</v>
+      </c>
+      <c r="M1049" s="6" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="N1049" s="8" t="n">
+        <v>2110.95</v>
+      </c>
+      <c r="O1049" s="7" t="n">
+        <v>2144.2</v>
+      </c>
+      <c r="P1049" s="9" t="n">
+        <v>2077.8</v>
+      </c>
+      <c r="Q1049" s="9" t="n">
+        <v>2044.65</v>
+      </c>
+      <c r="R1049" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="S1049" s="6" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T1049" s="6" t="n">
+        <v>2983</v>
+      </c>
+      <c r="U1049" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1049" s="6" t="inlineStr"/>
+      <c r="W1049" s="6" t="inlineStr"/>
+      <c r="X1049" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 18-Sep-2026 08:56 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1049"/>
+  <dimension ref="A1:X1053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -83862,6 +83862,326 @@
       <c r="W1049" s="6" t="inlineStr"/>
       <c r="X1049" s="6" t="inlineStr"/>
     </row>
+    <row r="1050">
+      <c r="A1050" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1050" s="2" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1050" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1050" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1050" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1050" s="2" t="n">
+        <v>1761.4</v>
+      </c>
+      <c r="G1050" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="H1050" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="I1050" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="J1050" s="2" t="n">
+        <v>1736.88</v>
+      </c>
+      <c r="K1050" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="L1050" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="M1050" s="2" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="N1050" s="4" t="n">
+        <v>1770.05</v>
+      </c>
+      <c r="O1050" s="5" t="n">
+        <v>1760.6</v>
+      </c>
+      <c r="P1050" s="3" t="n">
+        <v>1779.4</v>
+      </c>
+      <c r="Q1050" s="3" t="n">
+        <v>1788.75</v>
+      </c>
+      <c r="R1050" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="S1050" s="2" t="n">
+        <v>2665</v>
+      </c>
+      <c r="T1050" s="2" t="n">
+        <v>2637</v>
+      </c>
+      <c r="U1050" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1050" s="2" t="inlineStr"/>
+      <c r="W1050" s="2" t="inlineStr"/>
+      <c r="X1050" s="2" t="inlineStr"/>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1051" s="2" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1051" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1051" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1051" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1051" s="2" t="n">
+        <v>1864</v>
+      </c>
+      <c r="G1051" s="2" t="n">
+        <v>1857.2</v>
+      </c>
+      <c r="H1051" s="2" t="n">
+        <v>1871.4</v>
+      </c>
+      <c r="I1051" s="2" t="n">
+        <v>1854.3</v>
+      </c>
+      <c r="J1051" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1051" s="2" t="n">
+        <v>1871.4</v>
+      </c>
+      <c r="L1051" s="2" t="n">
+        <v>1854.3</v>
+      </c>
+      <c r="M1051" s="2" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="N1051" s="4" t="n">
+        <v>1871.45</v>
+      </c>
+      <c r="O1051" s="5" t="n">
+        <v>1862.8</v>
+      </c>
+      <c r="P1051" s="3" t="n">
+        <v>1880</v>
+      </c>
+      <c r="Q1051" s="3" t="n">
+        <v>1888.55</v>
+      </c>
+      <c r="R1051" s="2" t="n">
+        <v>267</v>
+      </c>
+      <c r="S1051" s="2" t="n">
+        <v>2310</v>
+      </c>
+      <c r="T1051" s="2" t="n">
+        <v>2283</v>
+      </c>
+      <c r="U1051" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1051" s="2" t="inlineStr"/>
+      <c r="W1051" s="2" t="inlineStr"/>
+      <c r="X1051" s="2" t="inlineStr"/>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1052" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1052" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1052" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1052" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1052" s="6" t="n">
+        <v>1044</v>
+      </c>
+      <c r="G1052" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="H1052" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="I1052" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="J1052" s="6" t="n">
+        <v>1099.98</v>
+      </c>
+      <c r="K1052" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="L1052" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="M1052" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N1052" s="8" t="n">
+        <v>1039.25</v>
+      </c>
+      <c r="O1052" s="7" t="n">
+        <v>1050.65</v>
+      </c>
+      <c r="P1052" s="9" t="n">
+        <v>1027.95</v>
+      </c>
+      <c r="Q1052" s="9" t="n">
+        <v>1016.65</v>
+      </c>
+      <c r="R1052" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1052" s="6" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T1052" s="6" t="n">
+        <v>2949</v>
+      </c>
+      <c r="U1052" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1052" s="6" t="inlineStr"/>
+      <c r="W1052" s="6" t="inlineStr"/>
+      <c r="X1052" s="6" t="inlineStr"/>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1053" s="6" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="C1053" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1053" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1053" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1053" s="6" t="n">
+        <v>1242.2</v>
+      </c>
+      <c r="G1053" s="6" t="n">
+        <v>1258.3</v>
+      </c>
+      <c r="H1053" s="6" t="n">
+        <v>1260.8</v>
+      </c>
+      <c r="I1053" s="6" t="n">
+        <v>1235.6</v>
+      </c>
+      <c r="J1053" s="6" t="n">
+        <v>1286.39</v>
+      </c>
+      <c r="K1053" s="6" t="n">
+        <v>1260.8</v>
+      </c>
+      <c r="L1053" s="6" t="n">
+        <v>1235.6</v>
+      </c>
+      <c r="M1053" s="6" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="N1053" s="8" t="n">
+        <v>1235.55</v>
+      </c>
+      <c r="O1053" s="7" t="n">
+        <v>1248.25</v>
+      </c>
+      <c r="P1053" s="9" t="n">
+        <v>1222.95</v>
+      </c>
+      <c r="Q1053" s="9" t="n">
+        <v>1210.35</v>
+      </c>
+      <c r="R1053" s="6" t="n">
+        <v>234</v>
+      </c>
+      <c r="S1053" s="6" t="n">
+        <v>2972</v>
+      </c>
+      <c r="T1053" s="6" t="n">
+        <v>2948</v>
+      </c>
+      <c r="U1053" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1053" s="6" t="inlineStr"/>
+      <c r="W1053" s="6" t="inlineStr"/>
+      <c r="X1053" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 18-Sep-2026 09:01 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1053"/>
+  <dimension ref="A1:X1057"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -84182,6 +84182,326 @@
       <c r="W1053" s="6" t="inlineStr"/>
       <c r="X1053" s="6" t="inlineStr"/>
     </row>
+    <row r="1054">
+      <c r="A1054" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1054" s="2" t="inlineStr">
+        <is>
+          <t>BHEL</t>
+        </is>
+      </c>
+      <c r="C1054" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1054" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1054" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1054" s="2" t="n">
+        <v>432.5</v>
+      </c>
+      <c r="G1054" s="2" t="n">
+        <v>428.4</v>
+      </c>
+      <c r="H1054" s="2" t="n">
+        <v>435.5</v>
+      </c>
+      <c r="I1054" s="2" t="n">
+        <v>427.25</v>
+      </c>
+      <c r="J1054" s="2" t="n">
+        <v>425.8</v>
+      </c>
+      <c r="K1054" s="2" t="n">
+        <v>435.5</v>
+      </c>
+      <c r="L1054" s="2" t="n">
+        <v>427.25</v>
+      </c>
+      <c r="M1054" s="2" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="N1054" s="4" t="n">
+        <v>435.55</v>
+      </c>
+      <c r="O1054" s="5" t="n">
+        <v>431.33</v>
+      </c>
+      <c r="P1054" s="3" t="n">
+        <v>439.68</v>
+      </c>
+      <c r="Q1054" s="3" t="n">
+        <v>443.8</v>
+      </c>
+      <c r="R1054" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="S1054" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1054" s="2" t="n">
+        <v>2924</v>
+      </c>
+      <c r="U1054" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1054" s="2" t="inlineStr"/>
+      <c r="W1054" s="2" t="inlineStr"/>
+      <c r="X1054" s="2" t="inlineStr"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="2" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1055" s="2" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1055" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1055" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1055" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1055" s="2" t="n">
+        <v>1761.6</v>
+      </c>
+      <c r="G1055" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="H1055" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="I1055" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="J1055" s="2" t="n">
+        <v>1736.89</v>
+      </c>
+      <c r="K1055" s="2" t="n">
+        <v>1770</v>
+      </c>
+      <c r="L1055" s="2" t="n">
+        <v>1751.3</v>
+      </c>
+      <c r="M1055" s="2" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="N1055" s="4" t="n">
+        <v>1770.05</v>
+      </c>
+      <c r="O1055" s="5" t="n">
+        <v>1760.6</v>
+      </c>
+      <c r="P1055" s="3" t="n">
+        <v>1779.4</v>
+      </c>
+      <c r="Q1055" s="3" t="n">
+        <v>1788.75</v>
+      </c>
+      <c r="R1055" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="S1055" s="2" t="n">
+        <v>2665</v>
+      </c>
+      <c r="T1055" s="2" t="n">
+        <v>2637</v>
+      </c>
+      <c r="U1055" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1055" s="2" t="inlineStr"/>
+      <c r="W1055" s="2" t="inlineStr"/>
+      <c r="X1055" s="2" t="inlineStr"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1056" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1056" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1056" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1056" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1056" s="6" t="n">
+        <v>1045</v>
+      </c>
+      <c r="G1056" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="H1056" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="I1056" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="J1056" s="6" t="n">
+        <v>1099.96</v>
+      </c>
+      <c r="K1056" s="6" t="n">
+        <v>1061.9</v>
+      </c>
+      <c r="L1056" s="6" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="M1056" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N1056" s="8" t="n">
+        <v>1039.25</v>
+      </c>
+      <c r="O1056" s="7" t="n">
+        <v>1050.65</v>
+      </c>
+      <c r="P1056" s="9" t="n">
+        <v>1027.95</v>
+      </c>
+      <c r="Q1056" s="9" t="n">
+        <v>1016.65</v>
+      </c>
+      <c r="R1056" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1056" s="6" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T1056" s="6" t="n">
+        <v>2949</v>
+      </c>
+      <c r="U1056" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1056" s="6" t="inlineStr"/>
+      <c r="W1056" s="6" t="inlineStr"/>
+      <c r="X1056" s="6" t="inlineStr"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="6" t="inlineStr">
+        <is>
+          <t>18-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1057" s="6" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C1057" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1057" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1057" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1057" s="6" t="n">
+        <v>163.54</v>
+      </c>
+      <c r="G1057" s="6" t="n">
+        <v>166.9</v>
+      </c>
+      <c r="H1057" s="6" t="n">
+        <v>166.9</v>
+      </c>
+      <c r="I1057" s="6" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="J1057" s="6" t="n">
+        <v>174.37</v>
+      </c>
+      <c r="K1057" s="6" t="n">
+        <v>166.9</v>
+      </c>
+      <c r="L1057" s="6" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="M1057" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="N1057" s="8" t="n">
+        <v>163.25</v>
+      </c>
+      <c r="O1057" s="7" t="n">
+        <v>165.15</v>
+      </c>
+      <c r="P1057" s="9" t="n">
+        <v>161.45</v>
+      </c>
+      <c r="Q1057" s="9" t="n">
+        <v>159.65</v>
+      </c>
+      <c r="R1057" s="6" t="n">
+        <v>1578</v>
+      </c>
+      <c r="S1057" s="6" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1057" s="6" t="n">
+        <v>2840</v>
+      </c>
+      <c r="U1057" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1057" s="6" t="inlineStr"/>
+      <c r="W1057" s="6" t="inlineStr"/>
+      <c r="X1057" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 21-Sep-2026 09:02 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1057"/>
+  <dimension ref="A1:X1061"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -84502,6 +84502,326 @@
       <c r="W1057" s="6" t="inlineStr"/>
       <c r="X1057" s="6" t="inlineStr"/>
     </row>
+    <row r="1058">
+      <c r="A1058" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1058" s="2" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="C1058" s="2" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1058" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1058" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1058" s="2" t="n">
+        <v>267.05</v>
+      </c>
+      <c r="G1058" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="H1058" s="2" t="n">
+        <v>267.5</v>
+      </c>
+      <c r="I1058" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="J1058" s="2" t="n">
+        <v>264.31</v>
+      </c>
+      <c r="K1058" s="2" t="n">
+        <v>267.5</v>
+      </c>
+      <c r="L1058" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="M1058" s="2" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="N1058" s="4" t="n">
+        <v>267.55</v>
+      </c>
+      <c r="O1058" s="5" t="n">
+        <v>265.47</v>
+      </c>
+      <c r="P1058" s="3" t="n">
+        <v>269.53</v>
+      </c>
+      <c r="Q1058" s="3" t="n">
+        <v>271.5</v>
+      </c>
+      <c r="R1058" s="2" t="n">
+        <v>1440</v>
+      </c>
+      <c r="S1058" s="2" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1058" s="2" t="n">
+        <v>2851</v>
+      </c>
+      <c r="U1058" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1058" s="2" t="inlineStr"/>
+      <c r="W1058" s="2" t="inlineStr"/>
+      <c r="X1058" s="2" t="inlineStr"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1059" s="2" t="inlineStr">
+        <is>
+          <t>DABUR</t>
+        </is>
+      </c>
+      <c r="C1059" s="2" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1059" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1059" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1059" s="2" t="n">
+        <v>391.6</v>
+      </c>
+      <c r="G1059" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="H1059" s="2" t="n">
+        <v>392.8</v>
+      </c>
+      <c r="I1059" s="2" t="n">
+        <v>387.6</v>
+      </c>
+      <c r="J1059" s="2" t="n">
+        <v>383.66</v>
+      </c>
+      <c r="K1059" s="2" t="n">
+        <v>392.8</v>
+      </c>
+      <c r="L1059" s="2" t="n">
+        <v>387.6</v>
+      </c>
+      <c r="M1059" s="2" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="N1059" s="4" t="n">
+        <v>392.85</v>
+      </c>
+      <c r="O1059" s="5" t="n">
+        <v>390.15</v>
+      </c>
+      <c r="P1059" s="3" t="n">
+        <v>395.45</v>
+      </c>
+      <c r="Q1059" s="3" t="n">
+        <v>398.05</v>
+      </c>
+      <c r="R1059" s="2" t="n">
+        <v>1110</v>
+      </c>
+      <c r="S1059" s="2" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T1059" s="2" t="n">
+        <v>2886</v>
+      </c>
+      <c r="U1059" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1059" s="2" t="inlineStr"/>
+      <c r="W1059" s="2" t="inlineStr"/>
+      <c r="X1059" s="2" t="inlineStr"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1060" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1060" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1060" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1060" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1060" s="6" t="n">
+        <v>1774.2</v>
+      </c>
+      <c r="G1060" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="H1060" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="I1060" s="6" t="n">
+        <v>1763.5</v>
+      </c>
+      <c r="J1060" s="6" t="n">
+        <v>1825.01</v>
+      </c>
+      <c r="K1060" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="L1060" s="6" t="n">
+        <v>1763.5</v>
+      </c>
+      <c r="M1060" s="6" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="N1060" s="8" t="n">
+        <v>1763.45</v>
+      </c>
+      <c r="O1060" s="7" t="n">
+        <v>1784.8</v>
+      </c>
+      <c r="P1060" s="9" t="n">
+        <v>1742.2</v>
+      </c>
+      <c r="Q1060" s="9" t="n">
+        <v>1720.95</v>
+      </c>
+      <c r="R1060" s="6" t="n">
+        <v>138</v>
+      </c>
+      <c r="S1060" s="6" t="n">
+        <v>2946</v>
+      </c>
+      <c r="T1060" s="6" t="n">
+        <v>2932</v>
+      </c>
+      <c r="U1060" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1060" s="6" t="inlineStr"/>
+      <c r="W1060" s="6" t="inlineStr"/>
+      <c r="X1060" s="6" t="inlineStr"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1061" s="6" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="C1061" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1061" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1061" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1061" s="6" t="n">
+        <v>184</v>
+      </c>
+      <c r="G1061" s="6" t="n">
+        <v>184.55</v>
+      </c>
+      <c r="H1061" s="6" t="n">
+        <v>186.87</v>
+      </c>
+      <c r="I1061" s="6" t="n">
+        <v>183.8</v>
+      </c>
+      <c r="J1061" s="6" t="n">
+        <v>185.63</v>
+      </c>
+      <c r="K1061" s="6" t="n">
+        <v>186.87</v>
+      </c>
+      <c r="L1061" s="6" t="n">
+        <v>183.8</v>
+      </c>
+      <c r="M1061" s="6" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="N1061" s="8" t="n">
+        <v>183.75</v>
+      </c>
+      <c r="O1061" s="7" t="n">
+        <v>185.39</v>
+      </c>
+      <c r="P1061" s="9" t="n">
+        <v>182.22</v>
+      </c>
+      <c r="Q1061" s="9" t="n">
+        <v>180.68</v>
+      </c>
+      <c r="R1061" s="6" t="n">
+        <v>1827</v>
+      </c>
+      <c r="S1061" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1061" s="6" t="n">
+        <v>2795</v>
+      </c>
+      <c r="U1061" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1061" s="6" t="inlineStr"/>
+      <c r="W1061" s="6" t="inlineStr"/>
+      <c r="X1061" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 21-Sep-2026 09:13 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1061"/>
+  <dimension ref="A1:X1065"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -84822,6 +84822,326 @@
       <c r="W1061" s="6" t="inlineStr"/>
       <c r="X1061" s="6" t="inlineStr"/>
     </row>
+    <row r="1062">
+      <c r="A1062" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1062" s="2" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1062" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1062" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1062" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1062" s="2" t="n">
+        <v>1039.5</v>
+      </c>
+      <c r="G1062" s="2" t="n">
+        <v>1041.5</v>
+      </c>
+      <c r="H1062" s="2" t="n">
+        <v>1044.5</v>
+      </c>
+      <c r="I1062" s="2" t="n">
+        <v>1030.3</v>
+      </c>
+      <c r="J1062" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1062" s="2" t="n">
+        <v>1044.5</v>
+      </c>
+      <c r="L1062" s="2" t="n">
+        <v>1030.3</v>
+      </c>
+      <c r="M1062" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="N1062" s="4" t="n">
+        <v>1044.55</v>
+      </c>
+      <c r="O1062" s="5" t="n">
+        <v>1037.35</v>
+      </c>
+      <c r="P1062" s="3" t="n">
+        <v>1051.65</v>
+      </c>
+      <c r="Q1062" s="3" t="n">
+        <v>1058.75</v>
+      </c>
+      <c r="R1062" s="2" t="n">
+        <v>414</v>
+      </c>
+      <c r="S1062" s="2" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1062" s="2" t="n">
+        <v>2939</v>
+      </c>
+      <c r="U1062" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1062" s="2" t="inlineStr"/>
+      <c r="W1062" s="2" t="inlineStr"/>
+      <c r="X1062" s="2" t="inlineStr"/>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1063" s="2" t="inlineStr">
+        <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="C1063" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1063" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1063" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1063" s="2" t="n">
+        <v>4310.1</v>
+      </c>
+      <c r="G1063" s="2" t="n">
+        <v>4240</v>
+      </c>
+      <c r="H1063" s="2" t="n">
+        <v>4313</v>
+      </c>
+      <c r="I1063" s="2" t="n">
+        <v>4190.5</v>
+      </c>
+      <c r="J1063" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1063" s="2" t="n">
+        <v>4313</v>
+      </c>
+      <c r="L1063" s="2" t="n">
+        <v>4190.5</v>
+      </c>
+      <c r="M1063" s="2" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="N1063" s="4" t="n">
+        <v>4313.05</v>
+      </c>
+      <c r="O1063" s="5" t="n">
+        <v>4251.7</v>
+      </c>
+      <c r="P1063" s="3" t="n">
+        <v>4374.3</v>
+      </c>
+      <c r="Q1063" s="3" t="n">
+        <v>4435.55</v>
+      </c>
+      <c r="R1063" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="S1063" s="2" t="n">
+        <v>2945</v>
+      </c>
+      <c r="T1063" s="2" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1063" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1063" s="2" t="inlineStr"/>
+      <c r="W1063" s="2" t="inlineStr"/>
+      <c r="X1063" s="2" t="inlineStr"/>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1064" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1064" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1064" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1064" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1064" s="6" t="n">
+        <v>1025.5</v>
+      </c>
+      <c r="G1064" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="H1064" s="6" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="I1064" s="6" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J1064" s="6" t="n">
+        <v>1050</v>
+      </c>
+      <c r="K1064" s="6" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="L1064" s="6" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="M1064" s="6" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="N1064" s="8" t="n">
+        <v>1022.05</v>
+      </c>
+      <c r="O1064" s="7" t="n">
+        <v>1029.95</v>
+      </c>
+      <c r="P1064" s="9" t="n">
+        <v>1014.25</v>
+      </c>
+      <c r="Q1064" s="9" t="n">
+        <v>1006.45</v>
+      </c>
+      <c r="R1064" s="6" t="n">
+        <v>378</v>
+      </c>
+      <c r="S1064" s="6" t="n">
+        <v>2986</v>
+      </c>
+      <c r="T1064" s="6" t="n">
+        <v>2948</v>
+      </c>
+      <c r="U1064" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1064" s="6" t="inlineStr"/>
+      <c r="W1064" s="6" t="inlineStr"/>
+      <c r="X1064" s="6" t="inlineStr"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1065" s="6" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="C1065" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1065" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1065" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1065" s="6" t="n">
+        <v>184.05</v>
+      </c>
+      <c r="G1065" s="6" t="n">
+        <v>184.55</v>
+      </c>
+      <c r="H1065" s="6" t="n">
+        <v>186.87</v>
+      </c>
+      <c r="I1065" s="6" t="n">
+        <v>183.8</v>
+      </c>
+      <c r="J1065" s="6" t="n">
+        <v>185.63</v>
+      </c>
+      <c r="K1065" s="6" t="n">
+        <v>186.87</v>
+      </c>
+      <c r="L1065" s="6" t="n">
+        <v>183.8</v>
+      </c>
+      <c r="M1065" s="6" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="N1065" s="8" t="n">
+        <v>183.75</v>
+      </c>
+      <c r="O1065" s="7" t="n">
+        <v>185.39</v>
+      </c>
+      <c r="P1065" s="9" t="n">
+        <v>182.22</v>
+      </c>
+      <c r="Q1065" s="9" t="n">
+        <v>180.68</v>
+      </c>
+      <c r="R1065" s="6" t="n">
+        <v>1827</v>
+      </c>
+      <c r="S1065" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1065" s="6" t="n">
+        <v>2795</v>
+      </c>
+      <c r="U1065" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1065" s="6" t="inlineStr"/>
+      <c r="W1065" s="6" t="inlineStr"/>
+      <c r="X1065" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 21-Sep-2026 09:48 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1065"/>
+  <dimension ref="A1:X1069"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -85142,6 +85142,326 @@
       <c r="W1065" s="6" t="inlineStr"/>
       <c r="X1065" s="6" t="inlineStr"/>
     </row>
+    <row r="1066">
+      <c r="A1066" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1066" s="2" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="C1066" s="2" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1066" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1066" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1066" s="2" t="n">
+        <v>267.45</v>
+      </c>
+      <c r="G1066" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="H1066" s="2" t="n">
+        <v>267.95</v>
+      </c>
+      <c r="I1066" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="J1066" s="2" t="n">
+        <v>264.33</v>
+      </c>
+      <c r="K1066" s="2" t="n">
+        <v>267.95</v>
+      </c>
+      <c r="L1066" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="M1066" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N1066" s="4" t="n">
+        <v>268</v>
+      </c>
+      <c r="O1066" s="5" t="n">
+        <v>265.7</v>
+      </c>
+      <c r="P1066" s="3" t="n">
+        <v>270.2</v>
+      </c>
+      <c r="Q1066" s="3" t="n">
+        <v>272.4</v>
+      </c>
+      <c r="R1066" s="2" t="n">
+        <v>1302</v>
+      </c>
+      <c r="S1066" s="2" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1066" s="2" t="n">
+        <v>2864</v>
+      </c>
+      <c r="U1066" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1066" s="2" t="inlineStr"/>
+      <c r="W1066" s="2" t="inlineStr"/>
+      <c r="X1066" s="2" t="inlineStr"/>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1067" s="2" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1067" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1067" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1067" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1067" s="2" t="n">
+        <v>1040.5</v>
+      </c>
+      <c r="G1067" s="2" t="n">
+        <v>1041.5</v>
+      </c>
+      <c r="H1067" s="2" t="n">
+        <v>1044.5</v>
+      </c>
+      <c r="I1067" s="2" t="n">
+        <v>1030.3</v>
+      </c>
+      <c r="J1067" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1067" s="2" t="n">
+        <v>1044.5</v>
+      </c>
+      <c r="L1067" s="2" t="n">
+        <v>1030.3</v>
+      </c>
+      <c r="M1067" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="N1067" s="4" t="n">
+        <v>1044.55</v>
+      </c>
+      <c r="O1067" s="5" t="n">
+        <v>1037.35</v>
+      </c>
+      <c r="P1067" s="3" t="n">
+        <v>1051.65</v>
+      </c>
+      <c r="Q1067" s="3" t="n">
+        <v>1058.75</v>
+      </c>
+      <c r="R1067" s="2" t="n">
+        <v>414</v>
+      </c>
+      <c r="S1067" s="2" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1067" s="2" t="n">
+        <v>2939</v>
+      </c>
+      <c r="U1067" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1067" s="2" t="inlineStr"/>
+      <c r="W1067" s="2" t="inlineStr"/>
+      <c r="X1067" s="2" t="inlineStr"/>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1068" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="C1068" s="6" t="inlineStr">
+        <is>
+          <t>TELECOM</t>
+        </is>
+      </c>
+      <c r="D1068" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1068" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1068" s="6" t="n">
+        <v>1831.4</v>
+      </c>
+      <c r="G1068" s="6" t="n">
+        <v>1854.8</v>
+      </c>
+      <c r="H1068" s="6" t="n">
+        <v>1854.8</v>
+      </c>
+      <c r="I1068" s="6" t="n">
+        <v>1822</v>
+      </c>
+      <c r="J1068" s="6" t="n">
+        <v>1859.51</v>
+      </c>
+      <c r="K1068" s="6" t="n">
+        <v>1854.8</v>
+      </c>
+      <c r="L1068" s="6" t="n">
+        <v>1822</v>
+      </c>
+      <c r="M1068" s="6" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="N1068" s="8" t="n">
+        <v>1821.95</v>
+      </c>
+      <c r="O1068" s="7" t="n">
+        <v>1838.45</v>
+      </c>
+      <c r="P1068" s="9" t="n">
+        <v>1805.55</v>
+      </c>
+      <c r="Q1068" s="9" t="n">
+        <v>1789.15</v>
+      </c>
+      <c r="R1068" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="S1068" s="6" t="n">
+        <v>2970</v>
+      </c>
+      <c r="T1068" s="6" t="n">
+        <v>2952</v>
+      </c>
+      <c r="U1068" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1068" s="6" t="inlineStr"/>
+      <c r="W1068" s="6" t="inlineStr"/>
+      <c r="X1068" s="6" t="inlineStr"/>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1069" s="6" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="C1069" s="6" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1069" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1069" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1069" s="6" t="n">
+        <v>1270.4</v>
+      </c>
+      <c r="G1069" s="6" t="n">
+        <v>1281.3</v>
+      </c>
+      <c r="H1069" s="6" t="n">
+        <v>1287</v>
+      </c>
+      <c r="I1069" s="6" t="n">
+        <v>1268.9</v>
+      </c>
+      <c r="J1069" s="6" t="n">
+        <v>1301.39</v>
+      </c>
+      <c r="K1069" s="6" t="n">
+        <v>1287</v>
+      </c>
+      <c r="L1069" s="6" t="n">
+        <v>1268.9</v>
+      </c>
+      <c r="M1069" s="6" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="N1069" s="8" t="n">
+        <v>1268.85</v>
+      </c>
+      <c r="O1069" s="7" t="n">
+        <v>1278</v>
+      </c>
+      <c r="P1069" s="9" t="n">
+        <v>1259.8</v>
+      </c>
+      <c r="Q1069" s="9" t="n">
+        <v>1250.75</v>
+      </c>
+      <c r="R1069" s="6" t="n">
+        <v>327</v>
+      </c>
+      <c r="S1069" s="6" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T1069" s="6" t="n">
+        <v>2959</v>
+      </c>
+      <c r="U1069" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1069" s="6" t="inlineStr"/>
+      <c r="W1069" s="6" t="inlineStr"/>
+      <c r="X1069" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 21-Sep-2026 09:56 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1069"/>
+  <dimension ref="A1:X1073"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -85462,6 +85462,326 @@
       <c r="W1069" s="6" t="inlineStr"/>
       <c r="X1069" s="6" t="inlineStr"/>
     </row>
+    <row r="1070">
+      <c r="A1070" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1070" s="2" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="C1070" s="2" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1070" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1070" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1070" s="2" t="n">
+        <v>267.45</v>
+      </c>
+      <c r="G1070" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="H1070" s="2" t="n">
+        <v>267.95</v>
+      </c>
+      <c r="I1070" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="J1070" s="2" t="n">
+        <v>264.33</v>
+      </c>
+      <c r="K1070" s="2" t="n">
+        <v>267.95</v>
+      </c>
+      <c r="L1070" s="2" t="n">
+        <v>263.55</v>
+      </c>
+      <c r="M1070" s="2" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N1070" s="4" t="n">
+        <v>268</v>
+      </c>
+      <c r="O1070" s="5" t="n">
+        <v>265.7</v>
+      </c>
+      <c r="P1070" s="3" t="n">
+        <v>270.2</v>
+      </c>
+      <c r="Q1070" s="3" t="n">
+        <v>272.4</v>
+      </c>
+      <c r="R1070" s="2" t="n">
+        <v>1302</v>
+      </c>
+      <c r="S1070" s="2" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1070" s="2" t="n">
+        <v>2864</v>
+      </c>
+      <c r="U1070" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1070" s="2" t="inlineStr"/>
+      <c r="W1070" s="2" t="inlineStr"/>
+      <c r="X1070" s="2" t="inlineStr"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="2" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1071" s="2" t="inlineStr">
+        <is>
+          <t>MPHASIS</t>
+        </is>
+      </c>
+      <c r="C1071" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1071" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1071" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1071" s="2" t="n">
+        <v>2307</v>
+      </c>
+      <c r="G1071" s="2" t="n">
+        <v>2300.4</v>
+      </c>
+      <c r="H1071" s="2" t="n">
+        <v>2313.7</v>
+      </c>
+      <c r="I1071" s="2" t="n">
+        <v>2257.1</v>
+      </c>
+      <c r="J1071" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1071" s="2" t="n">
+        <v>2313.7</v>
+      </c>
+      <c r="L1071" s="2" t="n">
+        <v>2257.1</v>
+      </c>
+      <c r="M1071" s="2" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="N1071" s="4" t="n">
+        <v>2313.75</v>
+      </c>
+      <c r="O1071" s="5" t="n">
+        <v>2285.35</v>
+      </c>
+      <c r="P1071" s="3" t="n">
+        <v>2342.05</v>
+      </c>
+      <c r="Q1071" s="3" t="n">
+        <v>2370.35</v>
+      </c>
+      <c r="R1071" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="S1071" s="2" t="n">
+        <v>2982</v>
+      </c>
+      <c r="T1071" s="2" t="n">
+        <v>2972</v>
+      </c>
+      <c r="U1071" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1071" s="2" t="inlineStr"/>
+      <c r="W1071" s="2" t="inlineStr"/>
+      <c r="X1071" s="2" t="inlineStr"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1072" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1072" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1072" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1072" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1072" s="6" t="n">
+        <v>1024.7</v>
+      </c>
+      <c r="G1072" s="6" t="n">
+        <v>1035</v>
+      </c>
+      <c r="H1072" s="6" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="I1072" s="6" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="J1072" s="6" t="n">
+        <v>1049.8</v>
+      </c>
+      <c r="K1072" s="6" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="L1072" s="6" t="n">
+        <v>1022.1</v>
+      </c>
+      <c r="M1072" s="6" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="N1072" s="8" t="n">
+        <v>1022.05</v>
+      </c>
+      <c r="O1072" s="7" t="n">
+        <v>1029.95</v>
+      </c>
+      <c r="P1072" s="9" t="n">
+        <v>1014.25</v>
+      </c>
+      <c r="Q1072" s="9" t="n">
+        <v>1006.45</v>
+      </c>
+      <c r="R1072" s="6" t="n">
+        <v>378</v>
+      </c>
+      <c r="S1072" s="6" t="n">
+        <v>2986</v>
+      </c>
+      <c r="T1072" s="6" t="n">
+        <v>2948</v>
+      </c>
+      <c r="U1072" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1072" s="6" t="inlineStr"/>
+      <c r="W1072" s="6" t="inlineStr"/>
+      <c r="X1072" s="6" t="inlineStr"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="6" t="inlineStr">
+        <is>
+          <t>21-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1073" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1073" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1073" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1073" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1073" s="6" t="n">
+        <v>1768.5</v>
+      </c>
+      <c r="G1073" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="H1073" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="I1073" s="6" t="n">
+        <v>1763.5</v>
+      </c>
+      <c r="J1073" s="6" t="n">
+        <v>1824.56</v>
+      </c>
+      <c r="K1073" s="6" t="n">
+        <v>1806</v>
+      </c>
+      <c r="L1073" s="6" t="n">
+        <v>1763.5</v>
+      </c>
+      <c r="M1073" s="6" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="N1073" s="8" t="n">
+        <v>1763.45</v>
+      </c>
+      <c r="O1073" s="7" t="n">
+        <v>1784.8</v>
+      </c>
+      <c r="P1073" s="9" t="n">
+        <v>1742.2</v>
+      </c>
+      <c r="Q1073" s="9" t="n">
+        <v>1720.95</v>
+      </c>
+      <c r="R1073" s="6" t="n">
+        <v>138</v>
+      </c>
+      <c r="S1073" s="6" t="n">
+        <v>2946</v>
+      </c>
+      <c r="T1073" s="6" t="n">
+        <v>2932</v>
+      </c>
+      <c r="U1073" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1073" s="6" t="inlineStr"/>
+      <c r="W1073" s="6" t="inlineStr"/>
+      <c r="X1073" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 22-Sep-2026 08:37 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1073"/>
+  <dimension ref="A1:X1077"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -85782,6 +85782,326 @@
       <c r="W1073" s="6" t="inlineStr"/>
       <c r="X1073" s="6" t="inlineStr"/>
     </row>
+    <row r="1074">
+      <c r="A1074" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1074" s="2" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1074" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1074" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1074" s="2" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1074" s="2" t="n">
+        <v>426.35</v>
+      </c>
+      <c r="G1074" s="2" t="n">
+        <v>424.7</v>
+      </c>
+      <c r="H1074" s="2" t="n">
+        <v>428.75</v>
+      </c>
+      <c r="I1074" s="2" t="n">
+        <v>419.65</v>
+      </c>
+      <c r="J1074" s="2" t="n">
+        <v>415.07</v>
+      </c>
+      <c r="K1074" s="2" t="n">
+        <v>428.75</v>
+      </c>
+      <c r="L1074" s="2" t="n">
+        <v>419.65</v>
+      </c>
+      <c r="M1074" s="2" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="N1074" s="4" t="n">
+        <v>428.8</v>
+      </c>
+      <c r="O1074" s="5" t="n">
+        <v>424.15</v>
+      </c>
+      <c r="P1074" s="3" t="n">
+        <v>433.35</v>
+      </c>
+      <c r="Q1074" s="3" t="n">
+        <v>437.9</v>
+      </c>
+      <c r="R1074" s="2" t="n">
+        <v>645</v>
+      </c>
+      <c r="S1074" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1074" s="2" t="n">
+        <v>2935</v>
+      </c>
+      <c r="U1074" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1074" s="2" t="inlineStr"/>
+      <c r="W1074" s="2" t="inlineStr"/>
+      <c r="X1074" s="2" t="inlineStr"/>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1075" s="2" t="inlineStr">
+        <is>
+          <t>ZOMATO</t>
+        </is>
+      </c>
+      <c r="C1075" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1075" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1075" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1075" s="2" t="n">
+        <v>338.85</v>
+      </c>
+      <c r="G1075" s="2" t="n">
+        <v>337.7</v>
+      </c>
+      <c r="H1075" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="I1075" s="2" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="J1075" s="2" t="n">
+        <v>325.74</v>
+      </c>
+      <c r="K1075" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="L1075" s="2" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="M1075" s="2" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="N1075" s="4" t="n">
+        <v>340.05</v>
+      </c>
+      <c r="O1075" s="5" t="n">
+        <v>337.27</v>
+      </c>
+      <c r="P1075" s="3" t="n">
+        <v>342.73</v>
+      </c>
+      <c r="Q1075" s="3" t="n">
+        <v>345.4</v>
+      </c>
+      <c r="R1075" s="2" t="n">
+        <v>1077</v>
+      </c>
+      <c r="S1075" s="2" t="n">
+        <v>2994</v>
+      </c>
+      <c r="T1075" s="2" t="n">
+        <v>2886</v>
+      </c>
+      <c r="U1075" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1075" s="2" t="inlineStr"/>
+      <c r="W1075" s="2" t="inlineStr"/>
+      <c r="X1075" s="2" t="inlineStr"/>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1076" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1076" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1076" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1076" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1076" s="6" t="n">
+        <v>1024.2</v>
+      </c>
+      <c r="G1076" s="6" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="H1076" s="6" t="n">
+        <v>1041</v>
+      </c>
+      <c r="I1076" s="6" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="J1076" s="6" t="n">
+        <v>1088.57</v>
+      </c>
+      <c r="K1076" s="6" t="n">
+        <v>1041</v>
+      </c>
+      <c r="L1076" s="6" t="n">
+        <v>1019.2</v>
+      </c>
+      <c r="M1076" s="6" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="N1076" s="8" t="n">
+        <v>1019.15</v>
+      </c>
+      <c r="O1076" s="7" t="n">
+        <v>1030.15</v>
+      </c>
+      <c r="P1076" s="9" t="n">
+        <v>1008.25</v>
+      </c>
+      <c r="Q1076" s="9" t="n">
+        <v>997.35</v>
+      </c>
+      <c r="R1076" s="6" t="n">
+        <v>270</v>
+      </c>
+      <c r="S1076" s="6" t="n">
+        <v>2970</v>
+      </c>
+      <c r="T1076" s="6" t="n">
+        <v>2943</v>
+      </c>
+      <c r="U1076" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1076" s="6" t="inlineStr"/>
+      <c r="W1076" s="6" t="inlineStr"/>
+      <c r="X1076" s="6" t="inlineStr"/>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1077" s="6" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="C1077" s="6" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1077" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1077" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1077" s="6" t="n">
+        <v>1935.9</v>
+      </c>
+      <c r="G1077" s="6" t="n">
+        <v>1952</v>
+      </c>
+      <c r="H1077" s="6" t="n">
+        <v>1956.8</v>
+      </c>
+      <c r="I1077" s="6" t="n">
+        <v>1934.2</v>
+      </c>
+      <c r="J1077" s="6" t="n">
+        <v>1968.38</v>
+      </c>
+      <c r="K1077" s="6" t="n">
+        <v>1956.8</v>
+      </c>
+      <c r="L1077" s="6" t="n">
+        <v>1934.2</v>
+      </c>
+      <c r="M1077" s="6" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N1077" s="8" t="n">
+        <v>1934.15</v>
+      </c>
+      <c r="O1077" s="7" t="n">
+        <v>1945.55</v>
+      </c>
+      <c r="P1077" s="9" t="n">
+        <v>1922.85</v>
+      </c>
+      <c r="Q1077" s="9" t="n">
+        <v>1911.55</v>
+      </c>
+      <c r="R1077" s="6" t="n">
+        <v>258</v>
+      </c>
+      <c r="S1077" s="6" t="n">
+        <v>2941</v>
+      </c>
+      <c r="T1077" s="6" t="n">
+        <v>2915</v>
+      </c>
+      <c r="U1077" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1077" s="6" t="inlineStr"/>
+      <c r="W1077" s="6" t="inlineStr"/>
+      <c r="X1077" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 22-Sep-2026 08:44 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1077"/>
+  <dimension ref="A1:X1081"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -86102,6 +86102,326 @@
       <c r="W1077" s="6" t="inlineStr"/>
       <c r="X1077" s="6" t="inlineStr"/>
     </row>
+    <row r="1078">
+      <c r="A1078" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1078" s="2" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1078" s="2" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1078" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1078" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1078" s="2" t="n">
+        <v>235.66</v>
+      </c>
+      <c r="G1078" s="2" t="n">
+        <v>235.51</v>
+      </c>
+      <c r="H1078" s="2" t="n">
+        <v>236.37</v>
+      </c>
+      <c r="I1078" s="2" t="n">
+        <v>233.75</v>
+      </c>
+      <c r="J1078" s="2" t="n">
+        <v>234.89</v>
+      </c>
+      <c r="K1078" s="2" t="n">
+        <v>236.37</v>
+      </c>
+      <c r="L1078" s="2" t="n">
+        <v>233.75</v>
+      </c>
+      <c r="M1078" s="2" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="N1078" s="4" t="n">
+        <v>236.42</v>
+      </c>
+      <c r="O1078" s="5" t="n">
+        <v>235.01</v>
+      </c>
+      <c r="P1078" s="3" t="n">
+        <v>237.73</v>
+      </c>
+      <c r="Q1078" s="3" t="n">
+        <v>239.04</v>
+      </c>
+      <c r="R1078" s="2" t="n">
+        <v>2114</v>
+      </c>
+      <c r="S1078" s="2" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1078" s="2" t="n">
+        <v>2769</v>
+      </c>
+      <c r="U1078" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1078" s="2" t="inlineStr"/>
+      <c r="W1078" s="2" t="inlineStr"/>
+      <c r="X1078" s="2" t="inlineStr"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1079" s="2" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="C1079" s="2" t="inlineStr">
+        <is>
+          <t>REALTY</t>
+        </is>
+      </c>
+      <c r="D1079" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1079" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1079" s="2" t="n">
+        <v>666.4</v>
+      </c>
+      <c r="G1079" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="H1079" s="2" t="n">
+        <v>667.65</v>
+      </c>
+      <c r="I1079" s="2" t="n">
+        <v>659.05</v>
+      </c>
+      <c r="J1079" s="2" t="n">
+        <v>660.9400000000001</v>
+      </c>
+      <c r="K1079" s="2" t="n">
+        <v>667.65</v>
+      </c>
+      <c r="L1079" s="2" t="n">
+        <v>659.05</v>
+      </c>
+      <c r="M1079" s="2" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="N1079" s="4" t="n">
+        <v>667.7</v>
+      </c>
+      <c r="O1079" s="5" t="n">
+        <v>663.3</v>
+      </c>
+      <c r="P1079" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="Q1079" s="3" t="n">
+        <v>676.3</v>
+      </c>
+      <c r="R1079" s="2" t="n">
+        <v>681</v>
+      </c>
+      <c r="S1079" s="2" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1079" s="2" t="n">
+        <v>2928</v>
+      </c>
+      <c r="U1079" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1079" s="2" t="inlineStr"/>
+      <c r="W1079" s="2" t="inlineStr"/>
+      <c r="X1079" s="2" t="inlineStr"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1080" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1080" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1080" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1080" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1080" s="6" t="n">
+        <v>1011.6</v>
+      </c>
+      <c r="G1080" s="6" t="n">
+        <v>1025.3</v>
+      </c>
+      <c r="H1080" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="I1080" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="J1080" s="6" t="n">
+        <v>1047.24</v>
+      </c>
+      <c r="K1080" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="L1080" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="M1080" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="N1080" s="8" t="n">
+        <v>1004.95</v>
+      </c>
+      <c r="O1080" s="7" t="n">
+        <v>1017.15</v>
+      </c>
+      <c r="P1080" s="9" t="n">
+        <v>992.85</v>
+      </c>
+      <c r="Q1080" s="9" t="n">
+        <v>980.75</v>
+      </c>
+      <c r="R1080" s="6" t="n">
+        <v>243</v>
+      </c>
+      <c r="S1080" s="6" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1080" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1080" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1080" s="6" t="inlineStr"/>
+      <c r="W1080" s="6" t="inlineStr"/>
+      <c r="X1080" s="6" t="inlineStr"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1081" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1081" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1081" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1081" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1081" s="6" t="n">
+        <v>1827</v>
+      </c>
+      <c r="G1081" s="6" t="n">
+        <v>1862.7</v>
+      </c>
+      <c r="H1081" s="6" t="n">
+        <v>1863</v>
+      </c>
+      <c r="I1081" s="6" t="n">
+        <v>1823.8</v>
+      </c>
+      <c r="J1081" s="6" t="n">
+        <v>1940.83</v>
+      </c>
+      <c r="K1081" s="6" t="n">
+        <v>1863</v>
+      </c>
+      <c r="L1081" s="6" t="n">
+        <v>1823.8</v>
+      </c>
+      <c r="M1081" s="6" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="N1081" s="8" t="n">
+        <v>1823.75</v>
+      </c>
+      <c r="O1081" s="7" t="n">
+        <v>1843.45</v>
+      </c>
+      <c r="P1081" s="9" t="n">
+        <v>1804.15</v>
+      </c>
+      <c r="Q1081" s="9" t="n">
+        <v>1784.55</v>
+      </c>
+      <c r="R1081" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="S1081" s="6" t="n">
+        <v>2955</v>
+      </c>
+      <c r="T1081" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1081" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1081" s="6" t="inlineStr"/>
+      <c r="W1081" s="6" t="inlineStr"/>
+      <c r="X1081" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 22-Sep-2026 09:12 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1081"/>
+  <dimension ref="A1:X1085"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -86422,6 +86422,326 @@
       <c r="W1081" s="6" t="inlineStr"/>
       <c r="X1081" s="6" t="inlineStr"/>
     </row>
+    <row r="1082">
+      <c r="A1082" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1082" s="2" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="C1082" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1082" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1082" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1082" s="2" t="n">
+        <v>1272</v>
+      </c>
+      <c r="G1082" s="2" t="n">
+        <v>1274.7</v>
+      </c>
+      <c r="H1082" s="2" t="n">
+        <v>1277.5</v>
+      </c>
+      <c r="I1082" s="2" t="n">
+        <v>1264.6</v>
+      </c>
+      <c r="J1082" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1082" s="2" t="n">
+        <v>1277.5</v>
+      </c>
+      <c r="L1082" s="2" t="n">
+        <v>1264.6</v>
+      </c>
+      <c r="M1082" s="2" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="N1082" s="4" t="n">
+        <v>1277.55</v>
+      </c>
+      <c r="O1082" s="5" t="n">
+        <v>1271</v>
+      </c>
+      <c r="P1082" s="3" t="n">
+        <v>1284</v>
+      </c>
+      <c r="Q1082" s="3" t="n">
+        <v>1290.45</v>
+      </c>
+      <c r="R1082" s="2" t="n">
+        <v>391</v>
+      </c>
+      <c r="S1082" s="2" t="n">
+        <v>2561</v>
+      </c>
+      <c r="T1082" s="2" t="n">
+        <v>2522</v>
+      </c>
+      <c r="U1082" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1082" s="2" t="inlineStr"/>
+      <c r="W1082" s="2" t="inlineStr"/>
+      <c r="X1082" s="2" t="inlineStr"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1083" s="2" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="C1083" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1083" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1083" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1083" s="2" t="n">
+        <v>972.8</v>
+      </c>
+      <c r="G1083" s="2" t="n">
+        <v>987</v>
+      </c>
+      <c r="H1083" s="2" t="n">
+        <v>987.5</v>
+      </c>
+      <c r="I1083" s="2" t="n">
+        <v>967.1</v>
+      </c>
+      <c r="J1083" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1083" s="2" t="n">
+        <v>987.5</v>
+      </c>
+      <c r="L1083" s="2" t="n">
+        <v>967.1</v>
+      </c>
+      <c r="M1083" s="2" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="N1083" s="4" t="n">
+        <v>987.55</v>
+      </c>
+      <c r="O1083" s="5" t="n">
+        <v>977.25</v>
+      </c>
+      <c r="P1083" s="3" t="n">
+        <v>997.75</v>
+      </c>
+      <c r="Q1083" s="3" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="R1083" s="2" t="n">
+        <v>291</v>
+      </c>
+      <c r="S1083" s="2" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T1083" s="2" t="n">
+        <v>2968</v>
+      </c>
+      <c r="U1083" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1083" s="2" t="inlineStr"/>
+      <c r="W1083" s="2" t="inlineStr"/>
+      <c r="X1083" s="2" t="inlineStr"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1084" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1084" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1084" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1084" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1084" s="6" t="n">
+        <v>1012.1</v>
+      </c>
+      <c r="G1084" s="6" t="n">
+        <v>1025.3</v>
+      </c>
+      <c r="H1084" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="I1084" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="J1084" s="6" t="n">
+        <v>1047.06</v>
+      </c>
+      <c r="K1084" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="L1084" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="M1084" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="N1084" s="8" t="n">
+        <v>1004.95</v>
+      </c>
+      <c r="O1084" s="7" t="n">
+        <v>1017.15</v>
+      </c>
+      <c r="P1084" s="9" t="n">
+        <v>992.85</v>
+      </c>
+      <c r="Q1084" s="9" t="n">
+        <v>980.75</v>
+      </c>
+      <c r="R1084" s="6" t="n">
+        <v>243</v>
+      </c>
+      <c r="S1084" s="6" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1084" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1084" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1084" s="6" t="inlineStr"/>
+      <c r="W1084" s="6" t="inlineStr"/>
+      <c r="X1084" s="6" t="inlineStr"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1085" s="6" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="C1085" s="6" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="D1085" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1085" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1085" s="6" t="n">
+        <v>1938.3</v>
+      </c>
+      <c r="G1085" s="6" t="n">
+        <v>1952</v>
+      </c>
+      <c r="H1085" s="6" t="n">
+        <v>1956.8</v>
+      </c>
+      <c r="I1085" s="6" t="n">
+        <v>1934</v>
+      </c>
+      <c r="J1085" s="6" t="n">
+        <v>1968.37</v>
+      </c>
+      <c r="K1085" s="6" t="n">
+        <v>1956.8</v>
+      </c>
+      <c r="L1085" s="6" t="n">
+        <v>1934</v>
+      </c>
+      <c r="M1085" s="6" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="N1085" s="8" t="n">
+        <v>1933.95</v>
+      </c>
+      <c r="O1085" s="7" t="n">
+        <v>1945.45</v>
+      </c>
+      <c r="P1085" s="9" t="n">
+        <v>1922.55</v>
+      </c>
+      <c r="Q1085" s="9" t="n">
+        <v>1911.15</v>
+      </c>
+      <c r="R1085" s="6" t="n">
+        <v>258</v>
+      </c>
+      <c r="S1085" s="6" t="n">
+        <v>2967</v>
+      </c>
+      <c r="T1085" s="6" t="n">
+        <v>2941</v>
+      </c>
+      <c r="U1085" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1085" s="6" t="inlineStr"/>
+      <c r="W1085" s="6" t="inlineStr"/>
+      <c r="X1085" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 22-Sep-2026 09:21 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1085"/>
+  <dimension ref="A1:X1089"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -86742,6 +86742,326 @@
       <c r="W1085" s="6" t="inlineStr"/>
       <c r="X1085" s="6" t="inlineStr"/>
     </row>
+    <row r="1086">
+      <c r="A1086" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1086" s="2" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1086" s="2" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1086" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1086" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1086" s="2" t="n">
+        <v>235.53</v>
+      </c>
+      <c r="G1086" s="2" t="n">
+        <v>235.51</v>
+      </c>
+      <c r="H1086" s="2" t="n">
+        <v>236.37</v>
+      </c>
+      <c r="I1086" s="2" t="n">
+        <v>233.75</v>
+      </c>
+      <c r="J1086" s="2" t="n">
+        <v>234.89</v>
+      </c>
+      <c r="K1086" s="2" t="n">
+        <v>236.37</v>
+      </c>
+      <c r="L1086" s="2" t="n">
+        <v>233.75</v>
+      </c>
+      <c r="M1086" s="2" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="N1086" s="4" t="n">
+        <v>236.42</v>
+      </c>
+      <c r="O1086" s="5" t="n">
+        <v>235.01</v>
+      </c>
+      <c r="P1086" s="3" t="n">
+        <v>237.73</v>
+      </c>
+      <c r="Q1086" s="3" t="n">
+        <v>239.04</v>
+      </c>
+      <c r="R1086" s="2" t="n">
+        <v>2114</v>
+      </c>
+      <c r="S1086" s="2" t="n">
+        <v>2981</v>
+      </c>
+      <c r="T1086" s="2" t="n">
+        <v>2769</v>
+      </c>
+      <c r="U1086" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1086" s="2" t="inlineStr"/>
+      <c r="W1086" s="2" t="inlineStr"/>
+      <c r="X1086" s="2" t="inlineStr"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="2" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1087" s="2" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="C1087" s="2" t="inlineStr">
+        <is>
+          <t>REALTY</t>
+        </is>
+      </c>
+      <c r="D1087" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1087" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1087" s="2" t="n">
+        <v>670</v>
+      </c>
+      <c r="G1087" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="H1087" s="2" t="n">
+        <v>671.8</v>
+      </c>
+      <c r="I1087" s="2" t="n">
+        <v>659.05</v>
+      </c>
+      <c r="J1087" s="2" t="n">
+        <v>661.08</v>
+      </c>
+      <c r="K1087" s="2" t="n">
+        <v>671.8</v>
+      </c>
+      <c r="L1087" s="2" t="n">
+        <v>659.05</v>
+      </c>
+      <c r="M1087" s="2" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="N1087" s="4" t="n">
+        <v>671.85</v>
+      </c>
+      <c r="O1087" s="5" t="n">
+        <v>665.37</v>
+      </c>
+      <c r="P1087" s="3" t="n">
+        <v>678.23</v>
+      </c>
+      <c r="Q1087" s="3" t="n">
+        <v>684.6</v>
+      </c>
+      <c r="R1087" s="2" t="n">
+        <v>462</v>
+      </c>
+      <c r="S1087" s="2" t="n">
+        <v>2994</v>
+      </c>
+      <c r="T1087" s="2" t="n">
+        <v>2948</v>
+      </c>
+      <c r="U1087" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1087" s="2" t="inlineStr"/>
+      <c r="W1087" s="2" t="inlineStr"/>
+      <c r="X1087" s="2" t="inlineStr"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1088" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1088" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1088" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1088" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1088" s="6" t="n">
+        <v>1012.2</v>
+      </c>
+      <c r="G1088" s="6" t="n">
+        <v>1025.3</v>
+      </c>
+      <c r="H1088" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="I1088" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="J1088" s="6" t="n">
+        <v>1047.03</v>
+      </c>
+      <c r="K1088" s="6" t="n">
+        <v>1029.2</v>
+      </c>
+      <c r="L1088" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="M1088" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="N1088" s="8" t="n">
+        <v>1004.95</v>
+      </c>
+      <c r="O1088" s="7" t="n">
+        <v>1017.15</v>
+      </c>
+      <c r="P1088" s="9" t="n">
+        <v>992.85</v>
+      </c>
+      <c r="Q1088" s="9" t="n">
+        <v>980.75</v>
+      </c>
+      <c r="R1088" s="6" t="n">
+        <v>243</v>
+      </c>
+      <c r="S1088" s="6" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1088" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1088" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1088" s="6" t="inlineStr"/>
+      <c r="W1088" s="6" t="inlineStr"/>
+      <c r="X1088" s="6" t="inlineStr"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="6" t="inlineStr">
+        <is>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1089" s="6" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="C1089" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1089" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1089" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1089" s="6" t="n">
+        <v>1830.2</v>
+      </c>
+      <c r="G1089" s="6" t="n">
+        <v>1862.7</v>
+      </c>
+      <c r="H1089" s="6" t="n">
+        <v>1863</v>
+      </c>
+      <c r="I1089" s="6" t="n">
+        <v>1823.8</v>
+      </c>
+      <c r="J1089" s="6" t="n">
+        <v>1940.47</v>
+      </c>
+      <c r="K1089" s="6" t="n">
+        <v>1863</v>
+      </c>
+      <c r="L1089" s="6" t="n">
+        <v>1823.8</v>
+      </c>
+      <c r="M1089" s="6" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="N1089" s="8" t="n">
+        <v>1823.75</v>
+      </c>
+      <c r="O1089" s="7" t="n">
+        <v>1843.45</v>
+      </c>
+      <c r="P1089" s="9" t="n">
+        <v>1804.15</v>
+      </c>
+      <c r="Q1089" s="9" t="n">
+        <v>1784.55</v>
+      </c>
+      <c r="R1089" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="S1089" s="6" t="n">
+        <v>2955</v>
+      </c>
+      <c r="T1089" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1089" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1089" s="6" t="inlineStr"/>
+      <c r="W1089" s="6" t="inlineStr"/>
+      <c r="X1089" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 23-Sep-2026 08:39 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1089"/>
+  <dimension ref="A1:X1093"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -87062,6 +87062,326 @@
       <c r="W1089" s="6" t="inlineStr"/>
       <c r="X1089" s="6" t="inlineStr"/>
     </row>
+    <row r="1090">
+      <c r="A1090" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1090" s="2" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1090" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1090" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1090" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1090" s="2" t="n">
+        <v>563.8</v>
+      </c>
+      <c r="G1090" s="2" t="n">
+        <v>561.9</v>
+      </c>
+      <c r="H1090" s="2" t="n">
+        <v>564.25</v>
+      </c>
+      <c r="I1090" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="J1090" s="2" t="n">
+        <v>539.08</v>
+      </c>
+      <c r="K1090" s="2" t="n">
+        <v>564.25</v>
+      </c>
+      <c r="L1090" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="M1090" s="2" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="N1090" s="4" t="n">
+        <v>564.3</v>
+      </c>
+      <c r="O1090" s="5" t="n">
+        <v>560.28</v>
+      </c>
+      <c r="P1090" s="3" t="n">
+        <v>568.22</v>
+      </c>
+      <c r="Q1090" s="3" t="n">
+        <v>572.15</v>
+      </c>
+      <c r="R1090" s="2" t="n">
+        <v>744</v>
+      </c>
+      <c r="S1090" s="2" t="n">
+        <v>2991</v>
+      </c>
+      <c r="T1090" s="2" t="n">
+        <v>2916</v>
+      </c>
+      <c r="U1090" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1090" s="2" t="inlineStr"/>
+      <c r="W1090" s="2" t="inlineStr"/>
+      <c r="X1090" s="2" t="inlineStr"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1091" s="2" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1091" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1091" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1091" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1091" s="2" t="n">
+        <v>402.25</v>
+      </c>
+      <c r="G1091" s="2" t="n">
+        <v>398.85</v>
+      </c>
+      <c r="H1091" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="I1091" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="J1091" s="2" t="n">
+        <v>399.17</v>
+      </c>
+      <c r="K1091" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="L1091" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="M1091" s="2" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="N1091" s="4" t="n">
+        <v>402.8</v>
+      </c>
+      <c r="O1091" s="5" t="n">
+        <v>400.13</v>
+      </c>
+      <c r="P1091" s="3" t="n">
+        <v>405.38</v>
+      </c>
+      <c r="Q1091" s="3" t="n">
+        <v>407.95</v>
+      </c>
+      <c r="R1091" s="2" t="n">
+        <v>1122</v>
+      </c>
+      <c r="S1091" s="2" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1091" s="2" t="n">
+        <v>2895</v>
+      </c>
+      <c r="U1091" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1091" s="2" t="inlineStr"/>
+      <c r="W1091" s="2" t="inlineStr"/>
+      <c r="X1091" s="2" t="inlineStr"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1092" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1092" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1092" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1092" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1092" s="6" t="n">
+        <v>1018.2</v>
+      </c>
+      <c r="G1092" s="6" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="H1092" s="6" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="I1092" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="J1092" s="6" t="n">
+        <v>1083.99</v>
+      </c>
+      <c r="K1092" s="6" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="L1092" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="M1092" s="6" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="N1092" s="8" t="n">
+        <v>1015.05</v>
+      </c>
+      <c r="O1092" s="7" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="P1092" s="9" t="n">
+        <v>1007.9</v>
+      </c>
+      <c r="Q1092" s="9" t="n">
+        <v>1000.75</v>
+      </c>
+      <c r="R1092" s="6" t="n">
+        <v>411</v>
+      </c>
+      <c r="S1092" s="6" t="n">
+        <v>2980</v>
+      </c>
+      <c r="T1092" s="6" t="n">
+        <v>2939</v>
+      </c>
+      <c r="U1092" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1092" s="6" t="inlineStr"/>
+      <c r="W1092" s="6" t="inlineStr"/>
+      <c r="X1092" s="6" t="inlineStr"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1093" s="6" t="inlineStr">
+        <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="C1093" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1093" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1093" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1093" s="6" t="n">
+        <v>4095.8</v>
+      </c>
+      <c r="G1093" s="6" t="n">
+        <v>4160</v>
+      </c>
+      <c r="H1093" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="I1093" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="J1093" s="6" t="n">
+        <v>4400.1</v>
+      </c>
+      <c r="K1093" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="L1093" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="M1093" s="6" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="N1093" s="8" t="n">
+        <v>4085.05</v>
+      </c>
+      <c r="O1093" s="7" t="n">
+        <v>4137.9</v>
+      </c>
+      <c r="P1093" s="9" t="n">
+        <v>4032.3</v>
+      </c>
+      <c r="Q1093" s="9" t="n">
+        <v>3979.55</v>
+      </c>
+      <c r="R1093" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="S1093" s="6" t="n">
+        <v>2854</v>
+      </c>
+      <c r="T1093" s="6" t="n">
+        <v>2848</v>
+      </c>
+      <c r="U1093" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1093" s="6" t="inlineStr"/>
+      <c r="W1093" s="6" t="inlineStr"/>
+      <c r="X1093" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 23-Sep-2026 08:47 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1093"/>
+  <dimension ref="A1:X1097"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -87382,6 +87382,326 @@
       <c r="W1093" s="6" t="inlineStr"/>
       <c r="X1093" s="6" t="inlineStr"/>
     </row>
+    <row r="1094">
+      <c r="A1094" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1094" s="2" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1094" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1094" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1094" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1094" s="2" t="n">
+        <v>563.6</v>
+      </c>
+      <c r="G1094" s="2" t="n">
+        <v>561.9</v>
+      </c>
+      <c r="H1094" s="2" t="n">
+        <v>564.25</v>
+      </c>
+      <c r="I1094" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="J1094" s="2" t="n">
+        <v>539.08</v>
+      </c>
+      <c r="K1094" s="2" t="n">
+        <v>564.25</v>
+      </c>
+      <c r="L1094" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="M1094" s="2" t="n">
+        <v>7.85</v>
+      </c>
+      <c r="N1094" s="4" t="n">
+        <v>564.3</v>
+      </c>
+      <c r="O1094" s="5" t="n">
+        <v>560.28</v>
+      </c>
+      <c r="P1094" s="3" t="n">
+        <v>568.22</v>
+      </c>
+      <c r="Q1094" s="3" t="n">
+        <v>572.15</v>
+      </c>
+      <c r="R1094" s="2" t="n">
+        <v>744</v>
+      </c>
+      <c r="S1094" s="2" t="n">
+        <v>2991</v>
+      </c>
+      <c r="T1094" s="2" t="n">
+        <v>2916</v>
+      </c>
+      <c r="U1094" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1094" s="2" t="inlineStr"/>
+      <c r="W1094" s="2" t="inlineStr"/>
+      <c r="X1094" s="2" t="inlineStr"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1095" s="2" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1095" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1095" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1095" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1095" s="2" t="n">
+        <v>1766.3</v>
+      </c>
+      <c r="G1095" s="2" t="n">
+        <v>1758</v>
+      </c>
+      <c r="H1095" s="2" t="n">
+        <v>1768</v>
+      </c>
+      <c r="I1095" s="2" t="n">
+        <v>1744.4</v>
+      </c>
+      <c r="J1095" s="2" t="n">
+        <v>1733.01</v>
+      </c>
+      <c r="K1095" s="2" t="n">
+        <v>1768</v>
+      </c>
+      <c r="L1095" s="2" t="n">
+        <v>1744.4</v>
+      </c>
+      <c r="M1095" s="2" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="N1095" s="4" t="n">
+        <v>1768.05</v>
+      </c>
+      <c r="O1095" s="5" t="n">
+        <v>1756.15</v>
+      </c>
+      <c r="P1095" s="3" t="n">
+        <v>1779.85</v>
+      </c>
+      <c r="Q1095" s="3" t="n">
+        <v>1791.65</v>
+      </c>
+      <c r="R1095" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="S1095" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1095" s="2" t="n">
+        <v>2974</v>
+      </c>
+      <c r="U1095" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1095" s="2" t="inlineStr"/>
+      <c r="W1095" s="2" t="inlineStr"/>
+      <c r="X1095" s="2" t="inlineStr"/>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1096" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1096" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1096" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1096" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1096" s="6" t="n">
+        <v>1018.8</v>
+      </c>
+      <c r="G1096" s="6" t="n">
+        <v>1021.8</v>
+      </c>
+      <c r="H1096" s="6" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="I1096" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="J1096" s="6" t="n">
+        <v>1083.98</v>
+      </c>
+      <c r="K1096" s="6" t="n">
+        <v>1029.4</v>
+      </c>
+      <c r="L1096" s="6" t="n">
+        <v>1015.1</v>
+      </c>
+      <c r="M1096" s="6" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="N1096" s="8" t="n">
+        <v>1015.05</v>
+      </c>
+      <c r="O1096" s="7" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="P1096" s="9" t="n">
+        <v>1007.9</v>
+      </c>
+      <c r="Q1096" s="9" t="n">
+        <v>1000.75</v>
+      </c>
+      <c r="R1096" s="6" t="n">
+        <v>411</v>
+      </c>
+      <c r="S1096" s="6" t="n">
+        <v>2980</v>
+      </c>
+      <c r="T1096" s="6" t="n">
+        <v>2939</v>
+      </c>
+      <c r="U1096" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1096" s="6" t="inlineStr"/>
+      <c r="W1096" s="6" t="inlineStr"/>
+      <c r="X1096" s="6" t="inlineStr"/>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1097" s="6" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C1097" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1097" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1097" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1097" s="6" t="n">
+        <v>2082.6</v>
+      </c>
+      <c r="G1097" s="6" t="n">
+        <v>2099</v>
+      </c>
+      <c r="H1097" s="6" t="n">
+        <v>2104.2</v>
+      </c>
+      <c r="I1097" s="6" t="n">
+        <v>2081.1</v>
+      </c>
+      <c r="J1097" s="6" t="n">
+        <v>2237.03</v>
+      </c>
+      <c r="K1097" s="6" t="n">
+        <v>2104.2</v>
+      </c>
+      <c r="L1097" s="6" t="n">
+        <v>2081.1</v>
+      </c>
+      <c r="M1097" s="6" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="N1097" s="8" t="n">
+        <v>2081.05</v>
+      </c>
+      <c r="O1097" s="7" t="n">
+        <v>2092.7</v>
+      </c>
+      <c r="P1097" s="9" t="n">
+        <v>2069.5</v>
+      </c>
+      <c r="Q1097" s="9" t="n">
+        <v>2057.95</v>
+      </c>
+      <c r="R1097" s="6" t="n">
+        <v>240</v>
+      </c>
+      <c r="S1097" s="6" t="n">
+        <v>2796</v>
+      </c>
+      <c r="T1097" s="6" t="n">
+        <v>2772</v>
+      </c>
+      <c r="U1097" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1097" s="6" t="inlineStr"/>
+      <c r="W1097" s="6" t="inlineStr"/>
+      <c r="X1097" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 23-Sep-2026 09:13 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1097"/>
+  <dimension ref="A1:X1101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -87702,6 +87702,326 @@
       <c r="W1097" s="6" t="inlineStr"/>
       <c r="X1097" s="6" t="inlineStr"/>
     </row>
+    <row r="1098">
+      <c r="A1098" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1098" s="2" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1098" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1098" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1098" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1098" s="2" t="n">
+        <v>564.7</v>
+      </c>
+      <c r="G1098" s="2" t="n">
+        <v>561.9</v>
+      </c>
+      <c r="H1098" s="2" t="n">
+        <v>565.5</v>
+      </c>
+      <c r="I1098" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="J1098" s="2" t="n">
+        <v>539.17</v>
+      </c>
+      <c r="K1098" s="2" t="n">
+        <v>565.5</v>
+      </c>
+      <c r="L1098" s="2" t="n">
+        <v>556.4</v>
+      </c>
+      <c r="M1098" s="2" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="N1098" s="4" t="n">
+        <v>565.55</v>
+      </c>
+      <c r="O1098" s="5" t="n">
+        <v>560.9</v>
+      </c>
+      <c r="P1098" s="3" t="n">
+        <v>570.1</v>
+      </c>
+      <c r="Q1098" s="3" t="n">
+        <v>574.65</v>
+      </c>
+      <c r="R1098" s="2" t="n">
+        <v>645</v>
+      </c>
+      <c r="S1098" s="2" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1098" s="2" t="n">
+        <v>2935</v>
+      </c>
+      <c r="U1098" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1098" s="2" t="inlineStr"/>
+      <c r="W1098" s="2" t="inlineStr"/>
+      <c r="X1098" s="2" t="inlineStr"/>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1099" s="2" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1099" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1099" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1099" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1099" s="2" t="n">
+        <v>401.1</v>
+      </c>
+      <c r="G1099" s="2" t="n">
+        <v>398.85</v>
+      </c>
+      <c r="H1099" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="I1099" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="J1099" s="2" t="n">
+        <v>399.16</v>
+      </c>
+      <c r="K1099" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="L1099" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="M1099" s="2" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="N1099" s="4" t="n">
+        <v>402.8</v>
+      </c>
+      <c r="O1099" s="5" t="n">
+        <v>400.13</v>
+      </c>
+      <c r="P1099" s="3" t="n">
+        <v>405.38</v>
+      </c>
+      <c r="Q1099" s="3" t="n">
+        <v>407.95</v>
+      </c>
+      <c r="R1099" s="2" t="n">
+        <v>1122</v>
+      </c>
+      <c r="S1099" s="2" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1099" s="2" t="n">
+        <v>2895</v>
+      </c>
+      <c r="U1099" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1099" s="2" t="inlineStr"/>
+      <c r="W1099" s="2" t="inlineStr"/>
+      <c r="X1099" s="2" t="inlineStr"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1100" s="6" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="C1100" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1100" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1100" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1100" s="6" t="n">
+        <v>1254</v>
+      </c>
+      <c r="G1100" s="6" t="n">
+        <v>1270</v>
+      </c>
+      <c r="H1100" s="6" t="n">
+        <v>1279.8</v>
+      </c>
+      <c r="I1100" s="6" t="n">
+        <v>1252.7</v>
+      </c>
+      <c r="J1100" s="6" t="n">
+        <v>1280.18</v>
+      </c>
+      <c r="K1100" s="6" t="n">
+        <v>1279.8</v>
+      </c>
+      <c r="L1100" s="6" t="n">
+        <v>1252.7</v>
+      </c>
+      <c r="M1100" s="6" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="N1100" s="8" t="n">
+        <v>1252.65</v>
+      </c>
+      <c r="O1100" s="7" t="n">
+        <v>1266.3</v>
+      </c>
+      <c r="P1100" s="9" t="n">
+        <v>1239.1</v>
+      </c>
+      <c r="Q1100" s="9" t="n">
+        <v>1225.55</v>
+      </c>
+      <c r="R1100" s="6" t="n">
+        <v>219</v>
+      </c>
+      <c r="S1100" s="6" t="n">
+        <v>2989</v>
+      </c>
+      <c r="T1100" s="6" t="n">
+        <v>2967</v>
+      </c>
+      <c r="U1100" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1100" s="6" t="inlineStr"/>
+      <c r="W1100" s="6" t="inlineStr"/>
+      <c r="X1100" s="6" t="inlineStr"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1101" s="6" t="inlineStr">
+        <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="C1101" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1101" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1101" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1101" s="6" t="n">
+        <v>4095.3</v>
+      </c>
+      <c r="G1101" s="6" t="n">
+        <v>4160</v>
+      </c>
+      <c r="H1101" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="I1101" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="J1101" s="6" t="n">
+        <v>4399.58</v>
+      </c>
+      <c r="K1101" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="L1101" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="M1101" s="6" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="N1101" s="8" t="n">
+        <v>4085.05</v>
+      </c>
+      <c r="O1101" s="7" t="n">
+        <v>4137.9</v>
+      </c>
+      <c r="P1101" s="9" t="n">
+        <v>4032.3</v>
+      </c>
+      <c r="Q1101" s="9" t="n">
+        <v>3979.55</v>
+      </c>
+      <c r="R1101" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="S1101" s="6" t="n">
+        <v>2854</v>
+      </c>
+      <c r="T1101" s="6" t="n">
+        <v>2848</v>
+      </c>
+      <c r="U1101" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1101" s="6" t="inlineStr"/>
+      <c r="W1101" s="6" t="inlineStr"/>
+      <c r="X1101" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 23-Sep-2026 09:20 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1101"/>
+  <dimension ref="A1:X1105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -88022,6 +88022,326 @@
       <c r="W1101" s="6" t="inlineStr"/>
       <c r="X1101" s="6" t="inlineStr"/>
     </row>
+    <row r="1102">
+      <c r="A1102" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1102" s="2" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="C1102" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1102" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1102" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1102" s="2" t="n">
+        <v>1761.7</v>
+      </c>
+      <c r="G1102" s="2" t="n">
+        <v>1758</v>
+      </c>
+      <c r="H1102" s="2" t="n">
+        <v>1770.1</v>
+      </c>
+      <c r="I1102" s="2" t="n">
+        <v>1744.4</v>
+      </c>
+      <c r="J1102" s="2" t="n">
+        <v>1733.16</v>
+      </c>
+      <c r="K1102" s="2" t="n">
+        <v>1770.1</v>
+      </c>
+      <c r="L1102" s="2" t="n">
+        <v>1744.4</v>
+      </c>
+      <c r="M1102" s="2" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="N1102" s="4" t="n">
+        <v>1770.15</v>
+      </c>
+      <c r="O1102" s="5" t="n">
+        <v>1757.2</v>
+      </c>
+      <c r="P1102" s="3" t="n">
+        <v>1783</v>
+      </c>
+      <c r="Q1102" s="3" t="n">
+        <v>1795.85</v>
+      </c>
+      <c r="R1102" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="S1102" s="2" t="n">
+        <v>2991</v>
+      </c>
+      <c r="T1102" s="2" t="n">
+        <v>2968</v>
+      </c>
+      <c r="U1102" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1102" s="2" t="inlineStr"/>
+      <c r="W1102" s="2" t="inlineStr"/>
+      <c r="X1102" s="2" t="inlineStr"/>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="2" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1103" s="2" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1103" s="2" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1103" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1103" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1103" s="2" t="n">
+        <v>401</v>
+      </c>
+      <c r="G1103" s="2" t="n">
+        <v>398.85</v>
+      </c>
+      <c r="H1103" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="I1103" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="J1103" s="2" t="n">
+        <v>399.16</v>
+      </c>
+      <c r="K1103" s="2" t="n">
+        <v>402.75</v>
+      </c>
+      <c r="L1103" s="2" t="n">
+        <v>397.6</v>
+      </c>
+      <c r="M1103" s="2" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="N1103" s="4" t="n">
+        <v>402.8</v>
+      </c>
+      <c r="O1103" s="5" t="n">
+        <v>400.13</v>
+      </c>
+      <c r="P1103" s="3" t="n">
+        <v>405.38</v>
+      </c>
+      <c r="Q1103" s="3" t="n">
+        <v>407.95</v>
+      </c>
+      <c r="R1103" s="2" t="n">
+        <v>1122</v>
+      </c>
+      <c r="S1103" s="2" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1103" s="2" t="n">
+        <v>2895</v>
+      </c>
+      <c r="U1103" s="2" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1103" s="2" t="inlineStr"/>
+      <c r="W1103" s="2" t="inlineStr"/>
+      <c r="X1103" s="2" t="inlineStr"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1104" s="6" t="inlineStr">
+        <is>
+          <t>LTIM</t>
+        </is>
+      </c>
+      <c r="C1104" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1104" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1104" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1104" s="6" t="n">
+        <v>4091.3</v>
+      </c>
+      <c r="G1104" s="6" t="n">
+        <v>4160</v>
+      </c>
+      <c r="H1104" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="I1104" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="J1104" s="6" t="n">
+        <v>4399.3</v>
+      </c>
+      <c r="K1104" s="6" t="n">
+        <v>4190.6</v>
+      </c>
+      <c r="L1104" s="6" t="n">
+        <v>4085.1</v>
+      </c>
+      <c r="M1104" s="6" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="N1104" s="8" t="n">
+        <v>4085.05</v>
+      </c>
+      <c r="O1104" s="7" t="n">
+        <v>4137.9</v>
+      </c>
+      <c r="P1104" s="9" t="n">
+        <v>4032.3</v>
+      </c>
+      <c r="Q1104" s="9" t="n">
+        <v>3979.55</v>
+      </c>
+      <c r="R1104" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="S1104" s="6" t="n">
+        <v>2854</v>
+      </c>
+      <c r="T1104" s="6" t="n">
+        <v>2848</v>
+      </c>
+      <c r="U1104" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1104" s="6" t="inlineStr"/>
+      <c r="W1104" s="6" t="inlineStr"/>
+      <c r="X1104" s="6" t="inlineStr"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="6" t="inlineStr">
+        <is>
+          <t>23-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1105" s="6" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+      <c r="C1105" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1105" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1105" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1105" s="6" t="n">
+        <v>5230.5</v>
+      </c>
+      <c r="G1105" s="6" t="n">
+        <v>5400</v>
+      </c>
+      <c r="H1105" s="6" t="n">
+        <v>5413</v>
+      </c>
+      <c r="I1105" s="6" t="n">
+        <v>5223.5</v>
+      </c>
+      <c r="J1105" s="6" t="n">
+        <v>5581.73</v>
+      </c>
+      <c r="K1105" s="6" t="n">
+        <v>5413</v>
+      </c>
+      <c r="L1105" s="6" t="n">
+        <v>5223.5</v>
+      </c>
+      <c r="M1105" s="6" t="n">
+        <v>189.5</v>
+      </c>
+      <c r="N1105" s="8" t="n">
+        <v>5223.45</v>
+      </c>
+      <c r="O1105" s="7" t="n">
+        <v>5318.3</v>
+      </c>
+      <c r="P1105" s="9" t="n">
+        <v>5128.7</v>
+      </c>
+      <c r="Q1105" s="9" t="n">
+        <v>5033.95</v>
+      </c>
+      <c r="R1105" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="S1105" s="6" t="n">
+        <v>2846</v>
+      </c>
+      <c r="T1105" s="6" t="n">
+        <v>2842</v>
+      </c>
+      <c r="U1105" s="6" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+      <c r="V1105" s="6" t="inlineStr"/>
+      <c r="W1105" s="6" t="inlineStr"/>
+      <c r="X1105" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 24-Sep-2026 08:33 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1105"/>
+  <dimension ref="A1:X1109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -88342,6 +88342,326 @@
       <c r="W1105" s="6" t="inlineStr"/>
       <c r="X1105" s="6" t="inlineStr"/>
     </row>
+    <row r="1106">
+      <c r="A1106" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1106" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1106" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1106" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1106" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1106" s="2" t="n">
+        <v>1199.7</v>
+      </c>
+      <c r="G1106" s="2" t="n">
+        <v>1210.9</v>
+      </c>
+      <c r="H1106" s="2" t="n">
+        <v>1213.9</v>
+      </c>
+      <c r="I1106" s="2" t="n">
+        <v>1199.2</v>
+      </c>
+      <c r="J1106" s="2" t="n">
+        <v>1175.3</v>
+      </c>
+      <c r="K1106" s="2" t="n">
+        <v>1213.9</v>
+      </c>
+      <c r="L1106" s="2" t="n">
+        <v>1199.2</v>
+      </c>
+      <c r="M1106" s="2" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="N1106" s="4" t="n">
+        <v>1213.95</v>
+      </c>
+      <c r="O1106" s="5" t="n">
+        <v>1206.5</v>
+      </c>
+      <c r="P1106" s="3" t="n">
+        <v>1221.3</v>
+      </c>
+      <c r="Q1106" s="3" t="n">
+        <v>1228.65</v>
+      </c>
+      <c r="R1106" s="2" t="n">
+        <v>402</v>
+      </c>
+      <c r="S1106" s="2" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1106" s="2" t="n">
+        <v>2955</v>
+      </c>
+      <c r="U1106" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1106" s="2" t="inlineStr"/>
+      <c r="W1106" s="2" t="inlineStr"/>
+      <c r="X1106" s="2" t="inlineStr"/>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1107" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C1107" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1107" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1107" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1107" s="2" t="n">
+        <v>1724.5</v>
+      </c>
+      <c r="G1107" s="2" t="n">
+        <v>1719.7</v>
+      </c>
+      <c r="H1107" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="I1107" s="2" t="n">
+        <v>1710</v>
+      </c>
+      <c r="J1107" s="2" t="n">
+        <v>1680.6</v>
+      </c>
+      <c r="K1107" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="L1107" s="2" t="n">
+        <v>1710</v>
+      </c>
+      <c r="M1107" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="N1107" s="4" t="n">
+        <v>1740.05</v>
+      </c>
+      <c r="O1107" s="5" t="n">
+        <v>1724.95</v>
+      </c>
+      <c r="P1107" s="3" t="n">
+        <v>1755.05</v>
+      </c>
+      <c r="Q1107" s="3" t="n">
+        <v>1770.05</v>
+      </c>
+      <c r="R1107" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="S1107" s="2" t="n">
+        <v>2990</v>
+      </c>
+      <c r="T1107" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1107" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1107" s="2" t="inlineStr"/>
+      <c r="W1107" s="2" t="inlineStr"/>
+      <c r="X1107" s="2" t="inlineStr"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1108" s="6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C1108" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1108" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1108" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1108" s="6" t="n">
+        <v>1178.5</v>
+      </c>
+      <c r="G1108" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="H1108" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="I1108" s="6" t="n">
+        <v>1177.9</v>
+      </c>
+      <c r="J1108" s="6" t="n">
+        <v>1248.58</v>
+      </c>
+      <c r="K1108" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="L1108" s="6" t="n">
+        <v>1177.9</v>
+      </c>
+      <c r="M1108" s="6" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="N1108" s="8" t="n">
+        <v>1177.85</v>
+      </c>
+      <c r="O1108" s="7" t="n">
+        <v>1201.6</v>
+      </c>
+      <c r="P1108" s="9" t="n">
+        <v>1154.2</v>
+      </c>
+      <c r="Q1108" s="9" t="n">
+        <v>1130.55</v>
+      </c>
+      <c r="R1108" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="S1108" s="6" t="n">
+        <v>2992</v>
+      </c>
+      <c r="T1108" s="6" t="n">
+        <v>2980</v>
+      </c>
+      <c r="U1108" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1108" s="6" t="inlineStr"/>
+      <c r="W1108" s="6" t="inlineStr"/>
+      <c r="X1108" s="6" t="inlineStr"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1109" s="6" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
+      <c r="C1109" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1109" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1109" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1109" s="6" t="n">
+        <v>916.7</v>
+      </c>
+      <c r="G1109" s="6" t="n">
+        <v>918</v>
+      </c>
+      <c r="H1109" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="I1109" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="J1109" s="6" t="n">
+        <v>970.6</v>
+      </c>
+      <c r="K1109" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="L1109" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="M1109" s="6" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="N1109" s="8" t="n">
+        <v>909.25</v>
+      </c>
+      <c r="O1109" s="7" t="n">
+        <v>919.15</v>
+      </c>
+      <c r="P1109" s="9" t="n">
+        <v>899.45</v>
+      </c>
+      <c r="Q1109" s="9" t="n">
+        <v>889.65</v>
+      </c>
+      <c r="R1109" s="6" t="n">
+        <v>303</v>
+      </c>
+      <c r="S1109" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1109" s="6" t="n">
+        <v>2969</v>
+      </c>
+      <c r="U1109" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1109" s="6" t="inlineStr"/>
+      <c r="W1109" s="6" t="inlineStr"/>
+      <c r="X1109" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 24-Sep-2026 08:41 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1109"/>
+  <dimension ref="A1:X1113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -88662,6 +88662,326 @@
       <c r="W1109" s="6" t="inlineStr"/>
       <c r="X1109" s="6" t="inlineStr"/>
     </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1110" s="2" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C1110" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1110" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1110" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1110" s="2" t="n">
+        <v>2075.3</v>
+      </c>
+      <c r="G1110" s="2" t="n">
+        <v>2076</v>
+      </c>
+      <c r="H1110" s="2" t="n">
+        <v>2096.9</v>
+      </c>
+      <c r="I1110" s="2" t="n">
+        <v>2067.1</v>
+      </c>
+      <c r="J1110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1110" s="2" t="n">
+        <v>2096.9</v>
+      </c>
+      <c r="L1110" s="2" t="n">
+        <v>2067.1</v>
+      </c>
+      <c r="M1110" s="2" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="N1110" s="4" t="n">
+        <v>2096.95</v>
+      </c>
+      <c r="O1110" s="5" t="n">
+        <v>2081.95</v>
+      </c>
+      <c r="P1110" s="3" t="n">
+        <v>2111.85</v>
+      </c>
+      <c r="Q1110" s="3" t="n">
+        <v>2126.75</v>
+      </c>
+      <c r="R1110" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="S1110" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="T1110" s="2" t="n">
+        <v>2950</v>
+      </c>
+      <c r="U1110" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1110" s="2" t="inlineStr"/>
+      <c r="W1110" s="2" t="inlineStr"/>
+      <c r="X1110" s="2" t="inlineStr"/>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1111" s="2" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="C1111" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1111" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1111" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1111" s="2" t="n">
+        <v>163.81</v>
+      </c>
+      <c r="G1111" s="2" t="n">
+        <v>164.16</v>
+      </c>
+      <c r="H1111" s="2" t="n">
+        <v>165.67</v>
+      </c>
+      <c r="I1111" s="2" t="n">
+        <v>163.58</v>
+      </c>
+      <c r="J1111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1111" s="2" t="n">
+        <v>165.67</v>
+      </c>
+      <c r="L1111" s="2" t="n">
+        <v>163.58</v>
+      </c>
+      <c r="M1111" s="2" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="N1111" s="4" t="n">
+        <v>165.72</v>
+      </c>
+      <c r="O1111" s="5" t="n">
+        <v>164.57</v>
+      </c>
+      <c r="P1111" s="3" t="n">
+        <v>166.76</v>
+      </c>
+      <c r="Q1111" s="3" t="n">
+        <v>167.81</v>
+      </c>
+      <c r="R1111" s="2" t="n">
+        <v>2607</v>
+      </c>
+      <c r="S1111" s="2" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1111" s="2" t="n">
+        <v>2711</v>
+      </c>
+      <c r="U1111" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1111" s="2" t="inlineStr"/>
+      <c r="W1111" s="2" t="inlineStr"/>
+      <c r="X1111" s="2" t="inlineStr"/>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1112" s="6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C1112" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1112" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1112" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1112" s="6" t="n">
+        <v>1178.1</v>
+      </c>
+      <c r="G1112" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="H1112" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="I1112" s="6" t="n">
+        <v>1177.3</v>
+      </c>
+      <c r="J1112" s="6" t="n">
+        <v>1248.45</v>
+      </c>
+      <c r="K1112" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="L1112" s="6" t="n">
+        <v>1177.3</v>
+      </c>
+      <c r="M1112" s="6" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="N1112" s="8" t="n">
+        <v>1177.25</v>
+      </c>
+      <c r="O1112" s="7" t="n">
+        <v>1201.3</v>
+      </c>
+      <c r="P1112" s="9" t="n">
+        <v>1153.3</v>
+      </c>
+      <c r="Q1112" s="9" t="n">
+        <v>1129.35</v>
+      </c>
+      <c r="R1112" s="6" t="n">
+        <v>123</v>
+      </c>
+      <c r="S1112" s="6" t="n">
+        <v>2958</v>
+      </c>
+      <c r="T1112" s="6" t="n">
+        <v>2946</v>
+      </c>
+      <c r="U1112" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1112" s="6" t="inlineStr"/>
+      <c r="W1112" s="6" t="inlineStr"/>
+      <c r="X1112" s="6" t="inlineStr"/>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1113" s="6" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
+      <c r="C1113" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1113" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1113" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1113" s="6" t="n">
+        <v>918</v>
+      </c>
+      <c r="G1113" s="6" t="n">
+        <v>918</v>
+      </c>
+      <c r="H1113" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="I1113" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="J1113" s="6" t="n">
+        <v>970.55</v>
+      </c>
+      <c r="K1113" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="L1113" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="M1113" s="6" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="N1113" s="8" t="n">
+        <v>909.25</v>
+      </c>
+      <c r="O1113" s="7" t="n">
+        <v>919.15</v>
+      </c>
+      <c r="P1113" s="9" t="n">
+        <v>899.45</v>
+      </c>
+      <c r="Q1113" s="9" t="n">
+        <v>889.65</v>
+      </c>
+      <c r="R1113" s="6" t="n">
+        <v>303</v>
+      </c>
+      <c r="S1113" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1113" s="6" t="n">
+        <v>2969</v>
+      </c>
+      <c r="U1113" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1113" s="6" t="inlineStr"/>
+      <c r="W1113" s="6" t="inlineStr"/>
+      <c r="X1113" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 24-Sep-2026 09:11 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1113"/>
+  <dimension ref="A1:X1117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -88982,6 +88982,326 @@
       <c r="W1113" s="6" t="inlineStr"/>
       <c r="X1113" s="6" t="inlineStr"/>
     </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="C1114" s="2" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1114" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1114" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1114" s="2" t="n">
+        <v>2072.4</v>
+      </c>
+      <c r="G1114" s="2" t="n">
+        <v>2076</v>
+      </c>
+      <c r="H1114" s="2" t="n">
+        <v>2096.9</v>
+      </c>
+      <c r="I1114" s="2" t="n">
+        <v>2067.1</v>
+      </c>
+      <c r="J1114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1114" s="2" t="n">
+        <v>2096.9</v>
+      </c>
+      <c r="L1114" s="2" t="n">
+        <v>2067.1</v>
+      </c>
+      <c r="M1114" s="2" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="N1114" s="4" t="n">
+        <v>2096.95</v>
+      </c>
+      <c r="O1114" s="5" t="n">
+        <v>2081.95</v>
+      </c>
+      <c r="P1114" s="3" t="n">
+        <v>2111.85</v>
+      </c>
+      <c r="Q1114" s="3" t="n">
+        <v>2126.75</v>
+      </c>
+      <c r="R1114" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="S1114" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="T1114" s="2" t="n">
+        <v>2950</v>
+      </c>
+      <c r="U1114" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1114" s="2" t="inlineStr"/>
+      <c r="W1114" s="2" t="inlineStr"/>
+      <c r="X1114" s="2" t="inlineStr"/>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1115" s="2" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="C1115" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1115" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1115" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1115" s="2" t="n">
+        <v>1852.1</v>
+      </c>
+      <c r="G1115" s="2" t="n">
+        <v>1859</v>
+      </c>
+      <c r="H1115" s="2" t="n">
+        <v>1880</v>
+      </c>
+      <c r="I1115" s="2" t="n">
+        <v>1849.9</v>
+      </c>
+      <c r="J1115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1115" s="2" t="n">
+        <v>1880</v>
+      </c>
+      <c r="L1115" s="2" t="n">
+        <v>1849.9</v>
+      </c>
+      <c r="M1115" s="2" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="N1115" s="4" t="n">
+        <v>1880.05</v>
+      </c>
+      <c r="O1115" s="5" t="n">
+        <v>1864.9</v>
+      </c>
+      <c r="P1115" s="3" t="n">
+        <v>1895.1</v>
+      </c>
+      <c r="Q1115" s="3" t="n">
+        <v>1910.15</v>
+      </c>
+      <c r="R1115" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="S1115" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1115" s="2" t="n">
+        <v>2980</v>
+      </c>
+      <c r="U1115" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1115" s="2" t="inlineStr"/>
+      <c r="W1115" s="2" t="inlineStr"/>
+      <c r="X1115" s="2" t="inlineStr"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1116" s="6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="C1116" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1116" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1116" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1116" s="6" t="n">
+        <v>1180.5</v>
+      </c>
+      <c r="G1116" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="H1116" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="I1116" s="6" t="n">
+        <v>1175</v>
+      </c>
+      <c r="J1116" s="6" t="n">
+        <v>1247.9</v>
+      </c>
+      <c r="K1116" s="6" t="n">
+        <v>1225.2</v>
+      </c>
+      <c r="L1116" s="6" t="n">
+        <v>1175</v>
+      </c>
+      <c r="M1116" s="6" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="N1116" s="8" t="n">
+        <v>1174.95</v>
+      </c>
+      <c r="O1116" s="7" t="n">
+        <v>1200.15</v>
+      </c>
+      <c r="P1116" s="9" t="n">
+        <v>1149.85</v>
+      </c>
+      <c r="Q1116" s="9" t="n">
+        <v>1124.75</v>
+      </c>
+      <c r="R1116" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="S1116" s="6" t="n">
+        <v>2948</v>
+      </c>
+      <c r="T1116" s="6" t="n">
+        <v>2937</v>
+      </c>
+      <c r="U1116" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1116" s="6" t="inlineStr"/>
+      <c r="W1116" s="6" t="inlineStr"/>
+      <c r="X1116" s="6" t="inlineStr"/>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1117" s="6" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="C1117" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1117" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1117" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1117" s="6" t="n">
+        <v>978.2</v>
+      </c>
+      <c r="G1117" s="6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="H1117" s="6" t="n">
+        <v>1015</v>
+      </c>
+      <c r="I1117" s="6" t="n">
+        <v>974</v>
+      </c>
+      <c r="J1117" s="6" t="n">
+        <v>1038.56</v>
+      </c>
+      <c r="K1117" s="6" t="n">
+        <v>1015</v>
+      </c>
+      <c r="L1117" s="6" t="n">
+        <v>974</v>
+      </c>
+      <c r="M1117" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="N1117" s="8" t="n">
+        <v>973.95</v>
+      </c>
+      <c r="O1117" s="7" t="n">
+        <v>994.55</v>
+      </c>
+      <c r="P1117" s="9" t="n">
+        <v>953.45</v>
+      </c>
+      <c r="Q1117" s="9" t="n">
+        <v>932.95</v>
+      </c>
+      <c r="R1117" s="6" t="n">
+        <v>144</v>
+      </c>
+      <c r="S1117" s="6" t="n">
+        <v>2966</v>
+      </c>
+      <c r="T1117" s="6" t="n">
+        <v>2952</v>
+      </c>
+      <c r="U1117" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1117" s="6" t="inlineStr"/>
+      <c r="W1117" s="6" t="inlineStr"/>
+      <c r="X1117" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 24-Sep-2026 09:20 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1117"/>
+  <dimension ref="A1:X1121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -89302,6 +89302,326 @@
       <c r="W1117" s="6" t="inlineStr"/>
       <c r="X1117" s="6" t="inlineStr"/>
     </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1118" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1118" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1118" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1118" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1118" s="2" t="n">
+        <v>1200.1</v>
+      </c>
+      <c r="G1118" s="2" t="n">
+        <v>1210.9</v>
+      </c>
+      <c r="H1118" s="2" t="n">
+        <v>1213.9</v>
+      </c>
+      <c r="I1118" s="2" t="n">
+        <v>1197</v>
+      </c>
+      <c r="J1118" s="2" t="n">
+        <v>1175.52</v>
+      </c>
+      <c r="K1118" s="2" t="n">
+        <v>1213.9</v>
+      </c>
+      <c r="L1118" s="2" t="n">
+        <v>1197</v>
+      </c>
+      <c r="M1118" s="2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="N1118" s="4" t="n">
+        <v>1213.95</v>
+      </c>
+      <c r="O1118" s="5" t="n">
+        <v>1205.4</v>
+      </c>
+      <c r="P1118" s="3" t="n">
+        <v>1222.4</v>
+      </c>
+      <c r="Q1118" s="3" t="n">
+        <v>1230.85</v>
+      </c>
+      <c r="R1118" s="2" t="n">
+        <v>348</v>
+      </c>
+      <c r="S1118" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="T1118" s="2" t="n">
+        <v>2941</v>
+      </c>
+      <c r="U1118" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1118" s="2" t="inlineStr"/>
+      <c r="W1118" s="2" t="inlineStr"/>
+      <c r="X1118" s="2" t="inlineStr"/>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="2" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1119" s="2" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="C1119" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1119" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1119" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1119" s="2" t="n">
+        <v>1715.2</v>
+      </c>
+      <c r="G1119" s="2" t="n">
+        <v>1719.7</v>
+      </c>
+      <c r="H1119" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="I1119" s="2" t="n">
+        <v>1710</v>
+      </c>
+      <c r="J1119" s="2" t="n">
+        <v>1680.68</v>
+      </c>
+      <c r="K1119" s="2" t="n">
+        <v>1740</v>
+      </c>
+      <c r="L1119" s="2" t="n">
+        <v>1710</v>
+      </c>
+      <c r="M1119" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="N1119" s="4" t="n">
+        <v>1740.05</v>
+      </c>
+      <c r="O1119" s="5" t="n">
+        <v>1724.95</v>
+      </c>
+      <c r="P1119" s="3" t="n">
+        <v>1755.05</v>
+      </c>
+      <c r="Q1119" s="3" t="n">
+        <v>1770.05</v>
+      </c>
+      <c r="R1119" s="2" t="n">
+        <v>198</v>
+      </c>
+      <c r="S1119" s="2" t="n">
+        <v>2990</v>
+      </c>
+      <c r="T1119" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1119" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1119" s="2" t="inlineStr"/>
+      <c r="W1119" s="2" t="inlineStr"/>
+      <c r="X1119" s="2" t="inlineStr"/>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1120" s="6" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
+      <c r="C1120" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1120" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1120" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1120" s="6" t="n">
+        <v>918.7</v>
+      </c>
+      <c r="G1120" s="6" t="n">
+        <v>918</v>
+      </c>
+      <c r="H1120" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="I1120" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="J1120" s="6" t="n">
+        <v>969.95</v>
+      </c>
+      <c r="K1120" s="6" t="n">
+        <v>928.9</v>
+      </c>
+      <c r="L1120" s="6" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="M1120" s="6" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="N1120" s="8" t="n">
+        <v>909.25</v>
+      </c>
+      <c r="O1120" s="7" t="n">
+        <v>919.15</v>
+      </c>
+      <c r="P1120" s="9" t="n">
+        <v>899.45</v>
+      </c>
+      <c r="Q1120" s="9" t="n">
+        <v>889.65</v>
+      </c>
+      <c r="R1120" s="6" t="n">
+        <v>303</v>
+      </c>
+      <c r="S1120" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="T1120" s="6" t="n">
+        <v>2969</v>
+      </c>
+      <c r="U1120" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1120" s="6" t="inlineStr"/>
+      <c r="W1120" s="6" t="inlineStr"/>
+      <c r="X1120" s="6" t="inlineStr"/>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="6" t="inlineStr">
+        <is>
+          <t>24-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1121" s="6" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="C1121" s="6" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1121" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1121" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1121" s="6" t="n">
+        <v>234.37</v>
+      </c>
+      <c r="G1121" s="6" t="n">
+        <v>234.5</v>
+      </c>
+      <c r="H1121" s="6" t="n">
+        <v>236.22</v>
+      </c>
+      <c r="I1121" s="6" t="n">
+        <v>233.77</v>
+      </c>
+      <c r="J1121" s="6" t="n">
+        <v>237</v>
+      </c>
+      <c r="K1121" s="6" t="n">
+        <v>236.22</v>
+      </c>
+      <c r="L1121" s="6" t="n">
+        <v>233.77</v>
+      </c>
+      <c r="M1121" s="6" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="N1121" s="8" t="n">
+        <v>233.72</v>
+      </c>
+      <c r="O1121" s="7" t="n">
+        <v>235.05</v>
+      </c>
+      <c r="P1121" s="9" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="Q1121" s="9" t="n">
+        <v>231.27</v>
+      </c>
+      <c r="R1121" s="6" t="n">
+        <v>2139</v>
+      </c>
+      <c r="S1121" s="6" t="n">
+        <v>2845</v>
+      </c>
+      <c r="T1121" s="6" t="n">
+        <v>2610</v>
+      </c>
+      <c r="U1121" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1121" s="6" t="inlineStr"/>
+      <c r="W1121" s="6" t="inlineStr"/>
+      <c r="X1121" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 25-Sep-2026 08:56 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1121"/>
+  <dimension ref="A1:X1125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -89622,6 +89622,326 @@
       <c r="W1121" s="6" t="inlineStr"/>
       <c r="X1121" s="6" t="inlineStr"/>
     </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1122" s="2" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="C1122" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1122" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1122" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1122" s="2" t="n">
+        <v>4950.5</v>
+      </c>
+      <c r="G1122" s="2" t="n">
+        <v>4911.5</v>
+      </c>
+      <c r="H1122" s="2" t="n">
+        <v>4982</v>
+      </c>
+      <c r="I1122" s="2" t="n">
+        <v>4906.5</v>
+      </c>
+      <c r="J1122" s="2" t="n">
+        <v>4921.02</v>
+      </c>
+      <c r="K1122" s="2" t="n">
+        <v>4982</v>
+      </c>
+      <c r="L1122" s="2" t="n">
+        <v>4906.5</v>
+      </c>
+      <c r="M1122" s="2" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="N1122" s="4" t="n">
+        <v>4982.05</v>
+      </c>
+      <c r="O1122" s="5" t="n">
+        <v>4944.2</v>
+      </c>
+      <c r="P1122" s="3" t="n">
+        <v>5019.8</v>
+      </c>
+      <c r="Q1122" s="3" t="n">
+        <v>5057.55</v>
+      </c>
+      <c r="R1122" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="S1122" s="2" t="n">
+        <v>2952</v>
+      </c>
+      <c r="T1122" s="2" t="n">
+        <v>2944</v>
+      </c>
+      <c r="U1122" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1122" s="2" t="inlineStr"/>
+      <c r="W1122" s="2" t="inlineStr"/>
+      <c r="X1122" s="2" t="inlineStr"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1123" s="2" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="C1123" s="2" t="inlineStr">
+        <is>
+          <t>BANKING</t>
+        </is>
+      </c>
+      <c r="D1123" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1123" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1123" s="2" t="n">
+        <v>1324.2</v>
+      </c>
+      <c r="G1123" s="2" t="n">
+        <v>1332.9</v>
+      </c>
+      <c r="H1123" s="2" t="n">
+        <v>1340.8</v>
+      </c>
+      <c r="I1123" s="2" t="n">
+        <v>1323.1</v>
+      </c>
+      <c r="J1123" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1123" s="2" t="n">
+        <v>1340.8</v>
+      </c>
+      <c r="L1123" s="2" t="n">
+        <v>1323.1</v>
+      </c>
+      <c r="M1123" s="2" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="N1123" s="4" t="n">
+        <v>1340.85</v>
+      </c>
+      <c r="O1123" s="5" t="n">
+        <v>1331.9</v>
+      </c>
+      <c r="P1123" s="3" t="n">
+        <v>1349.7</v>
+      </c>
+      <c r="Q1123" s="3" t="n">
+        <v>1358.55</v>
+      </c>
+      <c r="R1123" s="2" t="n">
+        <v>333</v>
+      </c>
+      <c r="S1123" s="2" t="n">
+        <v>2980</v>
+      </c>
+      <c r="T1123" s="2" t="n">
+        <v>2947</v>
+      </c>
+      <c r="U1123" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1123" s="2" t="inlineStr"/>
+      <c r="W1123" s="2" t="inlineStr"/>
+      <c r="X1123" s="2" t="inlineStr"/>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1124" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1124" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1124" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1124" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1124" s="6" t="n">
+        <v>1654.7</v>
+      </c>
+      <c r="G1124" s="6" t="n">
+        <v>1678.1</v>
+      </c>
+      <c r="H1124" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="I1124" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="J1124" s="6" t="n">
+        <v>1780.94</v>
+      </c>
+      <c r="K1124" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="L1124" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="M1124" s="6" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="N1124" s="8" t="n">
+        <v>1637.55</v>
+      </c>
+      <c r="O1124" s="7" t="n">
+        <v>1659.8</v>
+      </c>
+      <c r="P1124" s="9" t="n">
+        <v>1615.4</v>
+      </c>
+      <c r="Q1124" s="9" t="n">
+        <v>1593.25</v>
+      </c>
+      <c r="R1124" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1124" s="6" t="n">
+        <v>2937</v>
+      </c>
+      <c r="T1124" s="6" t="n">
+        <v>2924</v>
+      </c>
+      <c r="U1124" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1124" s="6" t="inlineStr"/>
+      <c r="W1124" s="6" t="inlineStr"/>
+      <c r="X1124" s="6" t="inlineStr"/>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1125" s="6" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="C1125" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1125" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1125" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1125" s="6" t="n">
+        <v>337.75</v>
+      </c>
+      <c r="G1125" s="6" t="n">
+        <v>340</v>
+      </c>
+      <c r="H1125" s="6" t="n">
+        <v>340.05</v>
+      </c>
+      <c r="I1125" s="6" t="n">
+        <v>336.3</v>
+      </c>
+      <c r="J1125" s="6" t="n">
+        <v>347.34</v>
+      </c>
+      <c r="K1125" s="6" t="n">
+        <v>340.05</v>
+      </c>
+      <c r="L1125" s="6" t="n">
+        <v>336.3</v>
+      </c>
+      <c r="M1125" s="6" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="N1125" s="8" t="n">
+        <v>336.25</v>
+      </c>
+      <c r="O1125" s="7" t="n">
+        <v>338.23</v>
+      </c>
+      <c r="P1125" s="9" t="n">
+        <v>334.38</v>
+      </c>
+      <c r="Q1125" s="9" t="n">
+        <v>332.5</v>
+      </c>
+      <c r="R1125" s="6" t="n">
+        <v>1486</v>
+      </c>
+      <c r="S1125" s="6" t="n">
+        <v>2942</v>
+      </c>
+      <c r="T1125" s="6" t="n">
+        <v>2779</v>
+      </c>
+      <c r="U1125" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1125" s="6" t="inlineStr"/>
+      <c r="W1125" s="6" t="inlineStr"/>
+      <c r="X1125" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 25-Sep-2026 09:03 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1125"/>
+  <dimension ref="A1:X1129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -89942,6 +89942,326 @@
       <c r="W1125" s="6" t="inlineStr"/>
       <c r="X1125" s="6" t="inlineStr"/>
     </row>
+    <row r="1126">
+      <c r="A1126" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1126" s="2" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C1126" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1126" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1126" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1126" s="2" t="n">
+        <v>37825</v>
+      </c>
+      <c r="G1126" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="H1126" s="2" t="n">
+        <v>37845</v>
+      </c>
+      <c r="I1126" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="J1126" s="2" t="n">
+        <v>35924.49</v>
+      </c>
+      <c r="K1126" s="2" t="n">
+        <v>37845</v>
+      </c>
+      <c r="L1126" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="M1126" s="2" t="n">
+        <v>495</v>
+      </c>
+      <c r="N1126" s="4" t="n">
+        <v>37845.05</v>
+      </c>
+      <c r="O1126" s="5" t="n">
+        <v>37597.45</v>
+      </c>
+      <c r="P1126" s="3" t="n">
+        <v>38092.55</v>
+      </c>
+      <c r="Q1126" s="3" t="n">
+        <v>38340.05</v>
+      </c>
+      <c r="R1126" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="S1126" s="2" t="n">
+        <v>2971</v>
+      </c>
+      <c r="T1126" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1126" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1126" s="2" t="inlineStr"/>
+      <c r="W1126" s="2" t="inlineStr"/>
+      <c r="X1126" s="2" t="inlineStr"/>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1127" s="2" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="C1127" s="2" t="inlineStr">
+        <is>
+          <t>REALTY</t>
+        </is>
+      </c>
+      <c r="D1127" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1127" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1127" s="2" t="n">
+        <v>678.75</v>
+      </c>
+      <c r="G1127" s="2" t="n">
+        <v>671.2</v>
+      </c>
+      <c r="H1127" s="2" t="n">
+        <v>681.9</v>
+      </c>
+      <c r="I1127" s="2" t="n">
+        <v>670.6</v>
+      </c>
+      <c r="J1127" s="2" t="n">
+        <v>661.49</v>
+      </c>
+      <c r="K1127" s="2" t="n">
+        <v>681.9</v>
+      </c>
+      <c r="L1127" s="2" t="n">
+        <v>670.6</v>
+      </c>
+      <c r="M1127" s="2" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="N1127" s="4" t="n">
+        <v>681.95</v>
+      </c>
+      <c r="O1127" s="5" t="n">
+        <v>676.2</v>
+      </c>
+      <c r="P1127" s="3" t="n">
+        <v>687.6</v>
+      </c>
+      <c r="Q1127" s="3" t="n">
+        <v>693.25</v>
+      </c>
+      <c r="R1127" s="2" t="n">
+        <v>519</v>
+      </c>
+      <c r="S1127" s="2" t="n">
+        <v>2984</v>
+      </c>
+      <c r="T1127" s="2" t="n">
+        <v>2932</v>
+      </c>
+      <c r="U1127" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1127" s="2" t="inlineStr"/>
+      <c r="W1127" s="2" t="inlineStr"/>
+      <c r="X1127" s="2" t="inlineStr"/>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1128" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1128" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1128" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1128" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1128" s="6" t="n">
+        <v>1656.5</v>
+      </c>
+      <c r="G1128" s="6" t="n">
+        <v>1678.1</v>
+      </c>
+      <c r="H1128" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="I1128" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="J1128" s="6" t="n">
+        <v>1780.59</v>
+      </c>
+      <c r="K1128" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="L1128" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="M1128" s="6" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="N1128" s="8" t="n">
+        <v>1637.55</v>
+      </c>
+      <c r="O1128" s="7" t="n">
+        <v>1659.8</v>
+      </c>
+      <c r="P1128" s="9" t="n">
+        <v>1615.4</v>
+      </c>
+      <c r="Q1128" s="9" t="n">
+        <v>1593.25</v>
+      </c>
+      <c r="R1128" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1128" s="6" t="n">
+        <v>2937</v>
+      </c>
+      <c r="T1128" s="6" t="n">
+        <v>2924</v>
+      </c>
+      <c r="U1128" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1128" s="6" t="inlineStr"/>
+      <c r="W1128" s="6" t="inlineStr"/>
+      <c r="X1128" s="6" t="inlineStr"/>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1129" s="6" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1129" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1129" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1129" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1129" s="6" t="n">
+        <v>388.25</v>
+      </c>
+      <c r="G1129" s="6" t="n">
+        <v>390.9</v>
+      </c>
+      <c r="H1129" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="I1129" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="J1129" s="6" t="n">
+        <v>397.44</v>
+      </c>
+      <c r="K1129" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="L1129" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="M1129" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N1129" s="8" t="n">
+        <v>384.75</v>
+      </c>
+      <c r="O1129" s="7" t="n">
+        <v>388.55</v>
+      </c>
+      <c r="P1129" s="9" t="n">
+        <v>381.05</v>
+      </c>
+      <c r="Q1129" s="9" t="n">
+        <v>377.35</v>
+      </c>
+      <c r="R1129" s="6" t="n">
+        <v>789</v>
+      </c>
+      <c r="S1129" s="6" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1129" s="6" t="n">
+        <v>2919</v>
+      </c>
+      <c r="U1129" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1129" s="6" t="inlineStr"/>
+      <c r="W1129" s="6" t="inlineStr"/>
+      <c r="X1129" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 25-Sep-2026 09:31 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1129"/>
+  <dimension ref="A1:X1133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -90262,6 +90262,326 @@
       <c r="W1129" s="6" t="inlineStr"/>
       <c r="X1129" s="6" t="inlineStr"/>
     </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1130" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C1130" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1130" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1130" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1130" s="2" t="n">
+        <v>1789.8</v>
+      </c>
+      <c r="G1130" s="2" t="n">
+        <v>1791.8</v>
+      </c>
+      <c r="H1130" s="2" t="n">
+        <v>1800.6</v>
+      </c>
+      <c r="I1130" s="2" t="n">
+        <v>1775</v>
+      </c>
+      <c r="J1130" s="2" t="n">
+        <v>1716.06</v>
+      </c>
+      <c r="K1130" s="2" t="n">
+        <v>1800.6</v>
+      </c>
+      <c r="L1130" s="2" t="n">
+        <v>1775</v>
+      </c>
+      <c r="M1130" s="2" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="N1130" s="4" t="n">
+        <v>1800.65</v>
+      </c>
+      <c r="O1130" s="5" t="n">
+        <v>1787.75</v>
+      </c>
+      <c r="P1130" s="3" t="n">
+        <v>1813.45</v>
+      </c>
+      <c r="Q1130" s="3" t="n">
+        <v>1826.25</v>
+      </c>
+      <c r="R1130" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="S1130" s="2" t="n">
+        <v>2980</v>
+      </c>
+      <c r="T1130" s="2" t="n">
+        <v>2957</v>
+      </c>
+      <c r="U1130" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1130" s="2" t="inlineStr"/>
+      <c r="W1130" s="2" t="inlineStr"/>
+      <c r="X1130" s="2" t="inlineStr"/>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1131" s="2" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="C1131" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1131" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1131" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1131" s="2" t="n">
+        <v>5374</v>
+      </c>
+      <c r="G1131" s="2" t="n">
+        <v>5340</v>
+      </c>
+      <c r="H1131" s="2" t="n">
+        <v>5397</v>
+      </c>
+      <c r="I1131" s="2" t="n">
+        <v>5304</v>
+      </c>
+      <c r="J1131" s="2" t="n">
+        <v>5350.03</v>
+      </c>
+      <c r="K1131" s="2" t="n">
+        <v>5397</v>
+      </c>
+      <c r="L1131" s="2" t="n">
+        <v>5304</v>
+      </c>
+      <c r="M1131" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="N1131" s="4" t="n">
+        <v>5397.05</v>
+      </c>
+      <c r="O1131" s="5" t="n">
+        <v>5350.45</v>
+      </c>
+      <c r="P1131" s="3" t="n">
+        <v>5443.55</v>
+      </c>
+      <c r="Q1131" s="3" t="n">
+        <v>5490.05</v>
+      </c>
+      <c r="R1131" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="S1131" s="2" t="n">
+        <v>2936</v>
+      </c>
+      <c r="T1131" s="2" t="n">
+        <v>2930</v>
+      </c>
+      <c r="U1131" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1131" s="2" t="inlineStr"/>
+      <c r="W1131" s="2" t="inlineStr"/>
+      <c r="X1131" s="2" t="inlineStr"/>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1132" s="6" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1132" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1132" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1132" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1132" s="6" t="n">
+        <v>388.15</v>
+      </c>
+      <c r="G1132" s="6" t="n">
+        <v>390.9</v>
+      </c>
+      <c r="H1132" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="I1132" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="J1132" s="6" t="n">
+        <v>397.41</v>
+      </c>
+      <c r="K1132" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="L1132" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="M1132" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N1132" s="8" t="n">
+        <v>384.75</v>
+      </c>
+      <c r="O1132" s="7" t="n">
+        <v>388.55</v>
+      </c>
+      <c r="P1132" s="9" t="n">
+        <v>381.05</v>
+      </c>
+      <c r="Q1132" s="9" t="n">
+        <v>377.35</v>
+      </c>
+      <c r="R1132" s="6" t="n">
+        <v>789</v>
+      </c>
+      <c r="S1132" s="6" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1132" s="6" t="n">
+        <v>2919</v>
+      </c>
+      <c r="U1132" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1132" s="6" t="inlineStr"/>
+      <c r="W1132" s="6" t="inlineStr"/>
+      <c r="X1132" s="6" t="inlineStr"/>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1133" s="6" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="C1133" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1133" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1133" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1133" s="6" t="n">
+        <v>990.4</v>
+      </c>
+      <c r="G1133" s="6" t="n">
+        <v>990</v>
+      </c>
+      <c r="H1133" s="6" t="n">
+        <v>1002</v>
+      </c>
+      <c r="I1133" s="6" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="J1133" s="6" t="n">
+        <v>1027.09</v>
+      </c>
+      <c r="K1133" s="6" t="n">
+        <v>1002</v>
+      </c>
+      <c r="L1133" s="6" t="n">
+        <v>986.4</v>
+      </c>
+      <c r="M1133" s="6" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="N1133" s="8" t="n">
+        <v>986.35</v>
+      </c>
+      <c r="O1133" s="7" t="n">
+        <v>994.25</v>
+      </c>
+      <c r="P1133" s="9" t="n">
+        <v>978.55</v>
+      </c>
+      <c r="Q1133" s="9" t="n">
+        <v>970.75</v>
+      </c>
+      <c r="R1133" s="6" t="n">
+        <v>378</v>
+      </c>
+      <c r="S1133" s="6" t="n">
+        <v>2986</v>
+      </c>
+      <c r="T1133" s="6" t="n">
+        <v>2948</v>
+      </c>
+      <c r="U1133" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1133" s="6" t="inlineStr"/>
+      <c r="W1133" s="6" t="inlineStr"/>
+      <c r="X1133" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 25-Sep-2026 09:38 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1133"/>
+  <dimension ref="A1:X1137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -90582,6 +90582,326 @@
       <c r="W1133" s="6" t="inlineStr"/>
       <c r="X1133" s="6" t="inlineStr"/>
     </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1134" s="2" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="C1134" s="2" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="D1134" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1134" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1134" s="2" t="n">
+        <v>4982</v>
+      </c>
+      <c r="G1134" s="2" t="n">
+        <v>4911.5</v>
+      </c>
+      <c r="H1134" s="2" t="n">
+        <v>4990.5</v>
+      </c>
+      <c r="I1134" s="2" t="n">
+        <v>4906.5</v>
+      </c>
+      <c r="J1134" s="2" t="n">
+        <v>4922.29</v>
+      </c>
+      <c r="K1134" s="2" t="n">
+        <v>4990.5</v>
+      </c>
+      <c r="L1134" s="2" t="n">
+        <v>4906.5</v>
+      </c>
+      <c r="M1134" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="N1134" s="4" t="n">
+        <v>4990.55</v>
+      </c>
+      <c r="O1134" s="5" t="n">
+        <v>4948.45</v>
+      </c>
+      <c r="P1134" s="3" t="n">
+        <v>5032.55</v>
+      </c>
+      <c r="Q1134" s="3" t="n">
+        <v>5074.55</v>
+      </c>
+      <c r="R1134" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="S1134" s="2" t="n">
+        <v>2905</v>
+      </c>
+      <c r="T1134" s="2" t="n">
+        <v>2898</v>
+      </c>
+      <c r="U1134" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1134" s="2" t="inlineStr"/>
+      <c r="W1134" s="2" t="inlineStr"/>
+      <c r="X1134" s="2" t="inlineStr"/>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="2" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1135" s="2" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C1135" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1135" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1135" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1135" s="2" t="n">
+        <v>37685</v>
+      </c>
+      <c r="G1135" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="H1135" s="2" t="n">
+        <v>37845</v>
+      </c>
+      <c r="I1135" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="J1135" s="2" t="n">
+        <v>35930.49</v>
+      </c>
+      <c r="K1135" s="2" t="n">
+        <v>37845</v>
+      </c>
+      <c r="L1135" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="M1135" s="2" t="n">
+        <v>495</v>
+      </c>
+      <c r="N1135" s="4" t="n">
+        <v>37845.05</v>
+      </c>
+      <c r="O1135" s="5" t="n">
+        <v>37597.45</v>
+      </c>
+      <c r="P1135" s="3" t="n">
+        <v>38092.55</v>
+      </c>
+      <c r="Q1135" s="3" t="n">
+        <v>38340.05</v>
+      </c>
+      <c r="R1135" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="S1135" s="2" t="n">
+        <v>2971</v>
+      </c>
+      <c r="T1135" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1135" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1135" s="2" t="inlineStr"/>
+      <c r="W1135" s="2" t="inlineStr"/>
+      <c r="X1135" s="2" t="inlineStr"/>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1136" s="6" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="C1136" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1136" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1136" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1136" s="6" t="n">
+        <v>1651.6</v>
+      </c>
+      <c r="G1136" s="6" t="n">
+        <v>1678.1</v>
+      </c>
+      <c r="H1136" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="I1136" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="J1136" s="6" t="n">
+        <v>1778.92</v>
+      </c>
+      <c r="K1136" s="6" t="n">
+        <v>1681.9</v>
+      </c>
+      <c r="L1136" s="6" t="n">
+        <v>1637.6</v>
+      </c>
+      <c r="M1136" s="6" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="N1136" s="8" t="n">
+        <v>1637.55</v>
+      </c>
+      <c r="O1136" s="7" t="n">
+        <v>1659.8</v>
+      </c>
+      <c r="P1136" s="9" t="n">
+        <v>1615.4</v>
+      </c>
+      <c r="Q1136" s="9" t="n">
+        <v>1593.25</v>
+      </c>
+      <c r="R1136" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="S1136" s="6" t="n">
+        <v>2937</v>
+      </c>
+      <c r="T1136" s="6" t="n">
+        <v>2924</v>
+      </c>
+      <c r="U1136" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1136" s="6" t="inlineStr"/>
+      <c r="W1136" s="6" t="inlineStr"/>
+      <c r="X1136" s="6" t="inlineStr"/>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="6" t="inlineStr">
+        <is>
+          <t>25-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1137" s="6" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1137" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1137" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1137" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1137" s="6" t="n">
+        <v>388.1</v>
+      </c>
+      <c r="G1137" s="6" t="n">
+        <v>390.9</v>
+      </c>
+      <c r="H1137" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="I1137" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="J1137" s="6" t="n">
+        <v>397.4</v>
+      </c>
+      <c r="K1137" s="6" t="n">
+        <v>392.2</v>
+      </c>
+      <c r="L1137" s="6" t="n">
+        <v>384.8</v>
+      </c>
+      <c r="M1137" s="6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N1137" s="8" t="n">
+        <v>384.75</v>
+      </c>
+      <c r="O1137" s="7" t="n">
+        <v>388.55</v>
+      </c>
+      <c r="P1137" s="9" t="n">
+        <v>381.05</v>
+      </c>
+      <c r="Q1137" s="9" t="n">
+        <v>377.35</v>
+      </c>
+      <c r="R1137" s="6" t="n">
+        <v>789</v>
+      </c>
+      <c r="S1137" s="6" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1137" s="6" t="n">
+        <v>2919</v>
+      </c>
+      <c r="U1137" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1137" s="6" t="inlineStr"/>
+      <c r="W1137" s="6" t="inlineStr"/>
+      <c r="X1137" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 28-Sep-2026 09:52 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1137"/>
+  <dimension ref="A1:X1141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -90902,6 +90902,326 @@
       <c r="W1137" s="6" t="inlineStr"/>
       <c r="X1137" s="6" t="inlineStr"/>
     </row>
+    <row r="1138">
+      <c r="A1138" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1138" s="2" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C1138" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1138" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1138" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1138" s="2" t="n">
+        <v>37580</v>
+      </c>
+      <c r="G1138" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="H1138" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="I1138" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="J1138" s="2" t="n">
+        <v>35998.51</v>
+      </c>
+      <c r="K1138" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="L1138" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="M1138" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="N1138" s="4" t="n">
+        <v>37680.05</v>
+      </c>
+      <c r="O1138" s="5" t="n">
+        <v>37479.95</v>
+      </c>
+      <c r="P1138" s="3" t="n">
+        <v>37880.05</v>
+      </c>
+      <c r="Q1138" s="3" t="n">
+        <v>38080.05</v>
+      </c>
+      <c r="R1138" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="S1138" s="2" t="n">
+        <v>2401</v>
+      </c>
+      <c r="T1138" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="U1138" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1138" s="2" t="inlineStr"/>
+      <c r="W1138" s="2" t="inlineStr"/>
+      <c r="X1138" s="2" t="inlineStr"/>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1139" s="2" t="inlineStr">
+        <is>
+          <t>ZOMATO</t>
+        </is>
+      </c>
+      <c r="C1139" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1139" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1139" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1139" s="2" t="n">
+        <v>331.25</v>
+      </c>
+      <c r="G1139" s="2" t="n">
+        <v>335.05</v>
+      </c>
+      <c r="H1139" s="2" t="n">
+        <v>335.1</v>
+      </c>
+      <c r="I1139" s="2" t="n">
+        <v>328.45</v>
+      </c>
+      <c r="J1139" s="2" t="n">
+        <v>326.74</v>
+      </c>
+      <c r="K1139" s="2" t="n">
+        <v>335.1</v>
+      </c>
+      <c r="L1139" s="2" t="n">
+        <v>328.45</v>
+      </c>
+      <c r="M1139" s="2" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="N1139" s="4" t="n">
+        <v>335.15</v>
+      </c>
+      <c r="O1139" s="5" t="n">
+        <v>331.72</v>
+      </c>
+      <c r="P1139" s="3" t="n">
+        <v>338.47</v>
+      </c>
+      <c r="Q1139" s="3" t="n">
+        <v>341.8</v>
+      </c>
+      <c r="R1139" s="2" t="n">
+        <v>873</v>
+      </c>
+      <c r="S1139" s="2" t="n">
+        <v>2994</v>
+      </c>
+      <c r="T1139" s="2" t="n">
+        <v>2898</v>
+      </c>
+      <c r="U1139" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1139" s="2" t="inlineStr"/>
+      <c r="W1139" s="2" t="inlineStr"/>
+      <c r="X1139" s="2" t="inlineStr"/>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1140" s="6" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="C1140" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1140" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1140" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1140" s="6" t="n">
+        <v>530</v>
+      </c>
+      <c r="G1140" s="6" t="n">
+        <v>531</v>
+      </c>
+      <c r="H1140" s="6" t="n">
+        <v>534.5</v>
+      </c>
+      <c r="I1140" s="6" t="n">
+        <v>525.9</v>
+      </c>
+      <c r="J1140" s="6" t="n">
+        <v>534.6799999999999</v>
+      </c>
+      <c r="K1140" s="6" t="n">
+        <v>534.5</v>
+      </c>
+      <c r="L1140" s="6" t="n">
+        <v>525.9</v>
+      </c>
+      <c r="M1140" s="6" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="N1140" s="8" t="n">
+        <v>525.85</v>
+      </c>
+      <c r="O1140" s="7" t="n">
+        <v>530.25</v>
+      </c>
+      <c r="P1140" s="9" t="n">
+        <v>521.55</v>
+      </c>
+      <c r="Q1140" s="9" t="n">
+        <v>517.25</v>
+      </c>
+      <c r="R1140" s="6" t="n">
+        <v>681</v>
+      </c>
+      <c r="S1140" s="6" t="n">
+        <v>2996</v>
+      </c>
+      <c r="T1140" s="6" t="n">
+        <v>2928</v>
+      </c>
+      <c r="U1140" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1140" s="6" t="inlineStr"/>
+      <c r="W1140" s="6" t="inlineStr"/>
+      <c r="X1140" s="6" t="inlineStr"/>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1141" s="6" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="C1141" s="6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="D1141" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1141" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1141" s="6" t="n">
+        <v>384</v>
+      </c>
+      <c r="G1141" s="6" t="n">
+        <v>388.05</v>
+      </c>
+      <c r="H1141" s="6" t="n">
+        <v>388.85</v>
+      </c>
+      <c r="I1141" s="6" t="n">
+        <v>380.8</v>
+      </c>
+      <c r="J1141" s="6" t="n">
+        <v>396.74</v>
+      </c>
+      <c r="K1141" s="6" t="n">
+        <v>388.85</v>
+      </c>
+      <c r="L1141" s="6" t="n">
+        <v>380.8</v>
+      </c>
+      <c r="M1141" s="6" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="N1141" s="8" t="n">
+        <v>380.75</v>
+      </c>
+      <c r="O1141" s="7" t="n">
+        <v>384.88</v>
+      </c>
+      <c r="P1141" s="9" t="n">
+        <v>376.73</v>
+      </c>
+      <c r="Q1141" s="9" t="n">
+        <v>372.7</v>
+      </c>
+      <c r="R1141" s="6" t="n">
+        <v>726</v>
+      </c>
+      <c r="S1141" s="6" t="n">
+        <v>2998</v>
+      </c>
+      <c r="T1141" s="6" t="n">
+        <v>2919</v>
+      </c>
+      <c r="U1141" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1141" s="6" t="inlineStr"/>
+      <c r="W1141" s="6" t="inlineStr"/>
+      <c r="X1141" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 28-Sep-2026 10:05 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1141"/>
+  <dimension ref="A1:X1145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -91222,6 +91222,326 @@
       <c r="W1141" s="6" t="inlineStr"/>
       <c r="X1141" s="6" t="inlineStr"/>
     </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1142" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1142" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1142" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1142" s="2" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1142" s="2" t="n">
+        <v>1221</v>
+      </c>
+      <c r="G1142" s="2" t="n">
+        <v>1211.6</v>
+      </c>
+      <c r="H1142" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="I1142" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="J1142" s="2" t="n">
+        <v>1181.29</v>
+      </c>
+      <c r="K1142" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="L1142" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="M1142" s="2" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="N1142" s="4" t="n">
+        <v>1229.85</v>
+      </c>
+      <c r="O1142" s="5" t="n">
+        <v>1216.85</v>
+      </c>
+      <c r="P1142" s="3" t="n">
+        <v>1242.75</v>
+      </c>
+      <c r="Q1142" s="3" t="n">
+        <v>1255.65</v>
+      </c>
+      <c r="R1142" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S1142" s="2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="T1142" s="2" t="n">
+        <v>2941</v>
+      </c>
+      <c r="U1142" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1142" s="2" t="inlineStr"/>
+      <c r="W1142" s="2" t="inlineStr"/>
+      <c r="X1142" s="2" t="inlineStr"/>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1143" s="2" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C1143" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1143" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1143" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1143" s="2" t="n">
+        <v>37500</v>
+      </c>
+      <c r="G1143" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="H1143" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="I1143" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="J1143" s="2" t="n">
+        <v>35998.99</v>
+      </c>
+      <c r="K1143" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="L1143" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="M1143" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="N1143" s="4" t="n">
+        <v>37680.05</v>
+      </c>
+      <c r="O1143" s="5" t="n">
+        <v>37479.95</v>
+      </c>
+      <c r="P1143" s="3" t="n">
+        <v>37880.05</v>
+      </c>
+      <c r="Q1143" s="3" t="n">
+        <v>38080.05</v>
+      </c>
+      <c r="R1143" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="S1143" s="2" t="n">
+        <v>2401</v>
+      </c>
+      <c r="T1143" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="U1143" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1143" s="2" t="inlineStr"/>
+      <c r="W1143" s="2" t="inlineStr"/>
+      <c r="X1143" s="2" t="inlineStr"/>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1144" s="6" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="C1144" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1144" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1144" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1144" s="6" t="n">
+        <v>1197.6</v>
+      </c>
+      <c r="G1144" s="6" t="n">
+        <v>1218</v>
+      </c>
+      <c r="H1144" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="I1144" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="J1144" s="6" t="n">
+        <v>1265.61</v>
+      </c>
+      <c r="K1144" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="L1144" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="M1144" s="6" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="N1144" s="8" t="n">
+        <v>1196.95</v>
+      </c>
+      <c r="O1144" s="7" t="n">
+        <v>1208.4</v>
+      </c>
+      <c r="P1144" s="9" t="n">
+        <v>1185.6</v>
+      </c>
+      <c r="Q1144" s="9" t="n">
+        <v>1174.25</v>
+      </c>
+      <c r="R1144" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1144" s="6" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1144" s="6" t="n">
+        <v>2962</v>
+      </c>
+      <c r="U1144" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1144" s="6" t="inlineStr"/>
+      <c r="W1144" s="6" t="inlineStr"/>
+      <c r="X1144" s="6" t="inlineStr"/>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1145" s="6" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="C1145" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1145" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1145" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1145" s="6" t="n">
+        <v>302.25</v>
+      </c>
+      <c r="G1145" s="6" t="n">
+        <v>306.95</v>
+      </c>
+      <c r="H1145" s="6" t="n">
+        <v>308.5</v>
+      </c>
+      <c r="I1145" s="6" t="n">
+        <v>301</v>
+      </c>
+      <c r="J1145" s="6" t="n">
+        <v>311.31</v>
+      </c>
+      <c r="K1145" s="6" t="n">
+        <v>308.5</v>
+      </c>
+      <c r="L1145" s="6" t="n">
+        <v>301</v>
+      </c>
+      <c r="M1145" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="N1145" s="8" t="n">
+        <v>300.95</v>
+      </c>
+      <c r="O1145" s="7" t="n">
+        <v>304.8</v>
+      </c>
+      <c r="P1145" s="9" t="n">
+        <v>297.2</v>
+      </c>
+      <c r="Q1145" s="9" t="n">
+        <v>293.45</v>
+      </c>
+      <c r="R1145" s="6" t="n">
+        <v>777</v>
+      </c>
+      <c r="S1145" s="6" t="n">
+        <v>2991</v>
+      </c>
+      <c r="T1145" s="6" t="n">
+        <v>2914</v>
+      </c>
+      <c r="U1145" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1145" s="6" t="inlineStr"/>
+      <c r="W1145" s="6" t="inlineStr"/>
+      <c r="X1145" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 28-Sep-2026 10:44 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1145"/>
+  <dimension ref="A1:X1149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -91542,6 +91542,326 @@
       <c r="W1145" s="6" t="inlineStr"/>
       <c r="X1145" s="6" t="inlineStr"/>
     </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1146" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1146" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1146" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1146" s="2" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1146" s="2" t="n">
+        <v>1221</v>
+      </c>
+      <c r="G1146" s="2" t="n">
+        <v>1211.6</v>
+      </c>
+      <c r="H1146" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="I1146" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="J1146" s="2" t="n">
+        <v>1181.29</v>
+      </c>
+      <c r="K1146" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="L1146" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="M1146" s="2" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="N1146" s="4" t="n">
+        <v>1229.85</v>
+      </c>
+      <c r="O1146" s="5" t="n">
+        <v>1216.85</v>
+      </c>
+      <c r="P1146" s="3" t="n">
+        <v>1242.75</v>
+      </c>
+      <c r="Q1146" s="3" t="n">
+        <v>1255.65</v>
+      </c>
+      <c r="R1146" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S1146" s="2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="T1146" s="2" t="n">
+        <v>2941</v>
+      </c>
+      <c r="U1146" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1146" s="2" t="inlineStr"/>
+      <c r="W1146" s="2" t="inlineStr"/>
+      <c r="X1146" s="2" t="inlineStr"/>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1147" s="2" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="C1147" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1147" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1147" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1147" s="2" t="n">
+        <v>37500</v>
+      </c>
+      <c r="G1147" s="2" t="n">
+        <v>37350</v>
+      </c>
+      <c r="H1147" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="I1147" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="J1147" s="2" t="n">
+        <v>35998.99</v>
+      </c>
+      <c r="K1147" s="2" t="n">
+        <v>37680</v>
+      </c>
+      <c r="L1147" s="2" t="n">
+        <v>37280</v>
+      </c>
+      <c r="M1147" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="N1147" s="4" t="n">
+        <v>37680.05</v>
+      </c>
+      <c r="O1147" s="5" t="n">
+        <v>37479.95</v>
+      </c>
+      <c r="P1147" s="3" t="n">
+        <v>37880.05</v>
+      </c>
+      <c r="Q1147" s="3" t="n">
+        <v>38080.05</v>
+      </c>
+      <c r="R1147" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="S1147" s="2" t="n">
+        <v>2401</v>
+      </c>
+      <c r="T1147" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="U1147" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1147" s="2" t="inlineStr"/>
+      <c r="W1147" s="2" t="inlineStr"/>
+      <c r="X1147" s="2" t="inlineStr"/>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1148" s="6" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="C1148" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1148" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1148" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1148" s="6" t="n">
+        <v>1197.6</v>
+      </c>
+      <c r="G1148" s="6" t="n">
+        <v>1218</v>
+      </c>
+      <c r="H1148" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="I1148" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="J1148" s="6" t="n">
+        <v>1265.6</v>
+      </c>
+      <c r="K1148" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="L1148" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="M1148" s="6" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="N1148" s="8" t="n">
+        <v>1196.95</v>
+      </c>
+      <c r="O1148" s="7" t="n">
+        <v>1208.4</v>
+      </c>
+      <c r="P1148" s="9" t="n">
+        <v>1185.6</v>
+      </c>
+      <c r="Q1148" s="9" t="n">
+        <v>1174.25</v>
+      </c>
+      <c r="R1148" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1148" s="6" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1148" s="6" t="n">
+        <v>2962</v>
+      </c>
+      <c r="U1148" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1148" s="6" t="inlineStr"/>
+      <c r="W1148" s="6" t="inlineStr"/>
+      <c r="X1148" s="6" t="inlineStr"/>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1149" s="6" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1149" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1149" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1149" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1149" s="6" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1149" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="H1149" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="I1149" s="6" t="n">
+        <v>229.85</v>
+      </c>
+      <c r="J1149" s="6" t="n">
+        <v>235.27</v>
+      </c>
+      <c r="K1149" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="L1149" s="6" t="n">
+        <v>229.85</v>
+      </c>
+      <c r="M1149" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N1149" s="8" t="n">
+        <v>229.8</v>
+      </c>
+      <c r="O1149" s="7" t="n">
+        <v>232.9</v>
+      </c>
+      <c r="P1149" s="9" t="n">
+        <v>226.8</v>
+      </c>
+      <c r="Q1149" s="9" t="n">
+        <v>223.8</v>
+      </c>
+      <c r="R1149" s="6" t="n">
+        <v>966</v>
+      </c>
+      <c r="S1149" s="6" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1149" s="6" t="n">
+        <v>2898</v>
+      </c>
+      <c r="U1149" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1149" s="6" t="inlineStr"/>
+      <c r="W1149" s="6" t="inlineStr"/>
+      <c r="X1149" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 28-Sep-2026 10:54 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1149"/>
+  <dimension ref="A1:X1153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -91862,6 +91862,326 @@
       <c r="W1149" s="6" t="inlineStr"/>
       <c r="X1149" s="6" t="inlineStr"/>
     </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1150" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1150" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1150" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1150" s="2" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1150" s="2" t="n">
+        <v>1221</v>
+      </c>
+      <c r="G1150" s="2" t="n">
+        <v>1211.6</v>
+      </c>
+      <c r="H1150" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="I1150" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="J1150" s="2" t="n">
+        <v>1181.29</v>
+      </c>
+      <c r="K1150" s="2" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="L1150" s="2" t="n">
+        <v>1204</v>
+      </c>
+      <c r="M1150" s="2" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="N1150" s="4" t="n">
+        <v>1229.85</v>
+      </c>
+      <c r="O1150" s="5" t="n">
+        <v>1216.85</v>
+      </c>
+      <c r="P1150" s="3" t="n">
+        <v>1242.75</v>
+      </c>
+      <c r="Q1150" s="3" t="n">
+        <v>1255.65</v>
+      </c>
+      <c r="R1150" s="2" t="n">
+        <v>228</v>
+      </c>
+      <c r="S1150" s="2" t="n">
+        <v>2964</v>
+      </c>
+      <c r="T1150" s="2" t="n">
+        <v>2941</v>
+      </c>
+      <c r="U1150" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1150" s="2" t="inlineStr"/>
+      <c r="W1150" s="2" t="inlineStr"/>
+      <c r="X1150" s="2" t="inlineStr"/>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1151" s="2" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="C1151" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1151" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1151" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1151" s="2" t="n">
+        <v>9550</v>
+      </c>
+      <c r="G1151" s="2" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H1151" s="2" t="n">
+        <v>9655</v>
+      </c>
+      <c r="I1151" s="2" t="n">
+        <v>9473</v>
+      </c>
+      <c r="J1151" s="2" t="n">
+        <v>9360.309999999999</v>
+      </c>
+      <c r="K1151" s="2" t="n">
+        <v>9655</v>
+      </c>
+      <c r="L1151" s="2" t="n">
+        <v>9473</v>
+      </c>
+      <c r="M1151" s="2" t="n">
+        <v>182</v>
+      </c>
+      <c r="N1151" s="4" t="n">
+        <v>9655.049999999999</v>
+      </c>
+      <c r="O1151" s="5" t="n">
+        <v>9563.950000000001</v>
+      </c>
+      <c r="P1151" s="3" t="n">
+        <v>9746.049999999999</v>
+      </c>
+      <c r="Q1151" s="3" t="n">
+        <v>9837.049999999999</v>
+      </c>
+      <c r="R1151" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="S1151" s="2" t="n">
+        <v>2733</v>
+      </c>
+      <c r="T1151" s="2" t="n">
+        <v>2730</v>
+      </c>
+      <c r="U1151" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1151" s="2" t="inlineStr"/>
+      <c r="W1151" s="2" t="inlineStr"/>
+      <c r="X1151" s="2" t="inlineStr"/>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1152" s="6" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="C1152" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1152" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1152" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1152" s="6" t="n">
+        <v>1197.6</v>
+      </c>
+      <c r="G1152" s="6" t="n">
+        <v>1218</v>
+      </c>
+      <c r="H1152" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="I1152" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="J1152" s="6" t="n">
+        <v>1265.6</v>
+      </c>
+      <c r="K1152" s="6" t="n">
+        <v>1219.7</v>
+      </c>
+      <c r="L1152" s="6" t="n">
+        <v>1197</v>
+      </c>
+      <c r="M1152" s="6" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="N1152" s="8" t="n">
+        <v>1196.95</v>
+      </c>
+      <c r="O1152" s="7" t="n">
+        <v>1208.4</v>
+      </c>
+      <c r="P1152" s="9" t="n">
+        <v>1185.6</v>
+      </c>
+      <c r="Q1152" s="9" t="n">
+        <v>1174.25</v>
+      </c>
+      <c r="R1152" s="6" t="n">
+        <v>261</v>
+      </c>
+      <c r="S1152" s="6" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1152" s="6" t="n">
+        <v>2962</v>
+      </c>
+      <c r="U1152" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1152" s="6" t="inlineStr"/>
+      <c r="W1152" s="6" t="inlineStr"/>
+      <c r="X1152" s="6" t="inlineStr"/>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="6" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1153" s="6" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="C1153" s="6" t="inlineStr">
+        <is>
+          <t>ENERGY</t>
+        </is>
+      </c>
+      <c r="D1153" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1153" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1153" s="6" t="n">
+        <v>230</v>
+      </c>
+      <c r="G1153" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="H1153" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="I1153" s="6" t="n">
+        <v>229.85</v>
+      </c>
+      <c r="J1153" s="6" t="n">
+        <v>235.27</v>
+      </c>
+      <c r="K1153" s="6" t="n">
+        <v>235.85</v>
+      </c>
+      <c r="L1153" s="6" t="n">
+        <v>229.85</v>
+      </c>
+      <c r="M1153" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N1153" s="8" t="n">
+        <v>229.8</v>
+      </c>
+      <c r="O1153" s="7" t="n">
+        <v>232.9</v>
+      </c>
+      <c r="P1153" s="9" t="n">
+        <v>226.8</v>
+      </c>
+      <c r="Q1153" s="9" t="n">
+        <v>223.8</v>
+      </c>
+      <c r="R1153" s="6" t="n">
+        <v>966</v>
+      </c>
+      <c r="S1153" s="6" t="n">
+        <v>2995</v>
+      </c>
+      <c r="T1153" s="6" t="n">
+        <v>2898</v>
+      </c>
+      <c r="U1153" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1153" s="6" t="inlineStr"/>
+      <c r="W1153" s="6" t="inlineStr"/>
+      <c r="X1153" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 29-Sep-2026 09:55 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1153"/>
+  <dimension ref="A1:X1157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -92182,6 +92182,326 @@
       <c r="W1153" s="6" t="inlineStr"/>
       <c r="X1153" s="6" t="inlineStr"/>
     </row>
+    <row r="1154">
+      <c r="A1154" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1154" s="2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="C1154" s="2" t="inlineStr">
+        <is>
+          <t>INFRA</t>
+        </is>
+      </c>
+      <c r="D1154" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1154" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1154" s="2" t="n">
+        <v>1768.1</v>
+      </c>
+      <c r="G1154" s="2" t="n">
+        <v>1755.2</v>
+      </c>
+      <c r="H1154" s="2" t="n">
+        <v>1771.4</v>
+      </c>
+      <c r="I1154" s="2" t="n">
+        <v>1738.4</v>
+      </c>
+      <c r="J1154" s="2" t="n">
+        <v>1739.92</v>
+      </c>
+      <c r="K1154" s="2" t="n">
+        <v>1771.4</v>
+      </c>
+      <c r="L1154" s="2" t="n">
+        <v>1738.4</v>
+      </c>
+      <c r="M1154" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="N1154" s="4" t="n">
+        <v>1771.45</v>
+      </c>
+      <c r="O1154" s="5" t="n">
+        <v>1754.85</v>
+      </c>
+      <c r="P1154" s="3" t="n">
+        <v>1787.95</v>
+      </c>
+      <c r="Q1154" s="3" t="n">
+        <v>1804.45</v>
+      </c>
+      <c r="R1154" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="S1154" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1154" s="2" t="n">
+        <v>2970</v>
+      </c>
+      <c r="U1154" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1154" s="2" t="inlineStr"/>
+      <c r="W1154" s="2" t="inlineStr"/>
+      <c r="X1154" s="2" t="inlineStr"/>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1155" s="2" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="C1155" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1155" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1155" s="2" t="inlineStr">
+        <is>
+          <t>3/6</t>
+        </is>
+      </c>
+      <c r="F1155" s="2" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G1155" s="2" t="n">
+        <v>1853.9</v>
+      </c>
+      <c r="H1155" s="2" t="n">
+        <v>1862.3</v>
+      </c>
+      <c r="I1155" s="2" t="n">
+        <v>1836.6</v>
+      </c>
+      <c r="J1155" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1155" s="2" t="n">
+        <v>1862.3</v>
+      </c>
+      <c r="L1155" s="2" t="n">
+        <v>1836.6</v>
+      </c>
+      <c r="M1155" s="2" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="N1155" s="4" t="n">
+        <v>1862.35</v>
+      </c>
+      <c r="O1155" s="5" t="n">
+        <v>1849.4</v>
+      </c>
+      <c r="P1155" s="3" t="n">
+        <v>1875.2</v>
+      </c>
+      <c r="Q1155" s="3" t="n">
+        <v>1888.05</v>
+      </c>
+      <c r="R1155" s="2" t="n">
+        <v>231</v>
+      </c>
+      <c r="S1155" s="2" t="n">
+        <v>2991</v>
+      </c>
+      <c r="T1155" s="2" t="n">
+        <v>2968</v>
+      </c>
+      <c r="U1155" s="2" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1155" s="2" t="inlineStr"/>
+      <c r="W1155" s="2" t="inlineStr"/>
+      <c r="X1155" s="2" t="inlineStr"/>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1156" s="6" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="C1156" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1156" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1156" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1156" s="6" t="n">
+        <v>1228.4</v>
+      </c>
+      <c r="G1156" s="6" t="n">
+        <v>1252.6</v>
+      </c>
+      <c r="H1156" s="6" t="n">
+        <v>1261</v>
+      </c>
+      <c r="I1156" s="6" t="n">
+        <v>1225.5</v>
+      </c>
+      <c r="J1156" s="6" t="n">
+        <v>1269.04</v>
+      </c>
+      <c r="K1156" s="6" t="n">
+        <v>1261</v>
+      </c>
+      <c r="L1156" s="6" t="n">
+        <v>1225.5</v>
+      </c>
+      <c r="M1156" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="N1156" s="8" t="n">
+        <v>1225.45</v>
+      </c>
+      <c r="O1156" s="7" t="n">
+        <v>1243.3</v>
+      </c>
+      <c r="P1156" s="9" t="n">
+        <v>1207.7</v>
+      </c>
+      <c r="Q1156" s="9" t="n">
+        <v>1189.95</v>
+      </c>
+      <c r="R1156" s="6" t="n">
+        <v>168</v>
+      </c>
+      <c r="S1156" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1156" s="6" t="n">
+        <v>2982</v>
+      </c>
+      <c r="U1156" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1156" s="6" t="inlineStr"/>
+      <c r="W1156" s="6" t="inlineStr"/>
+      <c r="X1156" s="6" t="inlineStr"/>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1157" s="6" t="inlineStr">
+        <is>
+          <t>VOLTAS</t>
+        </is>
+      </c>
+      <c r="C1157" s="6" t="inlineStr">
+        <is>
+          <t>CONSUMER</t>
+        </is>
+      </c>
+      <c r="D1157" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1157" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1157" s="6" t="n">
+        <v>1098.1</v>
+      </c>
+      <c r="G1157" s="6" t="n">
+        <v>1135.2</v>
+      </c>
+      <c r="H1157" s="6" t="n">
+        <v>1137.9</v>
+      </c>
+      <c r="I1157" s="6" t="n">
+        <v>1097</v>
+      </c>
+      <c r="J1157" s="6" t="n">
+        <v>1142.7</v>
+      </c>
+      <c r="K1157" s="6" t="n">
+        <v>1137.9</v>
+      </c>
+      <c r="L1157" s="6" t="n">
+        <v>1097</v>
+      </c>
+      <c r="M1157" s="6" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="N1157" s="8" t="n">
+        <v>1096.95</v>
+      </c>
+      <c r="O1157" s="7" t="n">
+        <v>1117.5</v>
+      </c>
+      <c r="P1157" s="9" t="n">
+        <v>1076.5</v>
+      </c>
+      <c r="Q1157" s="9" t="n">
+        <v>1056.05</v>
+      </c>
+      <c r="R1157" s="6" t="n">
+        <v>144</v>
+      </c>
+      <c r="S1157" s="6" t="n">
+        <v>2959</v>
+      </c>
+      <c r="T1157" s="6" t="n">
+        <v>2945</v>
+      </c>
+      <c r="U1157" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH</t>
+        </is>
+      </c>
+      <c r="V1157" s="6" t="inlineStr"/>
+      <c r="W1157" s="6" t="inlineStr"/>
+      <c r="X1157" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 29-Sep-2026 10:03 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1157"/>
+  <dimension ref="A1:X1161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -92502,6 +92502,326 @@
       <c r="W1157" s="6" t="inlineStr"/>
       <c r="X1157" s="6" t="inlineStr"/>
     </row>
+    <row r="1158">
+      <c r="A1158" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1158" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1158" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1158" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1158" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1158" s="2" t="n">
+        <v>1251.9</v>
+      </c>
+      <c r="G1158" s="2" t="n">
+        <v>1243.2</v>
+      </c>
+      <c r="H1158" s="2" t="n">
+        <v>1252.8</v>
+      </c>
+      <c r="I1158" s="2" t="n">
+        <v>1229</v>
+      </c>
+      <c r="J1158" s="2" t="n">
+        <v>1192.58</v>
+      </c>
+      <c r="K1158" s="2" t="n">
+        <v>1252.8</v>
+      </c>
+      <c r="L1158" s="2" t="n">
+        <v>1229</v>
+      </c>
+      <c r="M1158" s="2" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="N1158" s="4" t="n">
+        <v>1252.85</v>
+      </c>
+      <c r="O1158" s="5" t="n">
+        <v>1240.85</v>
+      </c>
+      <c r="P1158" s="3" t="n">
+        <v>1264.75</v>
+      </c>
+      <c r="Q1158" s="3" t="n">
+        <v>1276.65</v>
+      </c>
+      <c r="R1158" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="S1158" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1158" s="2" t="n">
+        <v>2963</v>
+      </c>
+      <c r="U1158" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1158" s="2" t="inlineStr"/>
+      <c r="W1158" s="2" t="inlineStr"/>
+      <c r="X1158" s="2" t="inlineStr"/>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1159" s="2" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1159" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1159" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1159" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1159" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="G1159" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="H1159" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="I1159" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="J1159" s="2" t="n">
+        <v>421.07</v>
+      </c>
+      <c r="K1159" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="L1159" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="M1159" s="2" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="N1159" s="4" t="n">
+        <v>426.05</v>
+      </c>
+      <c r="O1159" s="5" t="n">
+        <v>423.22</v>
+      </c>
+      <c r="P1159" s="3" t="n">
+        <v>428.78</v>
+      </c>
+      <c r="Q1159" s="3" t="n">
+        <v>431.5</v>
+      </c>
+      <c r="R1159" s="2" t="n">
+        <v>1059</v>
+      </c>
+      <c r="S1159" s="2" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T1159" s="2" t="n">
+        <v>2891</v>
+      </c>
+      <c r="U1159" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1159" s="2" t="inlineStr"/>
+      <c r="W1159" s="2" t="inlineStr"/>
+      <c r="X1159" s="2" t="inlineStr"/>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1160" s="6" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="C1160" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1160" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1160" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1160" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="G1160" s="6" t="n">
+        <v>1542.3</v>
+      </c>
+      <c r="H1160" s="6" t="n">
+        <v>1557.5</v>
+      </c>
+      <c r="I1160" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="J1160" s="6" t="n">
+        <v>1562.43</v>
+      </c>
+      <c r="K1160" s="6" t="n">
+        <v>1557.5</v>
+      </c>
+      <c r="L1160" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="M1160" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="N1160" s="8" t="n">
+        <v>1510.45</v>
+      </c>
+      <c r="O1160" s="7" t="n">
+        <v>1534.05</v>
+      </c>
+      <c r="P1160" s="9" t="n">
+        <v>1486.95</v>
+      </c>
+      <c r="Q1160" s="9" t="n">
+        <v>1463.45</v>
+      </c>
+      <c r="R1160" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="S1160" s="6" t="n">
+        <v>2974</v>
+      </c>
+      <c r="T1160" s="6" t="n">
+        <v>2961</v>
+      </c>
+      <c r="U1160" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1160" s="6" t="inlineStr"/>
+      <c r="W1160" s="6" t="inlineStr"/>
+      <c r="X1160" s="6" t="inlineStr"/>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1161" s="6" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="C1161" s="6" t="inlineStr">
+        <is>
+          <t>CEMENT</t>
+        </is>
+      </c>
+      <c r="D1161" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1161" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1161" s="6" t="n">
+        <v>10829</v>
+      </c>
+      <c r="G1161" s="6" t="n">
+        <v>11010</v>
+      </c>
+      <c r="H1161" s="6" t="n">
+        <v>11027</v>
+      </c>
+      <c r="I1161" s="6" t="n">
+        <v>10826</v>
+      </c>
+      <c r="J1161" s="6" t="n">
+        <v>11045.18</v>
+      </c>
+      <c r="K1161" s="6" t="n">
+        <v>11027</v>
+      </c>
+      <c r="L1161" s="6" t="n">
+        <v>10826</v>
+      </c>
+      <c r="M1161" s="6" t="n">
+        <v>201</v>
+      </c>
+      <c r="N1161" s="8" t="n">
+        <v>10825.95</v>
+      </c>
+      <c r="O1161" s="7" t="n">
+        <v>10926.55</v>
+      </c>
+      <c r="P1161" s="9" t="n">
+        <v>10725.45</v>
+      </c>
+      <c r="Q1161" s="9" t="n">
+        <v>10624.95</v>
+      </c>
+      <c r="R1161" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="S1161" s="6" t="n">
+        <v>2716</v>
+      </c>
+      <c r="T1161" s="6" t="n">
+        <v>2714</v>
+      </c>
+      <c r="U1161" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1161" s="6" t="inlineStr"/>
+      <c r="W1161" s="6" t="inlineStr"/>
+      <c r="X1161" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 29-Sep-2026 10:32 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1161"/>
+  <dimension ref="A1:X1165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -92822,6 +92822,326 @@
       <c r="W1161" s="6" t="inlineStr"/>
       <c r="X1161" s="6" t="inlineStr"/>
     </row>
+    <row r="1162">
+      <c r="A1162" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1162" s="2" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1162" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1162" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1162" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1162" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="G1162" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="H1162" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="I1162" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="J1162" s="2" t="n">
+        <v>421.07</v>
+      </c>
+      <c r="K1162" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="L1162" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="M1162" s="2" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="N1162" s="4" t="n">
+        <v>426.05</v>
+      </c>
+      <c r="O1162" s="5" t="n">
+        <v>423.22</v>
+      </c>
+      <c r="P1162" s="3" t="n">
+        <v>428.78</v>
+      </c>
+      <c r="Q1162" s="3" t="n">
+        <v>431.5</v>
+      </c>
+      <c r="R1162" s="2" t="n">
+        <v>1059</v>
+      </c>
+      <c r="S1162" s="2" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T1162" s="2" t="n">
+        <v>2891</v>
+      </c>
+      <c r="U1162" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1162" s="2" t="inlineStr"/>
+      <c r="W1162" s="2" t="inlineStr"/>
+      <c r="X1162" s="2" t="inlineStr"/>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1163" s="2" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="C1163" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1163" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1163" s="2" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="F1163" s="2" t="n">
+        <v>9431</v>
+      </c>
+      <c r="G1163" s="2" t="n">
+        <v>9562</v>
+      </c>
+      <c r="H1163" s="2" t="n">
+        <v>9610.5</v>
+      </c>
+      <c r="I1163" s="2" t="n">
+        <v>9431</v>
+      </c>
+      <c r="J1163" s="2" t="n">
+        <v>9369.049999999999</v>
+      </c>
+      <c r="K1163" s="2" t="n">
+        <v>9610.5</v>
+      </c>
+      <c r="L1163" s="2" t="n">
+        <v>9431</v>
+      </c>
+      <c r="M1163" s="2" t="n">
+        <v>179.5</v>
+      </c>
+      <c r="N1163" s="4" t="n">
+        <v>9610.549999999999</v>
+      </c>
+      <c r="O1163" s="5" t="n">
+        <v>9520.700000000001</v>
+      </c>
+      <c r="P1163" s="3" t="n">
+        <v>9700.299999999999</v>
+      </c>
+      <c r="Q1163" s="3" t="n">
+        <v>9790.049999999999</v>
+      </c>
+      <c r="R1163" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="S1163" s="2" t="n">
+        <v>2965</v>
+      </c>
+      <c r="T1163" s="2" t="n">
+        <v>2962</v>
+      </c>
+      <c r="U1163" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1163" s="2" t="inlineStr"/>
+      <c r="W1163" s="2" t="inlineStr"/>
+      <c r="X1163" s="2" t="inlineStr"/>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1164" s="6" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="C1164" s="6" t="inlineStr">
+        <is>
+          <t>CEMENT</t>
+        </is>
+      </c>
+      <c r="D1164" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1164" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1164" s="6" t="n">
+        <v>21900</v>
+      </c>
+      <c r="G1164" s="6" t="n">
+        <v>22170</v>
+      </c>
+      <c r="H1164" s="6" t="n">
+        <v>22360</v>
+      </c>
+      <c r="I1164" s="6" t="n">
+        <v>21550</v>
+      </c>
+      <c r="J1164" s="6" t="n">
+        <v>22295.11</v>
+      </c>
+      <c r="K1164" s="6" t="n">
+        <v>22360</v>
+      </c>
+      <c r="L1164" s="6" t="n">
+        <v>21550</v>
+      </c>
+      <c r="M1164" s="6" t="n">
+        <v>810</v>
+      </c>
+      <c r="N1164" s="8" t="n">
+        <v>21549.95</v>
+      </c>
+      <c r="O1164" s="7" t="n">
+        <v>21955.05</v>
+      </c>
+      <c r="P1164" s="9" t="n">
+        <v>21144.95</v>
+      </c>
+      <c r="Q1164" s="9" t="n">
+        <v>20739.95</v>
+      </c>
+      <c r="R1164" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S1164" s="6" t="n">
+        <v>2431</v>
+      </c>
+      <c r="T1164" s="6" t="n">
+        <v>2430</v>
+      </c>
+      <c r="U1164" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1164" s="6" t="inlineStr"/>
+      <c r="W1164" s="6" t="inlineStr"/>
+      <c r="X1164" s="6" t="inlineStr"/>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1165" s="6" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="C1165" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1165" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1165" s="6" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1165" s="6" t="n">
+        <v>1015.4</v>
+      </c>
+      <c r="G1165" s="6" t="n">
+        <v>1002.6</v>
+      </c>
+      <c r="H1165" s="6" t="n">
+        <v>1015.4</v>
+      </c>
+      <c r="I1165" s="6" t="n">
+        <v>980.4</v>
+      </c>
+      <c r="J1165" s="6" t="n">
+        <v>1058.94</v>
+      </c>
+      <c r="K1165" s="6" t="n">
+        <v>1015.4</v>
+      </c>
+      <c r="L1165" s="6" t="n">
+        <v>980.4</v>
+      </c>
+      <c r="M1165" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="N1165" s="8" t="n">
+        <v>980.35</v>
+      </c>
+      <c r="O1165" s="7" t="n">
+        <v>997.95</v>
+      </c>
+      <c r="P1165" s="9" t="n">
+        <v>962.85</v>
+      </c>
+      <c r="Q1165" s="9" t="n">
+        <v>945.35</v>
+      </c>
+      <c r="R1165" s="6" t="n">
+        <v>168</v>
+      </c>
+      <c r="S1165" s="6" t="n">
+        <v>2957</v>
+      </c>
+      <c r="T1165" s="6" t="n">
+        <v>2940</v>
+      </c>
+      <c r="U1165" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1165" s="6" t="inlineStr"/>
+      <c r="W1165" s="6" t="inlineStr"/>
+      <c r="X1165" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Market data 29-Sep-2026 10:41 IST
</commit_message>
<xml_diff>
--- a/trading_journal.xlsx
+++ b/trading_journal.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1165"/>
+  <dimension ref="A1:X1169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -93142,6 +93142,326 @@
       <c r="W1165" s="6" t="inlineStr"/>
       <c r="X1165" s="6" t="inlineStr"/>
     </row>
+    <row r="1166">
+      <c r="A1166" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1166" s="2" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="C1166" s="2" t="inlineStr">
+        <is>
+          <t>PHARMA</t>
+        </is>
+      </c>
+      <c r="D1166" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1166" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1166" s="2" t="n">
+        <v>1251.9</v>
+      </c>
+      <c r="G1166" s="2" t="n">
+        <v>1243.2</v>
+      </c>
+      <c r="H1166" s="2" t="n">
+        <v>1252.8</v>
+      </c>
+      <c r="I1166" s="2" t="n">
+        <v>1229</v>
+      </c>
+      <c r="J1166" s="2" t="n">
+        <v>1192.59</v>
+      </c>
+      <c r="K1166" s="2" t="n">
+        <v>1252.8</v>
+      </c>
+      <c r="L1166" s="2" t="n">
+        <v>1229</v>
+      </c>
+      <c r="M1166" s="2" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="N1166" s="4" t="n">
+        <v>1252.85</v>
+      </c>
+      <c r="O1166" s="5" t="n">
+        <v>1240.85</v>
+      </c>
+      <c r="P1166" s="3" t="n">
+        <v>1264.75</v>
+      </c>
+      <c r="Q1166" s="3" t="n">
+        <v>1276.65</v>
+      </c>
+      <c r="R1166" s="2" t="n">
+        <v>249</v>
+      </c>
+      <c r="S1166" s="2" t="n">
+        <v>2988</v>
+      </c>
+      <c r="T1166" s="2" t="n">
+        <v>2963</v>
+      </c>
+      <c r="U1166" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1166" s="2" t="inlineStr"/>
+      <c r="W1166" s="2" t="inlineStr"/>
+      <c r="X1166" s="2" t="inlineStr"/>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="2" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1167" s="2" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="C1167" s="2" t="inlineStr">
+        <is>
+          <t>METAL</t>
+        </is>
+      </c>
+      <c r="D1167" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E1167" s="2" t="inlineStr">
+        <is>
+          <t>5/6</t>
+        </is>
+      </c>
+      <c r="F1167" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="G1167" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="H1167" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="I1167" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="J1167" s="2" t="n">
+        <v>421.07</v>
+      </c>
+      <c r="K1167" s="2" t="n">
+        <v>426</v>
+      </c>
+      <c r="L1167" s="2" t="n">
+        <v>420.55</v>
+      </c>
+      <c r="M1167" s="2" t="n">
+        <v>5.45</v>
+      </c>
+      <c r="N1167" s="4" t="n">
+        <v>426.05</v>
+      </c>
+      <c r="O1167" s="5" t="n">
+        <v>423.22</v>
+      </c>
+      <c r="P1167" s="3" t="n">
+        <v>428.78</v>
+      </c>
+      <c r="Q1167" s="3" t="n">
+        <v>431.5</v>
+      </c>
+      <c r="R1167" s="2" t="n">
+        <v>1059</v>
+      </c>
+      <c r="S1167" s="2" t="n">
+        <v>2997</v>
+      </c>
+      <c r="T1167" s="2" t="n">
+        <v>2891</v>
+      </c>
+      <c r="U1167" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1167" s="2" t="inlineStr"/>
+      <c r="W1167" s="2" t="inlineStr"/>
+      <c r="X1167" s="2" t="inlineStr"/>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1168" s="6" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="C1168" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1168" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1168" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1168" s="6" t="n">
+        <v>1222</v>
+      </c>
+      <c r="G1168" s="6" t="n">
+        <v>1252.6</v>
+      </c>
+      <c r="H1168" s="6" t="n">
+        <v>1261</v>
+      </c>
+      <c r="I1168" s="6" t="n">
+        <v>1222</v>
+      </c>
+      <c r="J1168" s="6" t="n">
+        <v>1267.67</v>
+      </c>
+      <c r="K1168" s="6" t="n">
+        <v>1261</v>
+      </c>
+      <c r="L1168" s="6" t="n">
+        <v>1222</v>
+      </c>
+      <c r="M1168" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="N1168" s="8" t="n">
+        <v>1221.95</v>
+      </c>
+      <c r="O1168" s="7" t="n">
+        <v>1241.55</v>
+      </c>
+      <c r="P1168" s="9" t="n">
+        <v>1202.45</v>
+      </c>
+      <c r="Q1168" s="9" t="n">
+        <v>1182.95</v>
+      </c>
+      <c r="R1168" s="6" t="n">
+        <v>153</v>
+      </c>
+      <c r="S1168" s="6" t="n">
+        <v>2999</v>
+      </c>
+      <c r="T1168" s="6" t="n">
+        <v>2984</v>
+      </c>
+      <c r="U1168" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1168" s="6" t="inlineStr"/>
+      <c r="W1168" s="6" t="inlineStr"/>
+      <c r="X1168" s="6" t="inlineStr"/>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="6" t="inlineStr">
+        <is>
+          <t>29-Sep-2026</t>
+        </is>
+      </c>
+      <c r="B1169" s="6" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="C1169" s="6" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D1169" s="7" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E1169" s="6" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="F1169" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="G1169" s="6" t="n">
+        <v>1542.3</v>
+      </c>
+      <c r="H1169" s="6" t="n">
+        <v>1557.5</v>
+      </c>
+      <c r="I1169" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="J1169" s="6" t="n">
+        <v>1562.41</v>
+      </c>
+      <c r="K1169" s="6" t="n">
+        <v>1557.5</v>
+      </c>
+      <c r="L1169" s="6" t="n">
+        <v>1510.5</v>
+      </c>
+      <c r="M1169" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="N1169" s="8" t="n">
+        <v>1510.45</v>
+      </c>
+      <c r="O1169" s="7" t="n">
+        <v>1534.05</v>
+      </c>
+      <c r="P1169" s="9" t="n">
+        <v>1486.95</v>
+      </c>
+      <c r="Q1169" s="9" t="n">
+        <v>1463.45</v>
+      </c>
+      <c r="R1169" s="6" t="n">
+        <v>126</v>
+      </c>
+      <c r="S1169" s="6" t="n">
+        <v>2974</v>
+      </c>
+      <c r="T1169" s="6" t="n">
+        <v>2961</v>
+      </c>
+      <c r="U1169" s="6" t="inlineStr">
+        <is>
+          <t>NEUTRAL</t>
+        </is>
+      </c>
+      <c r="V1169" s="6" t="inlineStr"/>
+      <c r="W1169" s="6" t="inlineStr"/>
+      <c r="X1169" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>